<commit_message>
Fix v5 D column update: restore 都営地下鉄 entries
都営地下鉄 (112 rows) correctly retained as-is since 板橋 sheet
does not manage public transit clients. Yellow blanks reduced to
105 rows: 東急グループ (101) + 4 individual mismatches.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -769,7 +769,11 @@
           <t>新宿線新宿三丁目駅</t>
         </is>
       </c>
-      <c r="D2" s="35" t="n"/>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E2" s="19" t="n">
         <v>40</v>
       </c>
@@ -806,7 +810,11 @@
           <t>新宿線曙橋駅</t>
         </is>
       </c>
-      <c r="D3" s="35" t="n"/>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E3" s="19" t="n">
         <v>20</v>
       </c>
@@ -843,7 +851,11 @@
           <t>新宿線市ヶ谷駅</t>
         </is>
       </c>
-      <c r="D4" s="35" t="n"/>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E4" s="19" t="n">
         <v>30</v>
       </c>
@@ -880,7 +892,11 @@
           <t>新宿線神保町駅</t>
         </is>
       </c>
-      <c r="D5" s="35" t="n"/>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E5" s="19" t="n">
         <v>20</v>
       </c>
@@ -917,7 +933,11 @@
           <t>三田線神保町駅</t>
         </is>
       </c>
-      <c r="D6" s="35" t="n"/>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E6" s="19" t="n">
         <v>40</v>
       </c>
@@ -954,7 +974,11 @@
           <t>新宿線小川町駅</t>
         </is>
       </c>
-      <c r="D7" s="35" t="n"/>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E7" s="19" t="n">
         <v>40</v>
       </c>
@@ -991,7 +1015,11 @@
           <t>新宿線九段下駅</t>
         </is>
       </c>
-      <c r="D8" s="35" t="n"/>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E8" s="19" t="n">
         <v>20</v>
       </c>
@@ -1028,7 +1056,11 @@
           <t>新宿線岩本町駅</t>
         </is>
       </c>
-      <c r="D9" s="35" t="n"/>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E9" s="19" t="n">
         <v>30</v>
       </c>
@@ -1065,7 +1097,11 @@
           <t>浅草線人形町駅</t>
         </is>
       </c>
-      <c r="D10" s="35" t="n"/>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E10" s="19" t="n">
         <v>30</v>
       </c>
@@ -1102,7 +1138,11 @@
           <t>新宿線馬喰横山駅</t>
         </is>
       </c>
-      <c r="D11" s="35" t="n"/>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E11" s="19" t="n">
         <v>50</v>
       </c>
@@ -1139,7 +1179,11 @@
           <t>浅草線東日本橋駅</t>
         </is>
       </c>
-      <c r="D12" s="35" t="n"/>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E12" s="19" t="n">
         <v>30</v>
       </c>
@@ -1176,7 +1220,11 @@
           <t>浅草線浅草橋駅</t>
         </is>
       </c>
-      <c r="D13" s="35" t="n"/>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E13" s="19" t="n">
         <v>30</v>
       </c>
@@ -1213,7 +1261,11 @@
           <t>大江戸線蔵前駅</t>
         </is>
       </c>
-      <c r="D14" s="35" t="n"/>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E14" s="19" t="n">
         <v>10</v>
       </c>
@@ -1250,7 +1302,11 @@
           <t>浅草線浅草駅</t>
         </is>
       </c>
-      <c r="D15" s="35" t="n"/>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E15" s="19" t="n">
         <v>60</v>
       </c>
@@ -1287,7 +1343,11 @@
           <t>浅草線蔵前駅</t>
         </is>
       </c>
-      <c r="D16" s="35" t="n"/>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E16" s="19" t="n">
         <v>20</v>
       </c>
@@ -1324,7 +1384,11 @@
           <t>新宿線森下駅</t>
         </is>
       </c>
-      <c r="D17" s="35" t="n"/>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E17" s="19" t="n">
         <v>20</v>
       </c>
@@ -1361,7 +1425,11 @@
           <t>大江戸線森下駅</t>
         </is>
       </c>
-      <c r="D18" s="35" t="n"/>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E18" s="19" t="n">
         <v>10</v>
       </c>
@@ -1398,7 +1466,11 @@
           <t>新宿線菊川駅</t>
         </is>
       </c>
-      <c r="D19" s="35" t="n"/>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E19" s="19" t="n">
         <v>20</v>
       </c>
@@ -1435,7 +1507,11 @@
           <t>新宿線住吉駅</t>
         </is>
       </c>
-      <c r="D20" s="35" t="n"/>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E20" s="19" t="n">
         <v>20</v>
       </c>
@@ -1472,7 +1548,11 @@
           <t>新宿線西大島駅</t>
         </is>
       </c>
-      <c r="D21" s="35" t="n"/>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E21" s="19" t="n">
         <v>20</v>
       </c>
@@ -1509,7 +1589,11 @@
           <t>新宿線大島駅</t>
         </is>
       </c>
-      <c r="D22" s="35" t="n"/>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E22" s="19" t="n">
         <v>20</v>
       </c>
@@ -1546,7 +1630,11 @@
           <t>新宿線東大島駅</t>
         </is>
       </c>
-      <c r="D23" s="35" t="n"/>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E23" s="19" t="n">
         <v>30</v>
       </c>
@@ -1583,7 +1671,11 @@
           <t>大島乗務区（都交通局）</t>
         </is>
       </c>
-      <c r="D24" s="35" t="n"/>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E24" s="19" t="n">
         <v>80</v>
       </c>
@@ -1620,7 +1712,11 @@
           <t>新宿線船堀駅</t>
         </is>
       </c>
-      <c r="D25" s="35" t="n"/>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E25" s="19" t="n">
         <v>20</v>
       </c>
@@ -1657,7 +1753,11 @@
           <t>新宿線一之江駅</t>
         </is>
       </c>
-      <c r="D26" s="35" t="n"/>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E26" s="19" t="n">
         <v>20</v>
       </c>
@@ -1694,7 +1794,11 @@
           <t>新宿線瑞江駅</t>
         </is>
       </c>
-      <c r="D27" s="35" t="n"/>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E27" s="19" t="n">
         <v>20</v>
       </c>
@@ -1731,7 +1835,11 @@
           <t>新宿線篠崎駅</t>
         </is>
       </c>
-      <c r="D28" s="35" t="n"/>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E28" s="19" t="n">
         <v>20</v>
       </c>
@@ -1768,7 +1876,11 @@
           <t>新宿線浜町駅</t>
         </is>
       </c>
-      <c r="D29" s="35" t="n"/>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E29" s="19" t="n">
         <v>20</v>
       </c>
@@ -1846,7 +1958,11 @@
           <t>大江戸線飯田橋駅</t>
         </is>
       </c>
-      <c r="D31" s="35" t="n"/>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E31" s="19" t="n">
         <v>20</v>
       </c>
@@ -1883,7 +1999,11 @@
           <t>大江戸線若松河田駅</t>
         </is>
       </c>
-      <c r="D32" s="35" t="n"/>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E32" s="19" t="n">
         <v>20</v>
       </c>
@@ -1920,7 +2040,11 @@
           <t>大江戸線東新宿駅</t>
         </is>
       </c>
-      <c r="D33" s="35" t="n"/>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E33" s="19" t="n">
         <v>20</v>
       </c>
@@ -2121,7 +2245,11 @@
           <t>大江戸線新宿西口駅</t>
         </is>
       </c>
-      <c r="D38" s="35" t="n"/>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E38" s="19" t="n">
         <v>40</v>
       </c>
@@ -2158,7 +2286,11 @@
           <t>大江戸線都庁前駅</t>
         </is>
       </c>
-      <c r="D39" s="35" t="n"/>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E39" s="19" t="n">
         <v>60</v>
       </c>
@@ -2277,7 +2409,11 @@
           <t>大江戸線中野坂上駅</t>
         </is>
       </c>
-      <c r="D42" s="35" t="n"/>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E42" s="19" t="n">
         <v>80</v>
       </c>
@@ -2355,7 +2491,11 @@
           <t>大江戸線中井駅</t>
         </is>
       </c>
-      <c r="D44" s="35" t="n"/>
+      <c r="D44" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E44" s="19" t="n">
         <v>70</v>
       </c>
@@ -2392,7 +2532,11 @@
           <t>大江戸線落合南長崎駅</t>
         </is>
       </c>
-      <c r="D45" s="35" t="n"/>
+      <c r="D45" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E45" s="19" t="n">
         <v>20</v>
       </c>
@@ -2429,7 +2573,11 @@
           <t>大江戸線練馬駅</t>
         </is>
       </c>
-      <c r="D46" s="35" t="n"/>
+      <c r="D46" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E46" s="19" t="n">
         <v>20</v>
       </c>
@@ -2466,7 +2614,11 @@
           <t>大江戸線豊島園駅</t>
         </is>
       </c>
-      <c r="D47" s="35" t="n"/>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E47" s="19" t="n">
         <v>60</v>
       </c>
@@ -2503,7 +2655,11 @@
           <t>大江戸線練馬春日町駅</t>
         </is>
       </c>
-      <c r="D48" s="35" t="n"/>
+      <c r="D48" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E48" s="19" t="n">
         <v>30</v>
       </c>
@@ -2540,7 +2696,11 @@
           <t>大江戸線光が丘駅</t>
         </is>
       </c>
-      <c r="D49" s="35" t="n"/>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E49" s="19" t="n">
         <v>40</v>
       </c>
@@ -2577,7 +2737,11 @@
           <t>光が丘乗務区（都交通局）</t>
         </is>
       </c>
-      <c r="D50" s="35" t="n"/>
+      <c r="D50" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E50" s="19" t="n">
         <v>60</v>
       </c>
@@ -2614,7 +2778,11 @@
           <t>三田線西高島平駅</t>
         </is>
       </c>
-      <c r="D51" s="35" t="n"/>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E51" s="19" t="n">
         <v>60</v>
       </c>
@@ -2651,7 +2819,11 @@
           <t>三田線新高島平駅</t>
         </is>
       </c>
-      <c r="D52" s="35" t="n"/>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E52" s="19" t="n">
         <v>40</v>
       </c>
@@ -2688,7 +2860,11 @@
           <t>三田線高島平駅</t>
         </is>
       </c>
-      <c r="D53" s="35" t="n"/>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E53" s="19" t="n">
         <v>20</v>
       </c>
@@ -2725,7 +2901,11 @@
           <t>三田線西台駅</t>
         </is>
       </c>
-      <c r="D54" s="35" t="n"/>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E54" s="19" t="n">
         <v>40</v>
       </c>
@@ -2762,7 +2942,11 @@
           <t>三田線蓮根駅</t>
         </is>
       </c>
-      <c r="D55" s="35" t="n"/>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E55" s="19" t="n">
         <v>20</v>
       </c>
@@ -2799,7 +2983,11 @@
           <t>大江戸線牛込神楽坂駅</t>
         </is>
       </c>
-      <c r="D56" s="35" t="n"/>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E56" s="19" t="n">
         <v>20</v>
       </c>
@@ -2836,7 +3024,11 @@
           <t>大江戸線牛込柳町駅</t>
         </is>
       </c>
-      <c r="D57" s="35" t="n"/>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E57" s="19" t="n">
         <v>20</v>
       </c>
@@ -2873,7 +3065,11 @@
           <t>大江戸線西新宿五丁目駅</t>
         </is>
       </c>
-      <c r="D58" s="35" t="n"/>
+      <c r="D58" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E58" s="19" t="n">
         <v>20</v>
       </c>
@@ -2910,7 +3106,11 @@
           <t>大江戸線東中野駅</t>
         </is>
       </c>
-      <c r="D59" s="35" t="n"/>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E59" s="19" t="n">
         <v>20</v>
       </c>
@@ -2947,7 +3147,11 @@
           <t>大江戸線新江古田駅</t>
         </is>
       </c>
-      <c r="D60" s="35" t="n"/>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E60" s="19" t="n">
         <v>20</v>
       </c>
@@ -2984,7 +3188,11 @@
           <t>三田線志村三丁目</t>
         </is>
       </c>
-      <c r="D61" s="35" t="n"/>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E61" s="19" t="n">
         <v>40</v>
       </c>
@@ -3103,7 +3311,11 @@
           <t>大江戸線新宿駅</t>
         </is>
       </c>
-      <c r="D64" s="35" t="n"/>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E64" s="19" t="n">
         <v>40</v>
       </c>
@@ -3140,7 +3352,11 @@
           <t>大江戸線青山一丁目駅</t>
         </is>
       </c>
-      <c r="D65" s="35" t="n"/>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E65" s="19" t="n">
         <v>20</v>
       </c>
@@ -3177,7 +3393,11 @@
           <t>大江戸線六本木駅</t>
         </is>
       </c>
-      <c r="D66" s="35" t="n"/>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E66" s="19" t="n">
         <v>20</v>
       </c>
@@ -3214,7 +3434,11 @@
           <t>大江戸線赤羽橋駅</t>
         </is>
       </c>
-      <c r="D67" s="35" t="n"/>
+      <c r="D67" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E67" s="19" t="n">
         <v>20</v>
       </c>
@@ -3251,7 +3475,11 @@
           <t>浅草線泉岳寺駅</t>
         </is>
       </c>
-      <c r="D68" s="35" t="n"/>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E68" s="19" t="n">
         <v>20</v>
       </c>
@@ -3288,7 +3516,11 @@
           <t>浅草線三田駅</t>
         </is>
       </c>
-      <c r="D69" s="35" t="n"/>
+      <c r="D69" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E69" s="19" t="n">
         <v>20</v>
       </c>
@@ -3325,7 +3557,11 @@
           <t>三田線三田駅</t>
         </is>
       </c>
-      <c r="D70" s="35" t="n"/>
+      <c r="D70" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E70" s="19" t="n">
         <v>40</v>
       </c>
@@ -3362,7 +3598,11 @@
           <t>三田線芝公園駅</t>
         </is>
       </c>
-      <c r="D71" s="35" t="n"/>
+      <c r="D71" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E71" s="19" t="n">
         <v>10</v>
       </c>
@@ -3399,7 +3639,11 @@
           <t>大江戸線大門駅</t>
         </is>
       </c>
-      <c r="D72" s="35" t="n"/>
+      <c r="D72" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E72" s="19" t="n">
         <v>70</v>
       </c>
@@ -3436,7 +3680,11 @@
           <t>大江戸線築地市場駅</t>
         </is>
       </c>
-      <c r="D73" s="35" t="n"/>
+      <c r="D73" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E73" s="19" t="n">
         <v>20</v>
       </c>
@@ -3473,7 +3721,11 @@
           <t>大江戸線勝どき駅</t>
         </is>
       </c>
-      <c r="D74" s="35" t="n"/>
+      <c r="D74" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E74" s="19" t="n">
         <v>30</v>
       </c>
@@ -3510,7 +3762,11 @@
           <t>大江戸線月島駅</t>
         </is>
       </c>
-      <c r="D75" s="35" t="n"/>
+      <c r="D75" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E75" s="19" t="n">
         <v>20</v>
       </c>
@@ -3547,7 +3803,11 @@
           <t>大江戸線門前仲町駅</t>
         </is>
       </c>
-      <c r="D76" s="35" t="n"/>
+      <c r="D76" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E76" s="19" t="n">
         <v>30</v>
       </c>
@@ -3584,7 +3844,11 @@
           <t>清澄庁舎</t>
         </is>
       </c>
-      <c r="D77" s="35" t="n"/>
+      <c r="D77" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E77" s="19" t="n">
         <v>20</v>
       </c>
@@ -3621,7 +3885,11 @@
           <t>大江戸線両国駅</t>
         </is>
       </c>
-      <c r="D78" s="35" t="n"/>
+      <c r="D78" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E78" s="19" t="n">
         <v>10</v>
       </c>
@@ -3658,7 +3926,11 @@
           <t>浅草線本所吾妻橋駅</t>
         </is>
       </c>
-      <c r="D79" s="35" t="n"/>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E79" s="19" t="n">
         <v>20</v>
       </c>
@@ -3695,7 +3967,11 @@
           <t>日暮里舎人ライナー日暮里駅</t>
         </is>
       </c>
-      <c r="D80" s="35" t="n"/>
+      <c r="D80" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E80" s="19" t="n">
         <v>30</v>
       </c>
@@ -3732,7 +4008,11 @@
           <t>日暮里舎人ライナー西日暮里駅</t>
         </is>
       </c>
-      <c r="D81" s="35" t="n"/>
+      <c r="D81" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E81" s="19" t="n">
         <v>20</v>
       </c>
@@ -3851,7 +4131,11 @@
           <t>荒川電車営業所</t>
         </is>
       </c>
-      <c r="D84" s="35" t="n"/>
+      <c r="D84" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E84" s="19" t="n">
         <v>40</v>
       </c>
@@ -3929,7 +4213,11 @@
           <t>大江戸線代々木駅</t>
         </is>
       </c>
-      <c r="D86" s="35" t="n"/>
+      <c r="D86" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E86" s="19" t="n">
         <v>30</v>
       </c>
@@ -4007,7 +4295,11 @@
           <t>大江戸線国立競技場</t>
         </is>
       </c>
-      <c r="D88" s="35" t="n"/>
+      <c r="D88" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E88" s="19" t="n">
         <v>20</v>
       </c>
@@ -4044,7 +4336,11 @@
           <t>大江戸線汐留駅</t>
         </is>
       </c>
-      <c r="D89" s="35" t="n"/>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E89" s="19" t="n">
         <v>30</v>
       </c>
@@ -4081,7 +4377,11 @@
           <t>大江戸線清澄白河駅</t>
         </is>
       </c>
-      <c r="D90" s="35" t="n"/>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E90" s="19" t="n">
         <v>20</v>
       </c>
@@ -4118,7 +4418,11 @@
           <t>日暮里舎人ライナー舎人駅</t>
         </is>
       </c>
-      <c r="D91" s="35" t="n"/>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E91" s="19" t="n">
         <v>120</v>
       </c>
@@ -4155,7 +4459,11 @@
           <t>大江戸線麻布十番駅</t>
         </is>
       </c>
-      <c r="D92" s="35" t="n"/>
+      <c r="D92" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E92" s="19" t="n">
         <v>40</v>
       </c>
@@ -4192,7 +4500,11 @@
           <t>三ノ輪橋おもいで館</t>
         </is>
       </c>
-      <c r="D93" s="35" t="n"/>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E93" s="19" t="n">
         <v>10</v>
       </c>
@@ -4229,7 +4541,11 @@
           <t>浅草線日本橋駅</t>
         </is>
       </c>
-      <c r="D94" s="35" t="n"/>
+      <c r="D94" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E94" s="19" t="n">
         <v>24</v>
       </c>
@@ -4266,7 +4582,11 @@
           <t>都営新宿線本八幡駅</t>
         </is>
       </c>
-      <c r="D95" s="35" t="n"/>
+      <c r="D95" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E95" s="19" t="n">
         <v>0</v>
       </c>
@@ -4303,7 +4623,11 @@
           <t>浅草線高輪台駅</t>
         </is>
       </c>
-      <c r="D96" s="35" t="n"/>
+      <c r="D96" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E96" s="19" t="n">
         <v>32</v>
       </c>
@@ -4340,7 +4664,11 @@
           <t>浅草線五反田駅</t>
         </is>
       </c>
-      <c r="D97" s="35" t="n"/>
+      <c r="D97" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E97" s="19" t="n">
         <v>24</v>
       </c>
@@ -4377,7 +4705,11 @@
           <t>浅草線戸越駅</t>
         </is>
       </c>
-      <c r="D98" s="35" t="n"/>
+      <c r="D98" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E98" s="19" t="n">
         <v>16</v>
       </c>
@@ -4414,7 +4746,11 @@
           <t>旧西馬込乗務区庁舎（都交通局）</t>
         </is>
       </c>
-      <c r="D99" s="35" t="n"/>
+      <c r="D99" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E99" s="19" t="n">
         <v>0</v>
       </c>
@@ -4451,7 +4787,11 @@
           <t>浅草線西馬込駅</t>
         </is>
       </c>
-      <c r="D100" s="35" t="n"/>
+      <c r="D100" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E100" s="19" t="n">
         <v>40</v>
       </c>
@@ -4488,7 +4828,11 @@
           <t>浅草線馬込駅</t>
         </is>
       </c>
-      <c r="D101" s="35" t="n"/>
+      <c r="D101" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E101" s="19" t="n">
         <v>32</v>
       </c>
@@ -4525,7 +4869,11 @@
           <t>浅草線中延駅</t>
         </is>
       </c>
-      <c r="D102" s="35" t="n"/>
+      <c r="D102" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E102" s="19" t="n">
         <v>32</v>
       </c>
@@ -4562,7 +4910,11 @@
           <t>三田線御成門駅</t>
         </is>
       </c>
-      <c r="D103" s="35" t="n"/>
+      <c r="D103" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E103" s="19" t="n">
         <v>32</v>
       </c>
@@ -4599,7 +4951,11 @@
           <t>浅草線新橋駅</t>
         </is>
       </c>
-      <c r="D104" s="35" t="n"/>
+      <c r="D104" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E104" s="19" t="n">
         <v>40</v>
       </c>
@@ -4636,7 +4992,11 @@
           <t>荒川電車営業所（都交通局）</t>
         </is>
       </c>
-      <c r="D105" s="35" t="n"/>
+      <c r="D105" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E105" s="19" t="n">
         <v>144</v>
       </c>
@@ -4673,7 +5033,11 @@
           <t>大江戸線上野御徒町駅</t>
         </is>
       </c>
-      <c r="D106" s="35" t="n"/>
+      <c r="D106" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E106" s="19" t="n">
         <v>48</v>
       </c>
@@ -4710,7 +5074,11 @@
           <t>大江戸線新御徒町駅</t>
         </is>
       </c>
-      <c r="D107" s="35" t="n"/>
+      <c r="D107" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E107" s="19" t="n">
         <v>16</v>
       </c>
@@ -4747,7 +5115,11 @@
           <t>三田線大手町駅</t>
         </is>
       </c>
-      <c r="D108" s="35" t="n"/>
+      <c r="D108" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E108" s="19" t="n">
         <v>40</v>
       </c>
@@ -4784,7 +5156,11 @@
           <t>三田線日比谷駅</t>
         </is>
       </c>
-      <c r="D109" s="35" t="n"/>
+      <c r="D109" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E109" s="19" t="n">
         <v>40</v>
       </c>
@@ -4821,7 +5197,11 @@
           <t>三田線内幸町駅</t>
         </is>
       </c>
-      <c r="D110" s="35" t="n"/>
+      <c r="D110" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E110" s="19" t="n">
         <v>24</v>
       </c>
@@ -4858,7 +5238,11 @@
           <t>浅草線東銀座駅</t>
         </is>
       </c>
-      <c r="D111" s="35" t="n"/>
+      <c r="D111" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E111" s="19" t="n">
         <v>48</v>
       </c>
@@ -4895,7 +5279,11 @@
           <t>浅草線宝町駅</t>
         </is>
       </c>
-      <c r="D112" s="35" t="n"/>
+      <c r="D112" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E112" s="19" t="n">
         <v>8</v>
       </c>
@@ -4932,7 +5320,11 @@
           <t>三田線春日駅</t>
         </is>
       </c>
-      <c r="D113" s="35" t="n"/>
+      <c r="D113" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E113" s="19" t="n">
         <v>32</v>
       </c>
@@ -4969,7 +5361,11 @@
           <t>大江戸線春日駅</t>
         </is>
       </c>
-      <c r="D114" s="35" t="n"/>
+      <c r="D114" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E114" s="19" t="n">
         <v>0</v>
       </c>
@@ -5006,7 +5402,11 @@
           <t>三田線水道橋駅</t>
         </is>
       </c>
-      <c r="D115" s="35" t="n"/>
+      <c r="D115" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E115" s="19" t="n">
         <v>32</v>
       </c>
@@ -5043,7 +5443,11 @@
           <t>大江戸線本郷三丁目駅</t>
         </is>
       </c>
-      <c r="D116" s="35" t="n"/>
+      <c r="D116" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E116" s="19" t="n">
         <v>8</v>
       </c>
@@ -5080,7 +5484,11 @@
           <t>三田線白山駅</t>
         </is>
       </c>
-      <c r="D117" s="35" t="n"/>
+      <c r="D117" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E117" s="19" t="n">
         <v>16</v>
       </c>
@@ -5117,7 +5525,11 @@
           <t>三田線千石駅</t>
         </is>
       </c>
-      <c r="D118" s="35" t="n"/>
+      <c r="D118" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E118" s="19" t="n">
         <v>16</v>
       </c>
@@ -5154,7 +5566,11 @@
           <t>三田線巣鴨駅</t>
         </is>
       </c>
-      <c r="D119" s="35" t="n"/>
+      <c r="D119" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E119" s="19" t="n">
         <v>32</v>
       </c>
@@ -5191,7 +5607,11 @@
           <t>三田線西巣鴨駅</t>
         </is>
       </c>
-      <c r="D120" s="35" t="n"/>
+      <c r="D120" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E120" s="19" t="n">
         <v>16</v>
       </c>
@@ -5228,7 +5648,11 @@
           <t>三田線新板橋駅</t>
         </is>
       </c>
-      <c r="D121" s="35" t="n"/>
+      <c r="D121" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E121" s="19" t="n">
         <v>16</v>
       </c>
@@ -5265,7 +5689,11 @@
           <t>三田線板橋区役所前駅</t>
         </is>
       </c>
-      <c r="D122" s="35" t="n"/>
+      <c r="D122" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E122" s="19" t="n">
         <v>16</v>
       </c>
@@ -5302,7 +5730,11 @@
           <t>三田線板橋本町駅</t>
         </is>
       </c>
-      <c r="D123" s="35" t="n"/>
+      <c r="D123" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E123" s="19" t="n">
         <v>8</v>
       </c>
@@ -5339,7 +5771,11 @@
           <t>三田線本蓮沼駅</t>
         </is>
       </c>
-      <c r="D124" s="35" t="n"/>
+      <c r="D124" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E124" s="19" t="n">
         <v>16</v>
       </c>
@@ -5376,7 +5812,11 @@
           <t>三田線志村坂下駅</t>
         </is>
       </c>
-      <c r="D125" s="35" t="n"/>
+      <c r="D125" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E125" s="19" t="n">
         <v>8</v>
       </c>
@@ -5413,7 +5853,11 @@
           <t>三田線志村三丁目駅</t>
         </is>
       </c>
-      <c r="D126" s="35" t="n"/>
+      <c r="D126" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E126" s="19" t="n">
         <v>16</v>
       </c>
@@ -5450,7 +5894,11 @@
           <t>日暮里・舎人ライナー舎人駅</t>
         </is>
       </c>
-      <c r="D127" s="35" t="n"/>
+      <c r="D127" s="19" t="inlineStr">
+        <is>
+          <t>都営地下鉄</t>
+        </is>
+      </c>
       <c r="E127" s="19" t="n">
         <v>56</v>
       </c>

</xml_diff>

<commit_message>
Update v5 master: highlight 140 empty D column cells in yellow
Original D column values (360 filled) are untouched.
140 empty cells colored yellow to indicate pending 請求先名 input.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -278,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -328,12 +328,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -6222,7 +6221,11 @@
           <t>パシオス　西小山店</t>
         </is>
       </c>
-      <c r="D135" s="35" t="n"/>
+      <c r="D135" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E135" s="19" t="n">
         <v>20</v>
       </c>
@@ -7120,7 +7123,11 @@
           <t>東急電鉄　中目黒駅</t>
         </is>
       </c>
-      <c r="D157" s="35" t="n"/>
+      <c r="D157" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E157" s="19" t="n">
         <v>70</v>
       </c>
@@ -7157,7 +7164,11 @@
           <t>TOKS　中目黒駅</t>
         </is>
       </c>
-      <c r="D158" s="35" t="n"/>
+      <c r="D158" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E158" s="19" t="n">
         <v>10</v>
       </c>
@@ -7194,7 +7205,11 @@
           <t>中目黒高架下　共有部ーD</t>
         </is>
       </c>
-      <c r="D159" s="35" t="n"/>
+      <c r="D159" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E159" s="19" t="n">
         <v>0</v>
       </c>
@@ -7231,7 +7246,11 @@
           <t>ザ・シティベーカリー</t>
         </is>
       </c>
-      <c r="D160" s="36" t="n"/>
+      <c r="D160" s="21" t="inlineStr">
+        <is>
+          <t>（株）フォンス</t>
+        </is>
+      </c>
       <c r="E160" s="19" t="n">
         <v>50</v>
       </c>
@@ -7473,7 +7492,11 @@
           <t>中目黒高架下　共用部ーF</t>
         </is>
       </c>
-      <c r="D166" s="35" t="n"/>
+      <c r="D166" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E166" s="19" t="n">
         <v>0</v>
       </c>
@@ -7838,7 +7861,11 @@
           <t>中目黒高架下　共用部ーG</t>
         </is>
       </c>
-      <c r="D175" s="37" t="n"/>
+      <c r="D175" s="24" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E175" s="19" t="n">
         <v>0</v>
       </c>
@@ -7957,7 +7984,7 @@
           <t>あらちゃん</t>
         </is>
       </c>
-      <c r="D178" s="25" t="n"/>
+      <c r="D178" s="35" t="n"/>
       <c r="E178" s="19" t="n">
         <v>10</v>
       </c>
@@ -8076,7 +8103,11 @@
           <t>中目黒高架下　共用部ーH</t>
         </is>
       </c>
-      <c r="D181" s="37" t="n"/>
+      <c r="D181" s="24" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E181" s="19" t="n">
         <v>0</v>
       </c>
@@ -8236,7 +8267,7 @@
           <t>ASReal</t>
         </is>
       </c>
-      <c r="D185" s="19" t="n"/>
+      <c r="D185" s="36" t="n"/>
       <c r="E185" s="19" t="n">
         <v>0</v>
       </c>
@@ -8273,7 +8304,7 @@
           <t>ALWAYS OUT OF STOCK</t>
         </is>
       </c>
-      <c r="D186" s="19" t="n"/>
+      <c r="D186" s="36" t="n"/>
       <c r="E186" s="19" t="n">
         <v>0</v>
       </c>
@@ -8433,7 +8464,7 @@
           <t>GYM by LAVISUS</t>
         </is>
       </c>
-      <c r="D190" s="19" t="n"/>
+      <c r="D190" s="36" t="n"/>
       <c r="E190" s="19" t="n">
         <v>0</v>
       </c>
@@ -8511,7 +8542,7 @@
           <t>曼茶羅</t>
         </is>
       </c>
-      <c r="D192" s="19" t="n"/>
+      <c r="D192" s="36" t="n"/>
       <c r="E192" s="19" t="n">
         <v>0</v>
       </c>
@@ -8671,7 +8702,11 @@
           <t>目黒高架下　共用部ーI</t>
         </is>
       </c>
-      <c r="D196" s="37" t="n"/>
+      <c r="D196" s="24" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E196" s="19" t="n">
         <v>0</v>
       </c>
@@ -8708,7 +8743,7 @@
           <t>CHANCEジム中目黒店</t>
         </is>
       </c>
-      <c r="D197" s="19" t="n"/>
+      <c r="D197" s="36" t="n"/>
       <c r="E197" s="19" t="n">
         <v>3</v>
       </c>
@@ -8786,7 +8821,11 @@
           <t>中目黒高架下　共用部ーA</t>
         </is>
       </c>
-      <c r="D199" s="37" t="n"/>
+      <c r="D199" s="24" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E199" s="19" t="n">
         <v>0</v>
       </c>
@@ -9069,7 +9108,7 @@
           <t>GOOD LUCK 中目黒店</t>
         </is>
       </c>
-      <c r="D206" s="19" t="n"/>
+      <c r="D206" s="36" t="n"/>
       <c r="E206" s="19" t="n">
         <v>5</v>
       </c>
@@ -9188,7 +9227,11 @@
           <t>中目黒高架下　共用部ーB</t>
         </is>
       </c>
-      <c r="D209" s="35" t="n"/>
+      <c r="D209" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E209" s="19" t="n">
         <v>3</v>
       </c>
@@ -9225,7 +9268,11 @@
           <t>東急電鉄　祐天寺駅</t>
         </is>
       </c>
-      <c r="D210" s="35" t="n"/>
+      <c r="D210" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E210" s="19" t="n">
         <v>20</v>
       </c>
@@ -9262,7 +9309,11 @@
           <t>simplace Gakugei-daigaku by New</t>
         </is>
       </c>
-      <c r="D211" s="36" t="n"/>
+      <c r="D211" s="21" t="inlineStr">
+        <is>
+          <t>就労移行支援事業所</t>
+        </is>
+      </c>
       <c r="E211" s="19" t="n">
         <v>0</v>
       </c>
@@ -9668,7 +9719,11 @@
           <t>はせ川</t>
         </is>
       </c>
-      <c r="D221" s="36" t="n"/>
+      <c r="D221" s="21" t="inlineStr">
+        <is>
+          <t>はせ川（株）チャコ－ルグリルアンコ</t>
+        </is>
+      </c>
       <c r="E221" s="19" t="n">
         <v>5</v>
       </c>
@@ -9869,7 +9924,7 @@
           <t>Mix Bar Rose</t>
         </is>
       </c>
-      <c r="D226" s="19" t="n"/>
+      <c r="D226" s="36" t="n"/>
       <c r="E226" s="19" t="n">
         <v>0</v>
       </c>
@@ -9906,7 +9961,7 @@
           <t>sazan reef</t>
         </is>
       </c>
-      <c r="D227" s="19" t="n"/>
+      <c r="D227" s="36" t="n"/>
       <c r="E227" s="19" t="n">
         <v>1</v>
       </c>
@@ -9943,7 +9998,7 @@
           <t>CHI-FO</t>
         </is>
       </c>
-      <c r="D228" s="19" t="n"/>
+      <c r="D228" s="36" t="n"/>
       <c r="E228" s="19" t="n">
         <v>5</v>
       </c>
@@ -10103,7 +10158,7 @@
           <t>１０BL共用部分</t>
         </is>
       </c>
-      <c r="D232" s="19" t="n"/>
+      <c r="D232" s="36" t="n"/>
       <c r="E232" s="19" t="n">
         <v>0</v>
       </c>
@@ -10181,7 +10236,11 @@
           <t>パンの田島</t>
         </is>
       </c>
-      <c r="D234" s="38" t="n"/>
+      <c r="D234" s="26" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E234" s="19" t="n">
         <v>30</v>
       </c>
@@ -10218,7 +10277,11 @@
           <t>ドトール珈琲農園</t>
         </is>
       </c>
-      <c r="D235" s="35" t="n"/>
+      <c r="D235" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E235" s="19" t="n">
         <v>150</v>
       </c>
@@ -10255,7 +10318,7 @@
           <t>鮮魚　北浜　学芸大学店</t>
         </is>
       </c>
-      <c r="D236" s="19" t="n"/>
+      <c r="D236" s="36" t="n"/>
       <c r="E236" s="19" t="n">
         <v>5</v>
       </c>
@@ -10415,7 +10478,7 @@
           <t>学大マーチ＆シーズンカフェ</t>
         </is>
       </c>
-      <c r="D240" s="19" t="n"/>
+      <c r="D240" s="36" t="n"/>
       <c r="E240" s="19" t="n">
         <v>0</v>
       </c>
@@ -10493,7 +10556,7 @@
           <t>そばもん　学大店</t>
         </is>
       </c>
-      <c r="D242" s="19" t="n"/>
+      <c r="D242" s="36" t="n"/>
       <c r="E242" s="19" t="n">
         <v>5</v>
       </c>
@@ -10530,7 +10593,11 @@
           <t>東急電鉄　総合管理事務所　１３BL</t>
         </is>
       </c>
-      <c r="D243" s="35" t="n"/>
+      <c r="D243" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E243" s="19" t="n">
         <v>2</v>
       </c>
@@ -10649,7 +10716,11 @@
           <t>東急電鉄　学芸大学駅</t>
         </is>
       </c>
-      <c r="D246" s="35" t="n"/>
+      <c r="D246" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E246" s="19" t="n">
         <v>15</v>
       </c>
@@ -10727,7 +10798,7 @@
           <t>MAISON KUROSU学芸</t>
         </is>
       </c>
-      <c r="D248" s="19" t="n"/>
+      <c r="D248" s="36" t="n"/>
       <c r="E248" s="19" t="n">
         <v>30</v>
       </c>
@@ -11051,7 +11122,11 @@
           <t>お酒の美術館</t>
         </is>
       </c>
-      <c r="D256" s="36" t="n"/>
+      <c r="D256" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">お酒の美術館（ナカゾノ　　　　</t>
+        </is>
+      </c>
       <c r="E256" s="19" t="n">
         <v>0</v>
       </c>
@@ -11416,7 +11491,11 @@
           <t>東急グルメフロント</t>
         </is>
       </c>
-      <c r="D265" s="35" t="n"/>
+      <c r="D265" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E265" s="19" t="n">
         <v>20</v>
       </c>
@@ -11453,7 +11532,7 @@
           <t>DEAN&amp;DELUCA</t>
         </is>
       </c>
-      <c r="D266" s="19" t="n"/>
+      <c r="D266" s="36" t="n"/>
       <c r="E266" s="19" t="n">
         <v>80</v>
       </c>
@@ -11654,7 +11733,7 @@
           <t>あの小宮</t>
         </is>
       </c>
-      <c r="D271" s="19" t="n"/>
+      <c r="D271" s="36" t="n"/>
       <c r="E271" s="19" t="n">
         <v>100</v>
       </c>
@@ -11773,7 +11852,7 @@
           <t>あーる工房</t>
         </is>
       </c>
-      <c r="D274" s="19" t="n"/>
+      <c r="D274" s="36" t="n"/>
       <c r="E274" s="19" t="n">
         <v>1</v>
       </c>
@@ -11851,7 +11930,7 @@
           <t>NewWork　都立大</t>
         </is>
       </c>
-      <c r="D276" s="19" t="n"/>
+      <c r="D276" s="36" t="n"/>
       <c r="E276" s="19" t="n">
         <v>0</v>
       </c>
@@ -11929,7 +12008,11 @@
           <t>東急電鉄　都立大学駅</t>
         </is>
       </c>
-      <c r="D278" s="35" t="n"/>
+      <c r="D278" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E278" s="19" t="n">
         <v>5</v>
       </c>
@@ -11966,7 +12049,11 @@
           <t>TOKS　学芸大学駅</t>
         </is>
       </c>
-      <c r="D279" s="35" t="n"/>
+      <c r="D279" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E279" s="19" t="n">
         <v>0</v>
       </c>
@@ -12003,7 +12090,11 @@
           <t>東急電鉄　駒澤大学駅</t>
         </is>
       </c>
-      <c r="D280" s="35" t="n"/>
+      <c r="D280" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E280" s="19" t="n">
         <v>1</v>
       </c>
@@ -12040,7 +12131,7 @@
           <t>サーティーワンアイスクリーム</t>
         </is>
       </c>
-      <c r="D281" s="19" t="n"/>
+      <c r="D281" s="36" t="n"/>
       <c r="E281" s="19" t="n">
         <v>1</v>
       </c>
@@ -12077,7 +12168,7 @@
           <t>ルナアース</t>
         </is>
       </c>
-      <c r="D282" s="19" t="n"/>
+      <c r="D282" s="36" t="n"/>
       <c r="E282" s="19" t="n">
         <v>0</v>
       </c>
@@ -12155,7 +12246,7 @@
           <t>オープンマート駒澤大学駅中店</t>
         </is>
       </c>
-      <c r="D284" s="19" t="n"/>
+      <c r="D284" s="36" t="n"/>
       <c r="E284" s="19" t="n">
         <v>0</v>
       </c>
@@ -12192,7 +12283,7 @@
           <t>オハナ　明大前</t>
         </is>
       </c>
-      <c r="D285" s="19" t="n"/>
+      <c r="D285" s="36" t="n"/>
       <c r="E285" s="19" t="n">
         <v>40</v>
       </c>
@@ -12229,7 +12320,11 @@
           <t>東急電鉄　下高井戸駅</t>
         </is>
       </c>
-      <c r="D286" s="35" t="n"/>
+      <c r="D286" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E286" s="19" t="n">
         <v>5</v>
       </c>
@@ -12430,7 +12525,7 @@
           <t>roobby-fit 下高井戸店</t>
         </is>
       </c>
-      <c r="D291" s="19" t="n"/>
+      <c r="D291" s="36" t="n"/>
       <c r="E291" s="19" t="n">
         <v>0</v>
       </c>
@@ -12467,7 +12562,11 @@
           <t>東急プロパティマネジメント渋谷班</t>
         </is>
       </c>
-      <c r="D292" s="35" t="n"/>
+      <c r="D292" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E292" s="19" t="n">
         <v>0</v>
       </c>
@@ -12504,7 +12603,11 @@
           <t>東急電鉄渋谷駅（田園都市線）</t>
         </is>
       </c>
-      <c r="D293" s="35" t="n"/>
+      <c r="D293" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E293" s="19" t="n">
         <v>40</v>
       </c>
@@ -12541,7 +12644,11 @@
           <t>TOKS　田園都市渋谷駅</t>
         </is>
       </c>
-      <c r="D294" s="35" t="n"/>
+      <c r="D294" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E294" s="19" t="n">
         <v>0</v>
       </c>
@@ -12578,7 +12685,7 @@
           <t>MY SWEETS　渋谷店</t>
         </is>
       </c>
-      <c r="D295" s="19" t="n"/>
+      <c r="D295" s="36" t="n"/>
       <c r="E295" s="19" t="n">
         <v>0</v>
       </c>
@@ -12615,7 +12722,7 @@
           <t>ランキンランキン渋谷店</t>
         </is>
       </c>
-      <c r="D296" s="19" t="n"/>
+      <c r="D296" s="36" t="n"/>
       <c r="E296" s="19" t="n">
         <v>5</v>
       </c>
@@ -12652,7 +12759,7 @@
           <t>白洋舎　東京支店</t>
         </is>
       </c>
-      <c r="D297" s="19" t="n"/>
+      <c r="D297" s="36" t="n"/>
       <c r="E297" s="19" t="n">
         <v>150</v>
       </c>
@@ -12689,7 +12796,7 @@
           <t>河合塾　本郷校</t>
         </is>
       </c>
-      <c r="D298" s="19" t="n"/>
+      <c r="D298" s="36" t="n"/>
       <c r="E298" s="19" t="n">
         <v>100</v>
       </c>
@@ -12726,7 +12833,11 @@
           <t>東急電鉄上町駅</t>
         </is>
       </c>
-      <c r="D299" s="35" t="n"/>
+      <c r="D299" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E299" s="19" t="n">
         <v>40</v>
       </c>
@@ -12763,7 +12874,11 @@
           <t>東急電鉄三軒茶屋駅（田園都市線）</t>
         </is>
       </c>
-      <c r="D300" s="35" t="n"/>
+      <c r="D300" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E300" s="19" t="n">
         <v>35</v>
       </c>
@@ -12800,7 +12915,11 @@
           <t>ローソン＋toks 三軒茶屋店</t>
         </is>
       </c>
-      <c r="D301" s="35" t="n"/>
+      <c r="D301" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E301" s="19" t="n">
         <v>15</v>
       </c>
@@ -12837,7 +12956,7 @@
           <t>南大塚エースビル</t>
         </is>
       </c>
-      <c r="D302" s="19" t="n"/>
+      <c r="D302" s="36" t="n"/>
       <c r="E302" s="19" t="n">
         <v>45</v>
       </c>
@@ -12874,7 +12993,7 @@
           <t>(株)ハピラル・テストソリューションズ</t>
         </is>
       </c>
-      <c r="D303" s="19" t="n"/>
+      <c r="D303" s="36" t="n"/>
       <c r="E303" s="19" t="n">
         <v>15</v>
       </c>
@@ -12911,7 +13030,11 @@
           <t>東急電鉄山下駅</t>
         </is>
       </c>
-      <c r="D304" s="35" t="n"/>
+      <c r="D304" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E304" s="19" t="n">
         <v>0</v>
       </c>
@@ -12948,7 +13071,11 @@
           <t>東急電鉄桜新町駅</t>
         </is>
       </c>
-      <c r="D305" s="35" t="n"/>
+      <c r="D305" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E305" s="19" t="n">
         <v>10</v>
       </c>
@@ -12985,7 +13112,11 @@
           <t>東急電鉄用賀駅</t>
         </is>
       </c>
-      <c r="D306" s="35" t="n"/>
+      <c r="D306" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E306" s="19" t="n">
         <v>30</v>
       </c>
@@ -13022,7 +13153,11 @@
           <t>TOKS　用賀駅</t>
         </is>
       </c>
-      <c r="D307" s="35" t="n"/>
+      <c r="D307" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E307" s="19" t="n">
         <v>10</v>
       </c>
@@ -13059,7 +13194,7 @@
           <t>ミスターミニット　用賀店</t>
         </is>
       </c>
-      <c r="D308" s="19" t="n"/>
+      <c r="D308" s="36" t="n"/>
       <c r="E308" s="19" t="n">
         <v>5</v>
       </c>
@@ -13096,7 +13231,11 @@
           <t>東急電鉄　二子玉川信通事務所</t>
         </is>
       </c>
-      <c r="D309" s="35" t="n"/>
+      <c r="D309" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E309" s="19" t="n">
         <v>0</v>
       </c>
@@ -13133,7 +13272,11 @@
           <t>東急電鉄　二子玉川駅</t>
         </is>
       </c>
-      <c r="D310" s="35" t="n"/>
+      <c r="D310" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E310" s="19" t="n">
         <v>20</v>
       </c>
@@ -13170,7 +13313,11 @@
           <t>TOKS　二子玉川駅</t>
         </is>
       </c>
-      <c r="D311" s="35" t="n"/>
+      <c r="D311" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E311" s="19" t="n">
         <v>0</v>
       </c>
@@ -13207,7 +13354,11 @@
           <t>しぶそば　二子玉川駅店</t>
         </is>
       </c>
-      <c r="D312" s="35" t="n"/>
+      <c r="D312" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E312" s="19" t="n">
         <v>30</v>
       </c>
@@ -13244,7 +13395,11 @@
           <t>MY SWEETS　二子玉川店</t>
         </is>
       </c>
-      <c r="D313" s="35" t="n"/>
+      <c r="D313" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E313" s="19" t="n">
         <v>50</v>
       </c>
@@ -13281,7 +13436,7 @@
           <t>スタジオマリオグラン　二子玉川店</t>
         </is>
       </c>
-      <c r="D314" s="19" t="n"/>
+      <c r="D314" s="36" t="n"/>
       <c r="E314" s="19" t="n">
         <v>5</v>
       </c>
@@ -13318,7 +13473,11 @@
           <t>東急ストア　二子玉川駅構内店</t>
         </is>
       </c>
-      <c r="D315" s="35" t="n"/>
+      <c r="D315" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E315" s="19" t="n">
         <v>10</v>
       </c>
@@ -13355,7 +13514,11 @@
           <t>東急プロパティマネジメントサポートセンター</t>
         </is>
       </c>
-      <c r="D316" s="35" t="n"/>
+      <c r="D316" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E316" s="19" t="n">
         <v>5</v>
       </c>
@@ -13392,7 +13555,11 @@
           <t>東急電鉄上野毛駅</t>
         </is>
       </c>
-      <c r="D317" s="35" t="n"/>
+      <c r="D317" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E317" s="19" t="n">
         <v>0</v>
       </c>
@@ -13429,7 +13596,7 @@
           <t>こもれび保育園　上野毛園</t>
         </is>
       </c>
-      <c r="D318" s="19" t="n"/>
+      <c r="D318" s="36" t="n"/>
       <c r="E318" s="19" t="n">
         <v>20</v>
       </c>
@@ -13466,7 +13633,7 @@
           <t>あおい皮膚科　駅ナカ上野毛</t>
         </is>
       </c>
-      <c r="D319" s="19" t="n"/>
+      <c r="D319" s="36" t="n"/>
       <c r="E319" s="19" t="n">
         <v>0</v>
       </c>
@@ -13503,7 +13670,7 @@
           <t>大井町線上野毛駅構内店舗</t>
         </is>
       </c>
-      <c r="D320" s="19" t="n"/>
+      <c r="D320" s="36" t="n"/>
       <c r="E320" s="19" t="n">
         <v>0</v>
       </c>
@@ -13540,7 +13707,11 @@
           <t>東急電鉄等々力駅</t>
         </is>
       </c>
-      <c r="D321" s="35" t="n"/>
+      <c r="D321" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E321" s="19" t="n">
         <v>10</v>
       </c>
@@ -13577,7 +13748,11 @@
           <t>東急電鉄尾山台駅</t>
         </is>
       </c>
-      <c r="D322" s="35" t="n"/>
+      <c r="D322" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E322" s="19" t="n">
         <v>10</v>
       </c>
@@ -13614,7 +13789,11 @@
           <t>東急電鉄九品仏駅</t>
         </is>
       </c>
-      <c r="D323" s="35" t="n"/>
+      <c r="D323" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E323" s="19" t="n">
         <v>0</v>
       </c>
@@ -13651,7 +13830,11 @@
           <t>東急電鉄田園調布駅</t>
         </is>
       </c>
-      <c r="D324" s="35" t="n"/>
+      <c r="D324" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E324" s="19" t="n">
         <v>200</v>
       </c>
@@ -13688,7 +13871,7 @@
           <t>フラマンドール　田園調布店</t>
         </is>
       </c>
-      <c r="D325" s="19" t="n"/>
+      <c r="D325" s="36" t="n"/>
       <c r="E325" s="19" t="n">
         <v>50</v>
       </c>
@@ -13725,7 +13908,11 @@
           <t>ローソン＋TOKS　田園調布駅</t>
         </is>
       </c>
-      <c r="D326" s="35" t="n"/>
+      <c r="D326" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E326" s="19" t="n">
         <v>0</v>
       </c>
@@ -13762,7 +13949,11 @@
           <t>東急電鉄多摩川駅</t>
         </is>
       </c>
-      <c r="D327" s="35" t="n"/>
+      <c r="D327" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E327" s="19" t="n">
         <v>10</v>
       </c>
@@ -13799,7 +13990,11 @@
           <t>ローソン＋TOKS　多摩川駅店</t>
         </is>
       </c>
-      <c r="D328" s="35" t="n"/>
+      <c r="D328" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E328" s="19" t="n">
         <v>0</v>
       </c>
@@ -13836,7 +14031,7 @@
           <t>日吉エリア</t>
         </is>
       </c>
-      <c r="D329" s="19" t="n"/>
+      <c r="D329" s="36" t="n"/>
       <c r="E329" s="19" t="n">
         <v>5</v>
       </c>
@@ -13873,7 +14068,7 @@
           <t>リトルマーメイド　多摩川店</t>
         </is>
       </c>
-      <c r="D330" s="19" t="n"/>
+      <c r="D330" s="36" t="n"/>
       <c r="E330" s="19" t="n">
         <v>20</v>
       </c>
@@ -13910,7 +14105,7 @@
           <t>しぶそば　多摩川店</t>
         </is>
       </c>
-      <c r="D331" s="19" t="n"/>
+      <c r="D331" s="36" t="n"/>
       <c r="E331" s="19" t="n">
         <v>20</v>
       </c>
@@ -13947,7 +14142,7 @@
           <t>銀座マギー　商品センター</t>
         </is>
       </c>
-      <c r="D332" s="19" t="n"/>
+      <c r="D332" s="36" t="n"/>
       <c r="E332" s="19" t="n">
         <v>70</v>
       </c>
@@ -13984,7 +14179,7 @@
           <t>学校法人　聖ドミニコ学園</t>
         </is>
       </c>
-      <c r="D333" s="19" t="n"/>
+      <c r="D333" s="36" t="n"/>
       <c r="E333" s="19" t="n">
         <v>120</v>
       </c>
@@ -14021,7 +14216,7 @@
           <t>東京リーガルマインド　水道橋本校</t>
         </is>
       </c>
-      <c r="D334" s="19" t="n"/>
+      <c r="D334" s="36" t="n"/>
       <c r="E334" s="19" t="n">
         <v>30</v>
       </c>
@@ -14058,7 +14253,11 @@
           <t>東急電鉄　代官山駅</t>
         </is>
       </c>
-      <c r="D335" s="35" t="n"/>
+      <c r="D335" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E335" s="19" t="n">
         <v>15</v>
       </c>
@@ -14095,7 +14294,11 @@
           <t>TOKS　代官山駅</t>
         </is>
       </c>
-      <c r="D336" s="35" t="n"/>
+      <c r="D336" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E336" s="19" t="n">
         <v>5</v>
       </c>
@@ -14132,7 +14335,11 @@
           <t>東急電鉄池尻大橋駅</t>
         </is>
       </c>
-      <c r="D337" s="35" t="n"/>
+      <c r="D337" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E337" s="19" t="n">
         <v>20</v>
       </c>
@@ -14169,7 +14376,7 @@
           <t>天才キッズクラブ楽学館仲池上園</t>
         </is>
       </c>
-      <c r="D338" s="19" t="n"/>
+      <c r="D338" s="36" t="n"/>
       <c r="E338" s="19" t="n">
         <v>0</v>
       </c>
@@ -14206,7 +14413,7 @@
           <t>Far Yeast Brewing</t>
         </is>
       </c>
-      <c r="D339" s="19" t="n"/>
+      <c r="D339" s="36" t="n"/>
       <c r="E339" s="19" t="n">
         <v>10</v>
       </c>
@@ -14243,7 +14450,7 @@
           <t>貝々　味海</t>
         </is>
       </c>
-      <c r="D340" s="19" t="n"/>
+      <c r="D340" s="36" t="n"/>
       <c r="E340" s="19" t="n">
         <v>3</v>
       </c>
@@ -14280,7 +14487,7 @@
           <t>東京食堂</t>
         </is>
       </c>
-      <c r="D341" s="19" t="n"/>
+      <c r="D341" s="36" t="n"/>
       <c r="E341" s="19" t="n">
         <v>0</v>
       </c>
@@ -14317,7 +14524,7 @@
           <t>ファットバー</t>
         </is>
       </c>
-      <c r="D342" s="19" t="n"/>
+      <c r="D342" s="36" t="n"/>
       <c r="E342" s="19" t="n">
         <v>0</v>
       </c>
@@ -14354,7 +14561,7 @@
           <t>さみしがりや酒房　ささ</t>
         </is>
       </c>
-      <c r="D343" s="19" t="n"/>
+      <c r="D343" s="36" t="n"/>
       <c r="E343" s="19" t="n">
         <v>0</v>
       </c>
@@ -14391,7 +14598,7 @@
           <t>居酒屋めぐろ川前</t>
         </is>
       </c>
-      <c r="D344" s="19" t="n"/>
+      <c r="D344" s="36" t="n"/>
       <c r="E344" s="19" t="n">
         <v>2</v>
       </c>
@@ -14428,7 +14635,7 @@
           <t>キッチン　クレセント</t>
         </is>
       </c>
-      <c r="D345" s="19" t="n"/>
+      <c r="D345" s="36" t="n"/>
       <c r="E345" s="19" t="n">
         <v>0</v>
       </c>
@@ -14465,7 +14672,7 @@
           <t>イケマル酒場</t>
         </is>
       </c>
-      <c r="D346" s="19" t="n"/>
+      <c r="D346" s="36" t="n"/>
       <c r="E346" s="19" t="n">
         <v>0</v>
       </c>
@@ -14502,7 +14709,7 @@
           <t>桜小路　共用部</t>
         </is>
       </c>
-      <c r="D347" s="19" t="n"/>
+      <c r="D347" s="36" t="n"/>
       <c r="E347" s="19" t="n">
         <v>0</v>
       </c>
@@ -14539,7 +14746,11 @@
           <t>東急電鉄大井町駅</t>
         </is>
       </c>
-      <c r="D348" s="35" t="n"/>
+      <c r="D348" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E348" s="19" t="n">
         <v>15</v>
       </c>
@@ -14576,7 +14787,11 @@
           <t>ローソン＋TOKS　大井町駅</t>
         </is>
       </c>
-      <c r="D349" s="35" t="n"/>
+      <c r="D349" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E349" s="19" t="n">
         <v>5</v>
       </c>
@@ -14613,7 +14828,7 @@
           <t>スターバックスコーヒー大井町駅</t>
         </is>
       </c>
-      <c r="D350" s="19" t="n"/>
+      <c r="D350" s="36" t="n"/>
       <c r="E350" s="19" t="n">
         <v>45</v>
       </c>
@@ -14650,7 +14865,7 @@
           <t>MY SWEETS　大井町店</t>
         </is>
       </c>
-      <c r="D351" s="19" t="n"/>
+      <c r="D351" s="36" t="n"/>
       <c r="E351" s="19" t="n">
         <v>0</v>
       </c>
@@ -14687,7 +14902,7 @@
           <t>えん　大井町店</t>
         </is>
       </c>
-      <c r="D352" s="19" t="n"/>
+      <c r="D352" s="36" t="n"/>
       <c r="E352" s="19" t="n">
         <v>35</v>
       </c>
@@ -14724,7 +14939,7 @@
           <t>E-style大井町校</t>
         </is>
       </c>
-      <c r="D353" s="19" t="n"/>
+      <c r="D353" s="36" t="n"/>
       <c r="E353" s="19" t="n">
         <v>0</v>
       </c>
@@ -14761,7 +14976,11 @@
           <t>東急大井町駅建物（共用部）</t>
         </is>
       </c>
-      <c r="D354" s="35" t="n"/>
+      <c r="D354" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E354" s="19" t="n">
         <v>0</v>
       </c>
@@ -14798,7 +15017,11 @@
           <t>しぶそば　大井町店</t>
         </is>
       </c>
-      <c r="D355" s="35" t="n"/>
+      <c r="D355" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E355" s="19" t="n">
         <v>0</v>
       </c>
@@ -14835,7 +15058,7 @@
           <t>都立大学高架下共用部</t>
         </is>
       </c>
-      <c r="D356" s="19" t="n"/>
+      <c r="D356" s="36" t="n"/>
       <c r="E356" s="19" t="n">
         <v>0</v>
       </c>
@@ -14913,7 +15136,11 @@
           <t>サピックス　自由が丘校</t>
         </is>
       </c>
-      <c r="D358" s="35" t="n"/>
+      <c r="D358" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E358" s="19" t="n">
         <v>10</v>
       </c>
@@ -14950,7 +15177,7 @@
           <t>ロッジ</t>
         </is>
       </c>
-      <c r="D359" s="19" t="n"/>
+      <c r="D359" s="36" t="n"/>
       <c r="E359" s="19" t="n">
         <v>0</v>
       </c>
@@ -14987,7 +15214,7 @@
           <t>(株)銀座マギー　田園調布ビル</t>
         </is>
       </c>
-      <c r="D360" s="19" t="n"/>
+      <c r="D360" s="36" t="n"/>
       <c r="E360" s="19" t="n">
         <v>15</v>
       </c>
@@ -15024,7 +15251,11 @@
           <t>東急電鉄　雪が谷検車区</t>
         </is>
       </c>
-      <c r="D361" s="35" t="n"/>
+      <c r="D361" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E361" s="19" t="n">
         <v>15</v>
       </c>
@@ -15061,7 +15292,7 @@
           <t>丸三ストアー</t>
         </is>
       </c>
-      <c r="D362" s="19" t="n"/>
+      <c r="D362" s="36" t="n"/>
       <c r="E362" s="19" t="n">
         <v>30</v>
       </c>
@@ -15098,7 +15329,11 @@
           <t>東急電鉄石川台駅</t>
         </is>
       </c>
-      <c r="D363" s="35" t="n"/>
+      <c r="D363" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E363" s="19" t="n">
         <v>10</v>
       </c>
@@ -15135,7 +15370,7 @@
           <t>ローソン＋TOKS　石川台店</t>
         </is>
       </c>
-      <c r="D364" s="19" t="n"/>
+      <c r="D364" s="36" t="n"/>
       <c r="E364" s="19" t="n">
         <v>5</v>
       </c>
@@ -15172,7 +15407,11 @@
           <t>東急雪が谷大塚駅</t>
         </is>
       </c>
-      <c r="D365" s="35" t="n"/>
+      <c r="D365" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E365" s="19" t="n">
         <v>25</v>
       </c>
@@ -15209,7 +15448,7 @@
           <t>roobby　雪が谷大塚駅</t>
         </is>
       </c>
-      <c r="D366" s="19" t="n"/>
+      <c r="D366" s="36" t="n"/>
       <c r="E366" s="19" t="n">
         <v>3</v>
       </c>
@@ -15246,7 +15485,7 @@
           <t>ドトールコーヒー雪谷大塚店</t>
         </is>
       </c>
-      <c r="D367" s="19" t="n"/>
+      <c r="D367" s="36" t="n"/>
       <c r="E367" s="19" t="n">
         <v>5</v>
       </c>
@@ -15283,7 +15522,7 @@
           <t>カラダファクトリー雪谷大塚店</t>
         </is>
       </c>
-      <c r="D368" s="19" t="n"/>
+      <c r="D368" s="36" t="n"/>
       <c r="E368" s="19" t="n">
         <v>1</v>
       </c>
@@ -15320,7 +15559,11 @@
           <t>東急電鉄　武蔵新田駅</t>
         </is>
       </c>
-      <c r="D369" s="35" t="n"/>
+      <c r="D369" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E369" s="19" t="n">
         <v>15</v>
       </c>
@@ -15357,7 +15600,7 @@
           <t>武蔵新田駐輪場</t>
         </is>
       </c>
-      <c r="D370" s="19" t="n"/>
+      <c r="D370" s="36" t="n"/>
       <c r="E370" s="19" t="n">
         <v>0</v>
       </c>
@@ -15394,7 +15637,11 @@
           <t>東急電鉄　下丸子駅</t>
         </is>
       </c>
-      <c r="D371" s="35" t="n"/>
+      <c r="D371" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E371" s="19" t="n">
         <v>20</v>
       </c>
@@ -15431,7 +15678,11 @@
           <t>東急電鉄　鵜の木駅</t>
         </is>
       </c>
-      <c r="D372" s="35" t="n"/>
+      <c r="D372" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E372" s="19" t="n">
         <v>10</v>
       </c>
@@ -15509,7 +15760,7 @@
           <t>ドコモショップサテライト　エトモ鵜の木</t>
         </is>
       </c>
-      <c r="D374" s="19" t="n"/>
+      <c r="D374" s="36" t="n"/>
       <c r="E374" s="19" t="n">
         <v>0</v>
       </c>
@@ -15628,7 +15879,11 @@
           <t>東急電鉄　沼部駅</t>
         </is>
       </c>
-      <c r="D377" s="35" t="n"/>
+      <c r="D377" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E377" s="19" t="n">
         <v>30</v>
       </c>
@@ -15665,7 +15920,11 @@
           <t>東急電鉄　多摩川駅</t>
         </is>
       </c>
-      <c r="D378" s="35" t="n"/>
+      <c r="D378" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E378" s="19" t="n">
         <v>10</v>
       </c>
@@ -15702,7 +15961,7 @@
           <t>ローソン＋多摩川駅店</t>
         </is>
       </c>
-      <c r="D379" s="19" t="n"/>
+      <c r="D379" s="36" t="n"/>
       <c r="E379" s="19" t="n">
         <v>2</v>
       </c>
@@ -15739,7 +15998,11 @@
           <t>東急プロパティマネジメント多摩川班</t>
         </is>
       </c>
-      <c r="D380" s="35" t="n"/>
+      <c r="D380" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E380" s="19" t="n">
         <v>10</v>
       </c>
@@ -15776,7 +16039,7 @@
           <t>リトルマーメイド多摩川店</t>
         </is>
       </c>
-      <c r="D381" s="19" t="n"/>
+      <c r="D381" s="36" t="n"/>
       <c r="E381" s="19" t="n">
         <v>10</v>
       </c>
@@ -15813,7 +16076,11 @@
           <t>東急電鉄　大岡山駅</t>
         </is>
       </c>
-      <c r="D382" s="35" t="n"/>
+      <c r="D382" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E382" s="19" t="n">
         <v>15</v>
       </c>
@@ -15850,7 +16117,11 @@
           <t>東急電鉄　緑が丘駅</t>
         </is>
       </c>
-      <c r="D383" s="35" t="n"/>
+      <c r="D383" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E383" s="19" t="n">
         <v>10</v>
       </c>
@@ -15887,7 +16158,7 @@
           <t>緑が丘エキナカ保育園</t>
         </is>
       </c>
-      <c r="D384" s="19" t="n"/>
+      <c r="D384" s="36" t="n"/>
       <c r="E384" s="19" t="n">
         <v>0</v>
       </c>
@@ -15924,7 +16195,11 @@
           <t>東急電鉄　奥沢駅＆総合ビル</t>
         </is>
       </c>
-      <c r="D385" s="35" t="n"/>
+      <c r="D385" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E385" s="19" t="n">
         <v>35</v>
       </c>
@@ -15961,7 +16236,7 @@
           <t>FRORIST KADAN</t>
         </is>
       </c>
-      <c r="D386" s="19" t="n"/>
+      <c r="D386" s="36" t="n"/>
       <c r="E386" s="19" t="n">
         <v>0</v>
       </c>
@@ -16039,7 +16314,7 @@
           <t>ゴントラン　シェリエmini自由が丘</t>
         </is>
       </c>
-      <c r="D388" s="19" t="n"/>
+      <c r="D388" s="36" t="n"/>
       <c r="E388" s="19" t="n">
         <v>0</v>
       </c>
@@ -16076,7 +16351,7 @@
           <t>丸山珈琲</t>
         </is>
       </c>
-      <c r="D389" s="19" t="n"/>
+      <c r="D389" s="36" t="n"/>
       <c r="E389" s="19" t="n">
         <v>0</v>
       </c>
@@ -16113,7 +16388,7 @@
           <t>ローソン＋TOKS　自由が丘駅</t>
         </is>
       </c>
-      <c r="D390" s="19" t="n"/>
+      <c r="D390" s="36" t="n"/>
       <c r="E390" s="19" t="n">
         <v>10</v>
       </c>
@@ -16150,7 +16425,7 @@
           <t>スープストック　自由が丘店</t>
         </is>
       </c>
-      <c r="D391" s="19" t="n"/>
+      <c r="D391" s="36" t="n"/>
       <c r="E391" s="19" t="n">
         <v>30</v>
       </c>
@@ -16187,7 +16462,7 @@
           <t>TWG　Tea　自由が丘</t>
         </is>
       </c>
-      <c r="D392" s="19" t="n"/>
+      <c r="D392" s="36" t="n"/>
       <c r="E392" s="19" t="n">
         <v>5</v>
       </c>
@@ -16224,7 +16499,11 @@
           <t>東急電鉄　自由が丘駅</t>
         </is>
       </c>
-      <c r="D393" s="35" t="n"/>
+      <c r="D393" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E393" s="19" t="n">
         <v>45</v>
       </c>
@@ -16261,7 +16540,11 @@
           <t>東急ストア　自由が丘駅構内</t>
         </is>
       </c>
-      <c r="D394" s="35" t="n"/>
+      <c r="D394" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E394" s="19" t="n">
         <v>5</v>
       </c>
@@ -16298,7 +16581,7 @@
           <t>Ben's Cookies 自由が丘店</t>
         </is>
       </c>
-      <c r="D395" s="19" t="n"/>
+      <c r="D395" s="36" t="n"/>
       <c r="E395" s="19" t="n">
         <v>0</v>
       </c>
@@ -16335,7 +16618,7 @@
           <t>リンツショコラ　ブティック</t>
         </is>
       </c>
-      <c r="D396" s="19" t="n"/>
+      <c r="D396" s="36" t="n"/>
       <c r="E396" s="19" t="n">
         <v>3</v>
       </c>
@@ -16413,7 +16696,7 @@
           <t>ブランジェ浅野屋　自由が丘店</t>
         </is>
       </c>
-      <c r="D398" s="19" t="n"/>
+      <c r="D398" s="36" t="n"/>
       <c r="E398" s="19" t="n">
         <v>45</v>
       </c>
@@ -16491,7 +16774,7 @@
           <t>NATURAL KITCHEN　自由が丘</t>
         </is>
       </c>
-      <c r="D400" s="19" t="n"/>
+      <c r="D400" s="36" t="n"/>
       <c r="E400" s="19" t="n">
         <v>15</v>
       </c>
@@ -16528,7 +16811,7 @@
           <t>DUMBO Doughnuts</t>
         </is>
       </c>
-      <c r="D401" s="19" t="n"/>
+      <c r="D401" s="36" t="n"/>
       <c r="E401" s="19" t="n">
         <v>0</v>
       </c>
@@ -16647,7 +16930,7 @@
           <t>バガブー</t>
         </is>
       </c>
-      <c r="D404" s="19" t="n"/>
+      <c r="D404" s="36" t="n"/>
       <c r="E404" s="19" t="n">
         <v>0</v>
       </c>
@@ -16684,7 +16967,7 @@
           <t>ドリッピン　チュロス</t>
         </is>
       </c>
-      <c r="D405" s="19" t="n"/>
+      <c r="D405" s="36" t="n"/>
       <c r="E405" s="19" t="n">
         <v>1</v>
       </c>
@@ -16721,7 +17004,7 @@
           <t>トレインチ自由が丘　共有部</t>
         </is>
       </c>
-      <c r="D406" s="21" t="n"/>
+      <c r="D406" s="37" t="n"/>
       <c r="E406" s="19" t="n">
         <v>3</v>
       </c>
@@ -16758,7 +17041,7 @@
           <t>二子玉川乗務区</t>
         </is>
       </c>
-      <c r="D407" s="19" t="n"/>
+      <c r="D407" s="36" t="n"/>
       <c r="E407" s="19" t="n">
         <v>0</v>
       </c>
@@ -16795,7 +17078,7 @@
           <t>二子玉川駅駐輪場</t>
         </is>
       </c>
-      <c r="D408" s="19" t="n"/>
+      <c r="D408" s="36" t="n"/>
       <c r="E408" s="19" t="n">
         <v>5</v>
       </c>
@@ -16832,7 +17115,7 @@
           <t>コーモドドゥーエ</t>
         </is>
       </c>
-      <c r="D409" s="19" t="n"/>
+      <c r="D409" s="36" t="n"/>
       <c r="E409" s="19" t="n">
         <v>0</v>
       </c>
@@ -16869,7 +17152,7 @@
           <t>ファブリック</t>
         </is>
       </c>
-      <c r="D410" s="19" t="n"/>
+      <c r="D410" s="36" t="n"/>
       <c r="E410" s="19" t="n">
         <v>3</v>
       </c>
@@ -16947,7 +17230,7 @@
           <t>サキュレ　本社営業所</t>
         </is>
       </c>
-      <c r="D412" s="19" t="n"/>
+      <c r="D412" s="36" t="n"/>
       <c r="E412" s="19" t="n">
         <v>15</v>
       </c>
@@ -16984,7 +17267,7 @@
           <t>東京ガスリビングラインライフバル西大田</t>
         </is>
       </c>
-      <c r="D413" s="19" t="n"/>
+      <c r="D413" s="36" t="n"/>
       <c r="E413" s="19" t="n">
         <v>40</v>
       </c>
@@ -17021,7 +17304,7 @@
           <t>白百合幼稚園</t>
         </is>
       </c>
-      <c r="D414" s="19" t="n"/>
+      <c r="D414" s="36" t="n"/>
       <c r="E414" s="19" t="n">
         <v>0</v>
       </c>
@@ -17058,7 +17341,7 @@
           <t>MAISON KUROSU</t>
         </is>
       </c>
-      <c r="D415" s="19" t="n"/>
+      <c r="D415" s="36" t="n"/>
       <c r="E415" s="19" t="n">
         <v>0</v>
       </c>
@@ -17095,7 +17378,7 @@
           <t>TOKS　目黒駅</t>
         </is>
       </c>
-      <c r="D416" s="19" t="n"/>
+      <c r="D416" s="36" t="n"/>
       <c r="E416" s="19" t="n">
         <v>0</v>
       </c>
@@ -17132,7 +17415,7 @@
           <t>マツモトキヨシ　目黒店</t>
         </is>
       </c>
-      <c r="D417" s="19" t="n"/>
+      <c r="D417" s="36" t="n"/>
       <c r="E417" s="19" t="n">
         <v>0</v>
       </c>
@@ -17169,7 +17452,7 @@
           <t>キッズスペースキャンプ　大井町</t>
         </is>
       </c>
-      <c r="D418" s="19" t="n"/>
+      <c r="D418" s="36" t="n"/>
       <c r="E418" s="19" t="n">
         <v>0</v>
       </c>
@@ -17206,7 +17489,7 @@
           <t>KBCほいくえん　大井町</t>
         </is>
       </c>
-      <c r="D419" s="19" t="n"/>
+      <c r="D419" s="36" t="n"/>
       <c r="E419" s="19" t="n">
         <v>0</v>
       </c>
@@ -17243,7 +17526,11 @@
           <t>東急プロパティマネジメント大井班</t>
         </is>
       </c>
-      <c r="D420" s="35" t="n"/>
+      <c r="D420" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E420" s="19" t="n">
         <v>0</v>
       </c>
@@ -17280,7 +17567,7 @@
           <t>第一商事</t>
         </is>
       </c>
-      <c r="D421" s="19" t="n"/>
+      <c r="D421" s="36" t="n"/>
       <c r="E421" s="19" t="n">
         <v>10</v>
       </c>
@@ -17317,7 +17604,11 @@
           <t>東急電鉄　蒲田駅</t>
         </is>
       </c>
-      <c r="D422" s="35" t="n"/>
+      <c r="D422" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E422" s="19" t="n">
         <v>35</v>
       </c>
@@ -17354,7 +17645,7 @@
           <t>ミスターミニット　蒲田駅店</t>
         </is>
       </c>
-      <c r="D423" s="19" t="n"/>
+      <c r="D423" s="36" t="n"/>
       <c r="E423" s="19" t="n">
         <v>20</v>
       </c>
@@ -17391,7 +17682,7 @@
           <t>住まいと暮らしのコンシェルジュ</t>
         </is>
       </c>
-      <c r="D424" s="19" t="n"/>
+      <c r="D424" s="36" t="n"/>
       <c r="E424" s="19" t="n">
         <v>5</v>
       </c>
@@ -17428,7 +17719,7 @@
           <t>TOKS　蒲田改札口店</t>
         </is>
       </c>
-      <c r="D425" s="19" t="n"/>
+      <c r="D425" s="36" t="n"/>
       <c r="E425" s="19" t="n">
         <v>10</v>
       </c>
@@ -17465,7 +17756,11 @@
           <t>東急電鉄　池上駅</t>
         </is>
       </c>
-      <c r="D426" s="35" t="n"/>
+      <c r="D426" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E426" s="19" t="n">
         <v>35</v>
       </c>
@@ -17502,7 +17797,11 @@
           <t>東急電鉄　蓮沼駅</t>
         </is>
       </c>
-      <c r="D427" s="35" t="n"/>
+      <c r="D427" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E427" s="19" t="n">
         <v>5</v>
       </c>
@@ -17539,7 +17838,11 @@
           <t>東急電鉄　矢口渡駅</t>
         </is>
       </c>
-      <c r="D428" s="35" t="n"/>
+      <c r="D428" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E428" s="19" t="n">
         <v>15</v>
       </c>
@@ -17658,7 +17961,7 @@
           <t>学校法人上野塾東京高等学校</t>
         </is>
       </c>
-      <c r="D431" s="19" t="n"/>
+      <c r="D431" s="36" t="n"/>
       <c r="E431" s="19" t="n">
         <v>40</v>
       </c>
@@ -17695,7 +17998,7 @@
           <t>日本ロジテム三幸営業所</t>
         </is>
       </c>
-      <c r="D432" s="19" t="n"/>
+      <c r="D432" s="36" t="n"/>
       <c r="E432" s="19" t="n">
         <v>80</v>
       </c>
@@ -17732,7 +18035,11 @@
           <t>東急電鉄　千鳥町駅</t>
         </is>
       </c>
-      <c r="D433" s="35" t="n"/>
+      <c r="D433" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E433" s="19" t="n">
         <v>10</v>
       </c>
@@ -17769,7 +18076,11 @@
           <t>東急電鉄　久が原駅</t>
         </is>
       </c>
-      <c r="D434" s="35" t="n"/>
+      <c r="D434" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E434" s="19" t="n">
         <v>10</v>
       </c>
@@ -17806,7 +18117,11 @@
           <t>東急電鉄　御嶽山駅</t>
         </is>
       </c>
-      <c r="D435" s="35" t="n"/>
+      <c r="D435" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E435" s="19" t="n">
         <v>15</v>
       </c>
@@ -17843,7 +18158,11 @@
           <t>東急電鉄渋谷駅（副都心線）</t>
         </is>
       </c>
-      <c r="D436" s="35" t="n"/>
+      <c r="D436" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E436" s="19" t="n">
         <v>25</v>
       </c>
@@ -17880,7 +18199,7 @@
           <t>キャンバン</t>
         </is>
       </c>
-      <c r="D437" s="19" t="n"/>
+      <c r="D437" s="36" t="n"/>
       <c r="E437" s="19" t="n">
         <v>3</v>
       </c>
@@ -17917,7 +18236,7 @@
           <t>デルフォニックス</t>
         </is>
       </c>
-      <c r="D438" s="19" t="n"/>
+      <c r="D438" s="36" t="n"/>
       <c r="E438" s="19" t="n">
         <v>5</v>
       </c>
@@ -17954,7 +18273,11 @@
           <t>東急電鉄　三軒茶屋（田園都市線）</t>
         </is>
       </c>
-      <c r="D439" s="35" t="n"/>
+      <c r="D439" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E439" s="19" t="n">
         <v>30</v>
       </c>
@@ -17987,7 +18310,7 @@
           <t>ローソン＋TOKS　三軒茶屋店</t>
         </is>
       </c>
-      <c r="D440" s="19" t="n"/>
+      <c r="D440" s="36" t="n"/>
       <c r="E440" s="19" t="n">
         <v>20</v>
       </c>
@@ -18020,7 +18343,11 @@
           <t>東急電鉄　三軒茶屋（世田谷線）</t>
         </is>
       </c>
-      <c r="D441" s="35" t="n"/>
+      <c r="D441" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E441" s="19" t="n">
         <v>3</v>
       </c>
@@ -18053,7 +18380,11 @@
           <t>東急電鉄　上町駅</t>
         </is>
       </c>
-      <c r="D442" s="35" t="n"/>
+      <c r="D442" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E442" s="19" t="n">
         <v>0</v>
       </c>
@@ -18127,7 +18458,11 @@
           <t>東急電鉄　長原駅</t>
         </is>
       </c>
-      <c r="D444" s="35" t="n"/>
+      <c r="D444" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E444" s="19" t="n">
         <v>10</v>
       </c>
@@ -18164,7 +18499,11 @@
           <t>東急電鉄　洗足池駅</t>
         </is>
       </c>
-      <c r="D445" s="35" t="n"/>
+      <c r="D445" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E445" s="19" t="n">
         <v>10</v>
       </c>
@@ -18201,7 +18540,11 @@
           <t>東急電鉄　北千束駅</t>
         </is>
       </c>
-      <c r="D446" s="35" t="n"/>
+      <c r="D446" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E446" s="19" t="n">
         <v>5</v>
       </c>
@@ -18238,7 +18581,11 @@
           <t>東急電鉄　洗足駅</t>
         </is>
       </c>
-      <c r="D447" s="35" t="n"/>
+      <c r="D447" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E447" s="19" t="n">
         <v>5</v>
       </c>
@@ -18275,7 +18622,7 @@
           <t>西小山（南）駐輪場</t>
         </is>
       </c>
-      <c r="D448" s="19" t="n"/>
+      <c r="D448" s="36" t="n"/>
       <c r="E448" s="19" t="n">
         <v>0</v>
       </c>
@@ -18312,7 +18659,11 @@
           <t>東急電鉄　西小山駅</t>
         </is>
       </c>
-      <c r="D449" s="35" t="n"/>
+      <c r="D449" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E449" s="19" t="n">
         <v>10</v>
       </c>
@@ -18349,7 +18700,7 @@
           <t>武蔵小山西口駐輪場</t>
         </is>
       </c>
-      <c r="D450" s="19" t="n"/>
+      <c r="D450" s="36" t="n"/>
       <c r="E450" s="19" t="n">
         <v>0</v>
       </c>
@@ -18386,7 +18737,11 @@
           <t>東急電鉄　武蔵小山駅</t>
         </is>
       </c>
-      <c r="D451" s="35" t="n"/>
+      <c r="D451" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E451" s="19" t="n">
         <v>5</v>
       </c>
@@ -18423,7 +18778,11 @@
           <t>東急電鉄　目黒駅</t>
         </is>
       </c>
-      <c r="D452" s="35" t="n"/>
+      <c r="D452" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E452" s="19" t="n">
         <v>20</v>
       </c>
@@ -18460,7 +18819,11 @@
           <t>東急電鉄　五反田駅　４F</t>
         </is>
       </c>
-      <c r="D453" s="35" t="n"/>
+      <c r="D453" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E453" s="19" t="n">
         <v>0</v>
       </c>
@@ -18497,7 +18860,11 @@
           <t>TOKS　五反田駅店</t>
         </is>
       </c>
-      <c r="D454" s="35" t="n"/>
+      <c r="D454" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E454" s="19" t="n">
         <v>0</v>
       </c>
@@ -18534,7 +18901,7 @@
           <t>メガネスーパーコンタクト五反田エキナカ店</t>
         </is>
       </c>
-      <c r="D455" s="19" t="n"/>
+      <c r="D455" s="36" t="n"/>
       <c r="E455" s="19" t="n">
         <v>0</v>
       </c>
@@ -18571,7 +18938,11 @@
           <t>東急電鉄　五反田駅　１F</t>
         </is>
       </c>
-      <c r="D456" s="35" t="n"/>
+      <c r="D456" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E456" s="19" t="n">
         <v>3</v>
       </c>
@@ -18608,7 +18979,11 @@
           <t>東急電鉄　荏原中延駅</t>
         </is>
       </c>
-      <c r="D457" s="35" t="n"/>
+      <c r="D457" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E457" s="19" t="n">
         <v>1</v>
       </c>
@@ -18645,7 +19020,7 @@
           <t>荏原中延駐輪場</t>
         </is>
       </c>
-      <c r="D458" s="19" t="n"/>
+      <c r="D458" s="36" t="n"/>
       <c r="E458" s="19" t="n">
         <v>10</v>
       </c>
@@ -18682,7 +19057,11 @@
           <t>東急電鉄　戸越公園駅</t>
         </is>
       </c>
-      <c r="D459" s="35" t="n"/>
+      <c r="D459" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E459" s="19" t="n">
         <v>0</v>
       </c>
@@ -18719,7 +19098,7 @@
           <t>サキュレ本社営業所</t>
         </is>
       </c>
-      <c r="D460" s="19" t="n"/>
+      <c r="D460" s="36" t="n"/>
       <c r="E460" s="19" t="n">
         <v>5</v>
       </c>
@@ -18756,7 +19135,11 @@
           <t>東急電鉄　旗の台駅</t>
         </is>
       </c>
-      <c r="D461" s="35" t="n"/>
+      <c r="D461" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E461" s="19" t="n">
         <v>15</v>
       </c>
@@ -18793,7 +19176,7 @@
           <t>ミスターワッフル　旗の台エキナカ店</t>
         </is>
       </c>
-      <c r="D462" s="19" t="n"/>
+      <c r="D462" s="36" t="n"/>
       <c r="E462" s="19" t="n">
         <v>5</v>
       </c>
@@ -18830,7 +19213,7 @@
           <t>グローバルキッズ　荏原町保育園</t>
         </is>
       </c>
-      <c r="D463" s="19" t="n"/>
+      <c r="D463" s="36" t="n"/>
       <c r="E463" s="19" t="n">
         <v>20</v>
       </c>
@@ -18867,7 +19250,11 @@
           <t>東急電鉄　荏原町駅</t>
         </is>
       </c>
-      <c r="D464" s="35" t="n"/>
+      <c r="D464" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E464" s="19" t="n">
         <v>0</v>
       </c>
@@ -18904,7 +19291,11 @@
           <t>東急電鉄　中延駅</t>
         </is>
       </c>
-      <c r="D465" s="35" t="n"/>
+      <c r="D465" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E465" s="19" t="n">
         <v>0</v>
       </c>
@@ -18941,7 +19332,7 @@
           <t>中延駐輪場</t>
         </is>
       </c>
-      <c r="D466" s="19" t="n"/>
+      <c r="D466" s="36" t="n"/>
       <c r="E466" s="19" t="n">
         <v>0</v>
       </c>
@@ -18978,7 +19369,11 @@
           <t>東急電鉄　戸越銀座駅</t>
         </is>
       </c>
-      <c r="D467" s="35" t="n"/>
+      <c r="D467" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E467" s="19" t="n">
         <v>15</v>
       </c>
@@ -19015,7 +19410,11 @@
           <t>東急ウェルネス本社事務所</t>
         </is>
       </c>
-      <c r="D468" s="35" t="n"/>
+      <c r="D468" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E468" s="19" t="n">
         <v>6</v>
       </c>
@@ -19052,7 +19451,11 @@
           <t>東急電鉄　大崎広小路駅</t>
         </is>
       </c>
-      <c r="D469" s="35" t="n"/>
+      <c r="D469" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E469" s="19" t="n">
         <v>10</v>
       </c>
@@ -19089,7 +19492,11 @@
           <t>東急電鉄　不動前駅</t>
         </is>
       </c>
-      <c r="D470" s="35" t="n"/>
+      <c r="D470" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E470" s="19" t="n">
         <v>0</v>
       </c>
@@ -19126,7 +19533,7 @@
           <t>TOKS 不動前駅</t>
         </is>
       </c>
-      <c r="D471" s="19" t="n"/>
+      <c r="D471" s="36" t="n"/>
       <c r="E471" s="19" t="n">
         <v>5</v>
       </c>
@@ -19163,7 +19570,11 @@
           <t>東急都立大学高架下共用部</t>
         </is>
       </c>
-      <c r="D472" s="35" t="n"/>
+      <c r="D472" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E472" s="19" t="n">
         <v>0</v>
       </c>
@@ -19200,7 +19611,11 @@
           <t>東急電鉄　下神明駅</t>
         </is>
       </c>
-      <c r="D473" s="35" t="n"/>
+      <c r="D473" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E473" s="19" t="n">
         <v>5</v>
       </c>
@@ -19237,7 +19652,7 @@
           <t>しぶそば大井町店</t>
         </is>
       </c>
-      <c r="D474" s="19" t="n"/>
+      <c r="D474" s="36" t="n"/>
       <c r="E474" s="19" t="n">
         <v>10</v>
       </c>
@@ -19274,7 +19689,7 @@
           <t>大崎電気工業所</t>
         </is>
       </c>
-      <c r="D475" s="19" t="n"/>
+      <c r="D475" s="36" t="n"/>
       <c r="E475" s="19" t="n">
         <v>30</v>
       </c>
@@ -19311,7 +19726,7 @@
           <t>古賀電機株式会社</t>
         </is>
       </c>
-      <c r="D476" s="19" t="n"/>
+      <c r="D476" s="36" t="n"/>
       <c r="E476" s="19" t="n">
         <v>85</v>
       </c>
@@ -19348,7 +19763,7 @@
           <t>古賀電機(株)新第二工場</t>
         </is>
       </c>
-      <c r="D477" s="19" t="n"/>
+      <c r="D477" s="36" t="n"/>
       <c r="E477" s="19" t="n">
         <v>85</v>
       </c>
@@ -19385,7 +19800,7 @@
           <t>古賀電機第三工場</t>
         </is>
       </c>
-      <c r="D478" s="19" t="n"/>
+      <c r="D478" s="36" t="n"/>
       <c r="E478" s="19" t="n">
         <v>30</v>
       </c>
@@ -19422,7 +19837,7 @@
           <t>堤工業</t>
         </is>
       </c>
-      <c r="D479" s="19" t="n"/>
+      <c r="D479" s="36" t="n"/>
       <c r="E479" s="19" t="n">
         <v>40</v>
       </c>
@@ -19459,7 +19874,7 @@
           <t>共立工芸</t>
         </is>
       </c>
-      <c r="D480" s="19" t="n"/>
+      <c r="D480" s="36" t="n"/>
       <c r="E480" s="19" t="n">
         <v>35</v>
       </c>
@@ -19496,7 +19911,7 @@
           <t>山崎製作所</t>
         </is>
       </c>
-      <c r="D481" s="19" t="n"/>
+      <c r="D481" s="36" t="n"/>
       <c r="E481" s="19" t="n">
         <v>65</v>
       </c>
@@ -19533,7 +19948,11 @@
           <t>東急電鉄　二子玉川乗務区</t>
         </is>
       </c>
-      <c r="D482" s="35" t="n"/>
+      <c r="D482" s="19" t="inlineStr">
+        <is>
+          <t>東急グループ</t>
+        </is>
+      </c>
       <c r="E482" s="19" t="n">
         <v>0</v>
       </c>
@@ -19570,7 +19989,7 @@
           <t>マツモトキヨシ　荏原町駅前店</t>
         </is>
       </c>
-      <c r="D483" s="19" t="n"/>
+      <c r="D483" s="36" t="n"/>
       <c r="E483" s="19" t="n">
         <v>30</v>
       </c>
@@ -19607,7 +20026,7 @@
           <t>カラダファクトリー　雪谷大塚店</t>
         </is>
       </c>
-      <c r="D484" s="19" t="n"/>
+      <c r="D484" s="36" t="n"/>
       <c r="E484" s="19" t="n">
         <v>10</v>
       </c>
@@ -19644,7 +20063,7 @@
           <t>中目黒高架下A</t>
         </is>
       </c>
-      <c r="D485" s="19" t="n"/>
+      <c r="D485" s="36" t="n"/>
       <c r="E485" s="19" t="n">
         <v>15</v>
       </c>
@@ -19681,7 +20100,7 @@
           <t>中目黒高架下B</t>
         </is>
       </c>
-      <c r="D486" s="19" t="n"/>
+      <c r="D486" s="36" t="n"/>
       <c r="E486" s="19" t="n">
         <v>50</v>
       </c>
@@ -19718,7 +20137,7 @@
           <t>中目黒高架下D</t>
         </is>
       </c>
-      <c r="D487" s="19" t="n"/>
+      <c r="D487" s="36" t="n"/>
       <c r="E487" s="19" t="n">
         <v>20</v>
       </c>
@@ -19755,7 +20174,7 @@
           <t>中目黒高架下F</t>
         </is>
       </c>
-      <c r="D488" s="19" t="n"/>
+      <c r="D488" s="36" t="n"/>
       <c r="E488" s="19" t="n">
         <v>20</v>
       </c>
@@ -19792,7 +20211,7 @@
           <t>中目黒高架下G</t>
         </is>
       </c>
-      <c r="D489" s="19" t="n"/>
+      <c r="D489" s="36" t="n"/>
       <c r="E489" s="19" t="n">
         <v>20</v>
       </c>
@@ -19829,7 +20248,7 @@
           <t>中目黒高架下H</t>
         </is>
       </c>
-      <c r="D490" s="19" t="n"/>
+      <c r="D490" s="36" t="n"/>
       <c r="E490" s="19" t="n">
         <v>5</v>
       </c>
@@ -19866,7 +20285,7 @@
           <t>中目黒高架下J</t>
         </is>
       </c>
-      <c r="D491" s="19" t="n"/>
+      <c r="D491" s="36" t="n"/>
       <c r="E491" s="19" t="n">
         <v>0</v>
       </c>
@@ -19903,7 +20322,7 @@
           <t>学芸大学高架下（１０BL）</t>
         </is>
       </c>
-      <c r="D492" s="19" t="n"/>
+      <c r="D492" s="36" t="n"/>
       <c r="E492" s="19" t="n">
         <v>10</v>
       </c>
@@ -19940,7 +20359,7 @@
           <t>学芸大学高架下（１３BL）</t>
         </is>
       </c>
-      <c r="D493" s="19" t="n"/>
+      <c r="D493" s="36" t="n"/>
       <c r="E493" s="19" t="n">
         <v>140</v>
       </c>
@@ -19977,7 +20396,7 @@
           <t>学芸大学高架下（１４BL）</t>
         </is>
       </c>
-      <c r="D494" s="19" t="n"/>
+      <c r="D494" s="36" t="n"/>
       <c r="E494" s="19" t="n">
         <v>60</v>
       </c>
@@ -20014,7 +20433,7 @@
           <t>グルメフロント（１５BL）</t>
         </is>
       </c>
-      <c r="D495" s="19" t="n"/>
+      <c r="D495" s="36" t="n"/>
       <c r="E495" s="19" t="n">
         <v>10</v>
       </c>
@@ -20051,7 +20470,7 @@
           <t>学大コレクティブ（１６BL）</t>
         </is>
       </c>
-      <c r="D496" s="19" t="n"/>
+      <c r="D496" s="36" t="n"/>
       <c r="E496" s="19" t="n">
         <v>10</v>
       </c>
@@ -20088,7 +20507,7 @@
           <t>自由が丘駅/北口</t>
         </is>
       </c>
-      <c r="D497" s="19" t="n"/>
+      <c r="D497" s="36" t="n"/>
       <c r="E497" s="19" t="n">
         <v>100</v>
       </c>
@@ -20125,7 +20544,7 @@
           <t>自由が丘駅/南口</t>
         </is>
       </c>
-      <c r="D498" s="19" t="n"/>
+      <c r="D498" s="36" t="n"/>
       <c r="E498" s="19" t="n">
         <v>30</v>
       </c>
@@ -20162,7 +20581,7 @@
           <t>エトモ　荏原町店</t>
         </is>
       </c>
-      <c r="D499" s="19" t="n"/>
+      <c r="D499" s="36" t="n"/>
       <c r="E499" s="19" t="n">
         <v>40</v>
       </c>
@@ -20199,7 +20618,7 @@
           <t>ケンタッキーフライドチキン　二子玉川店</t>
         </is>
       </c>
-      <c r="D500" s="19" t="n"/>
+      <c r="D500" s="36" t="n"/>
       <c r="E500" s="19" t="n">
         <v>90</v>
       </c>
@@ -20236,7 +20655,7 @@
           <t>MAISON KUROSU　学芸大学</t>
         </is>
       </c>
-      <c r="D501" s="19" t="n"/>
+      <c r="D501" s="36" t="n"/>
       <c r="E501" s="19" t="n">
         <v>0</v>
       </c>
@@ -61279,11 +61698,11 @@
       <c r="C11" s="7" t="n">
         <v>14800</v>
       </c>
-      <c r="D11" s="39" t="n">
+      <c r="D11" s="38" t="n">
         <v>0.02702702702702697</v>
       </c>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="39" t="n"/>
+      <c r="F11" s="38" t="n"/>
       <c r="G11" s="7" t="n">
         <v>0.0053504</v>
       </c>
@@ -61300,11 +61719,11 @@
       <c r="C12" s="7" t="n">
         <v>2300</v>
       </c>
-      <c r="D12" s="39" t="n">
+      <c r="D12" s="38" t="n">
         <v>-0.08695652173913049</v>
       </c>
       <c r="E12" s="7" t="n"/>
-      <c r="F12" s="39" t="n"/>
+      <c r="F12" s="38" t="n"/>
       <c r="G12" s="7" t="n">
         <v>4.851e-05</v>
       </c>
@@ -61321,11 +61740,11 @@
       <c r="C13" s="7" t="n">
         <v>3100</v>
       </c>
-      <c r="D13" s="39" t="n">
+      <c r="D13" s="38" t="n">
         <v>0.09677419354838701</v>
       </c>
       <c r="E13" s="7" t="n"/>
-      <c r="F13" s="39" t="n"/>
+      <c r="F13" s="38" t="n"/>
       <c r="G13" s="7" t="n">
         <v>0.00012546</v>
       </c>
@@ -61342,11 +61761,11 @@
       <c r="C14" s="7" t="n">
         <v>1900</v>
       </c>
-      <c r="D14" s="39" t="n">
+      <c r="D14" s="38" t="n">
         <v>-0.05263157894736847</v>
       </c>
       <c r="E14" s="7" t="n"/>
-      <c r="F14" s="39" t="n"/>
+      <c r="F14" s="38" t="n"/>
       <c r="G14" s="7" t="n">
         <v>4.158e-05</v>
       </c>
@@ -61363,11 +61782,11 @@
       <c r="C15" s="7" t="n">
         <v>750</v>
       </c>
-      <c r="D15" s="39" t="n">
+      <c r="D15" s="38" t="n">
         <v>0.06666666666666665</v>
       </c>
       <c r="E15" s="7" t="n"/>
-      <c r="F15" s="39" t="n"/>
+      <c r="F15" s="38" t="n"/>
       <c r="G15" s="7" t="n">
         <v>2.952e-05</v>
       </c>
@@ -61384,11 +61803,11 @@
       <c r="C16" s="11" t="n">
         <v>22850</v>
       </c>
-      <c r="D16" s="40" t="n">
+      <c r="D16" s="39" t="n">
         <v>0.01969365426695835</v>
       </c>
       <c r="E16" s="11" t="n"/>
-      <c r="F16" s="40" t="n"/>
+      <c r="F16" s="39" t="n"/>
       <c r="G16" s="11" t="n">
         <v>0</v>
       </c>
@@ -61819,7 +62238,7 @@
       <c r="D11" s="7" t="n">
         <v>0.06336</v>
       </c>
-      <c r="E11" s="39" t="n">
+      <c r="E11" s="38" t="n">
         <v>0.719585420672408</v>
       </c>
     </row>
@@ -61838,7 +62257,7 @@
       <c r="D12" s="7" t="n">
         <v>0.0005775</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="38" t="n">
         <v>0.006558721282170386</v>
       </c>
     </row>
@@ -61857,7 +62276,7 @@
       <c r="D13" s="7" t="n">
         <v>0.001476</v>
       </c>
-      <c r="E13" s="39" t="n">
+      <c r="E13" s="38" t="n">
         <v>0.01676306945884587</v>
       </c>
     </row>
@@ -61876,7 +62295,7 @@
       <c r="D14" s="7" t="n">
         <v>0.0005082</v>
       </c>
-      <c r="E14" s="39" t="n">
+      <c r="E14" s="38" t="n">
         <v>0.00577167472830994</v>
       </c>
     </row>
@@ -61895,7 +62314,7 @@
       <c r="D15" s="7" t="n">
         <v>0.000369</v>
       </c>
-      <c r="E15" s="39" t="n">
+      <c r="E15" s="38" t="n">
         <v>0.004190767364711468</v>
       </c>
     </row>
@@ -61914,7 +62333,7 @@
       <c r="D16" s="7" t="n">
         <v>0.02176</v>
       </c>
-      <c r="E16" s="39" t="n">
+      <c r="E16" s="38" t="n">
         <v>0.2471303464935543</v>
       </c>
     </row>
@@ -61931,7 +62350,7 @@
       <c r="D17" s="11" t="n">
         <v>0.0880507</v>
       </c>
-      <c r="E17" s="40" t="inlineStr">
+      <c r="E17" s="39" t="inlineStr">
         <is>
           <t>100%</t>
         </is>

</xml_diff>

<commit_message>
Add fuzzy-matched D column entries in red font (23 rows)
Partial/normalized matching between v5 C column and 板橋 B column.
23 cells filled with red font + yellow background for user review.
117 cells remain blank with yellow highlight pending manual input.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -26,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
@@ -138,6 +138,9 @@
       <i val="1"/>
       <color rgb="FF595959"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <color rgb="00FF0000"/>
     </font>
   </fonts>
   <fills count="9">
@@ -278,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -328,8 +331,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7984,7 +7990,11 @@
           <t>あらちゃん</t>
         </is>
       </c>
-      <c r="D178" s="35" t="n"/>
+      <c r="D178" s="35" t="inlineStr">
+        <is>
+          <t>モスアイズリ－（株）アイデイ－ あらちゃん</t>
+        </is>
+      </c>
       <c r="E178" s="19" t="n">
         <v>10</v>
       </c>
@@ -8743,7 +8753,11 @@
           <t>CHANCEジム中目黒店</t>
         </is>
       </c>
-      <c r="D197" s="36" t="n"/>
+      <c r="D197" s="37" t="inlineStr">
+        <is>
+          <t>ＣＨＡＮＣＥ　ジム　中目黒</t>
+        </is>
+      </c>
       <c r="E197" s="19" t="n">
         <v>3</v>
       </c>
@@ -10798,7 +10812,11 @@
           <t>MAISON KUROSU学芸</t>
         </is>
       </c>
-      <c r="D248" s="36" t="n"/>
+      <c r="D248" s="37" t="inlineStr">
+        <is>
+          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
+        </is>
+      </c>
       <c r="E248" s="19" t="n">
         <v>30</v>
       </c>
@@ -14179,7 +14197,11 @@
           <t>学校法人　聖ドミニコ学園</t>
         </is>
       </c>
-      <c r="D333" s="36" t="n"/>
+      <c r="D333" s="37" t="inlineStr">
+        <is>
+          <t>聖ドミニコ学園</t>
+        </is>
+      </c>
       <c r="E333" s="19" t="n">
         <v>120</v>
       </c>
@@ -14216,7 +14238,11 @@
           <t>東京リーガルマインド　水道橋本校</t>
         </is>
       </c>
-      <c r="D334" s="36" t="n"/>
+      <c r="D334" s="37" t="inlineStr">
+        <is>
+          <t>（株）東京リーガルマインド</t>
+        </is>
+      </c>
       <c r="E334" s="19" t="n">
         <v>30</v>
       </c>
@@ -14561,7 +14587,11 @@
           <t>さみしがりや酒房　ささ</t>
         </is>
       </c>
-      <c r="D343" s="36" t="n"/>
+      <c r="D343" s="37" t="inlineStr">
+        <is>
+          <t>さみしがりや酒房　ささ</t>
+        </is>
+      </c>
       <c r="E343" s="19" t="n">
         <v>0</v>
       </c>
@@ -14672,7 +14702,11 @@
           <t>イケマル酒場</t>
         </is>
       </c>
-      <c r="D346" s="36" t="n"/>
+      <c r="D346" s="37" t="inlineStr">
+        <is>
+          <t>イケマル酒場（株）ロ－タスファイブ</t>
+        </is>
+      </c>
       <c r="E346" s="19" t="n">
         <v>0</v>
       </c>
@@ -16351,7 +16385,11 @@
           <t>丸山珈琲</t>
         </is>
       </c>
-      <c r="D389" s="36" t="n"/>
+      <c r="D389" s="37" t="inlineStr">
+        <is>
+          <t>（株）丸山珈琲</t>
+        </is>
+      </c>
       <c r="E389" s="19" t="n">
         <v>0</v>
       </c>
@@ -17004,7 +17042,7 @@
           <t>トレインチ自由が丘　共有部</t>
         </is>
       </c>
-      <c r="D406" s="37" t="n"/>
+      <c r="D406" s="38" t="n"/>
       <c r="E406" s="19" t="n">
         <v>3</v>
       </c>
@@ -17152,7 +17190,11 @@
           <t>ファブリック</t>
         </is>
       </c>
-      <c r="D410" s="36" t="n"/>
+      <c r="D410" s="37" t="inlineStr">
+        <is>
+          <t>マレンロウ.グル－プ．ジャパン（株）ファブリック</t>
+        </is>
+      </c>
       <c r="E410" s="19" t="n">
         <v>3</v>
       </c>
@@ -17267,7 +17309,11 @@
           <t>東京ガスリビングラインライフバル西大田</t>
         </is>
       </c>
-      <c r="D413" s="36" t="n"/>
+      <c r="D413" s="37" t="inlineStr">
+        <is>
+          <t>東京ガスリビングライン（株）</t>
+        </is>
+      </c>
       <c r="E413" s="19" t="n">
         <v>40</v>
       </c>
@@ -17304,7 +17350,11 @@
           <t>白百合幼稚園</t>
         </is>
       </c>
-      <c r="D414" s="36" t="n"/>
+      <c r="D414" s="37" t="inlineStr">
+        <is>
+          <t>白百合幼稚園（つくしの学園</t>
+        </is>
+      </c>
       <c r="E414" s="19" t="n">
         <v>0</v>
       </c>
@@ -17341,7 +17391,11 @@
           <t>MAISON KUROSU</t>
         </is>
       </c>
-      <c r="D415" s="36" t="n"/>
+      <c r="D415" s="37" t="inlineStr">
+        <is>
+          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
+        </is>
+      </c>
       <c r="E415" s="19" t="n">
         <v>0</v>
       </c>
@@ -17998,7 +18052,11 @@
           <t>日本ロジテム三幸営業所</t>
         </is>
       </c>
-      <c r="D432" s="36" t="n"/>
+      <c r="D432" s="37" t="inlineStr">
+        <is>
+          <t>日本ロジテム（株）</t>
+        </is>
+      </c>
       <c r="E432" s="19" t="n">
         <v>80</v>
       </c>
@@ -18199,7 +18257,11 @@
           <t>キャンバン</t>
         </is>
       </c>
-      <c r="D437" s="36" t="n"/>
+      <c r="D437" s="37" t="inlineStr">
+        <is>
+          <t>（株）キャンバン</t>
+        </is>
+      </c>
       <c r="E437" s="19" t="n">
         <v>3</v>
       </c>
@@ -18236,7 +18298,11 @@
           <t>デルフォニックス</t>
         </is>
       </c>
-      <c r="D438" s="36" t="n"/>
+      <c r="D438" s="37" t="inlineStr">
+        <is>
+          <t>（株）デルフォニックス</t>
+        </is>
+      </c>
       <c r="E438" s="19" t="n">
         <v>5</v>
       </c>
@@ -18901,7 +18967,11 @@
           <t>メガネスーパーコンタクト五反田エキナカ店</t>
         </is>
       </c>
-      <c r="D455" s="36" t="n"/>
+      <c r="D455" s="37" t="inlineStr">
+        <is>
+          <t>（株）メガネスーパー</t>
+        </is>
+      </c>
       <c r="E455" s="19" t="n">
         <v>0</v>
       </c>
@@ -19726,7 +19796,11 @@
           <t>古賀電機株式会社</t>
         </is>
       </c>
-      <c r="D476" s="36" t="n"/>
+      <c r="D476" s="37" t="inlineStr">
+        <is>
+          <t>古賀電機（株）</t>
+        </is>
+      </c>
       <c r="E476" s="19" t="n">
         <v>85</v>
       </c>
@@ -19763,7 +19837,11 @@
           <t>古賀電機(株)新第二工場</t>
         </is>
       </c>
-      <c r="D477" s="36" t="n"/>
+      <c r="D477" s="37" t="inlineStr">
+        <is>
+          <t>古賀電機（株）</t>
+        </is>
+      </c>
       <c r="E477" s="19" t="n">
         <v>85</v>
       </c>
@@ -19800,7 +19878,11 @@
           <t>古賀電機第三工場</t>
         </is>
       </c>
-      <c r="D478" s="36" t="n"/>
+      <c r="D478" s="37" t="inlineStr">
+        <is>
+          <t>古賀電機（株）</t>
+        </is>
+      </c>
       <c r="E478" s="19" t="n">
         <v>30</v>
       </c>
@@ -19837,7 +19919,11 @@
           <t>堤工業</t>
         </is>
       </c>
-      <c r="D479" s="36" t="n"/>
+      <c r="D479" s="37" t="inlineStr">
+        <is>
+          <t>堤工業（株）</t>
+        </is>
+      </c>
       <c r="E479" s="19" t="n">
         <v>40</v>
       </c>
@@ -19874,7 +19960,11 @@
           <t>共立工芸</t>
         </is>
       </c>
-      <c r="D480" s="36" t="n"/>
+      <c r="D480" s="37" t="inlineStr">
+        <is>
+          <t>（株）共立工芸</t>
+        </is>
+      </c>
       <c r="E480" s="19" t="n">
         <v>35</v>
       </c>
@@ -19911,7 +20001,11 @@
           <t>山崎製作所</t>
         </is>
       </c>
-      <c r="D481" s="36" t="n"/>
+      <c r="D481" s="37" t="inlineStr">
+        <is>
+          <t>（株）山崎製作所</t>
+        </is>
+      </c>
       <c r="E481" s="19" t="n">
         <v>65</v>
       </c>
@@ -20655,7 +20749,11 @@
           <t>MAISON KUROSU　学芸大学</t>
         </is>
       </c>
-      <c r="D501" s="36" t="n"/>
+      <c r="D501" s="37" t="inlineStr">
+        <is>
+          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
+        </is>
+      </c>
       <c r="E501" s="19" t="n">
         <v>0</v>
       </c>
@@ -61698,11 +61796,11 @@
       <c r="C11" s="7" t="n">
         <v>14800</v>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="39" t="n">
         <v>0.02702702702702697</v>
       </c>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="38" t="n"/>
+      <c r="F11" s="39" t="n"/>
       <c r="G11" s="7" t="n">
         <v>0.0053504</v>
       </c>
@@ -61719,11 +61817,11 @@
       <c r="C12" s="7" t="n">
         <v>2300</v>
       </c>
-      <c r="D12" s="38" t="n">
+      <c r="D12" s="39" t="n">
         <v>-0.08695652173913049</v>
       </c>
       <c r="E12" s="7" t="n"/>
-      <c r="F12" s="38" t="n"/>
+      <c r="F12" s="39" t="n"/>
       <c r="G12" s="7" t="n">
         <v>4.851e-05</v>
       </c>
@@ -61740,11 +61838,11 @@
       <c r="C13" s="7" t="n">
         <v>3100</v>
       </c>
-      <c r="D13" s="38" t="n">
+      <c r="D13" s="39" t="n">
         <v>0.09677419354838701</v>
       </c>
       <c r="E13" s="7" t="n"/>
-      <c r="F13" s="38" t="n"/>
+      <c r="F13" s="39" t="n"/>
       <c r="G13" s="7" t="n">
         <v>0.00012546</v>
       </c>
@@ -61761,11 +61859,11 @@
       <c r="C14" s="7" t="n">
         <v>1900</v>
       </c>
-      <c r="D14" s="38" t="n">
+      <c r="D14" s="39" t="n">
         <v>-0.05263157894736847</v>
       </c>
       <c r="E14" s="7" t="n"/>
-      <c r="F14" s="38" t="n"/>
+      <c r="F14" s="39" t="n"/>
       <c r="G14" s="7" t="n">
         <v>4.158e-05</v>
       </c>
@@ -61782,11 +61880,11 @@
       <c r="C15" s="7" t="n">
         <v>750</v>
       </c>
-      <c r="D15" s="38" t="n">
+      <c r="D15" s="39" t="n">
         <v>0.06666666666666665</v>
       </c>
       <c r="E15" s="7" t="n"/>
-      <c r="F15" s="38" t="n"/>
+      <c r="F15" s="39" t="n"/>
       <c r="G15" s="7" t="n">
         <v>2.952e-05</v>
       </c>
@@ -61803,11 +61901,11 @@
       <c r="C16" s="11" t="n">
         <v>22850</v>
       </c>
-      <c r="D16" s="39" t="n">
+      <c r="D16" s="40" t="n">
         <v>0.01969365426695835</v>
       </c>
       <c r="E16" s="11" t="n"/>
-      <c r="F16" s="39" t="n"/>
+      <c r="F16" s="40" t="n"/>
       <c r="G16" s="11" t="n">
         <v>0</v>
       </c>
@@ -62238,7 +62336,7 @@
       <c r="D11" s="7" t="n">
         <v>0.06336</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="39" t="n">
         <v>0.719585420672408</v>
       </c>
     </row>
@@ -62257,7 +62355,7 @@
       <c r="D12" s="7" t="n">
         <v>0.0005775</v>
       </c>
-      <c r="E12" s="38" t="n">
+      <c r="E12" s="39" t="n">
         <v>0.006558721282170386</v>
       </c>
     </row>
@@ -62276,7 +62374,7 @@
       <c r="D13" s="7" t="n">
         <v>0.001476</v>
       </c>
-      <c r="E13" s="38" t="n">
+      <c r="E13" s="39" t="n">
         <v>0.01676306945884587</v>
       </c>
     </row>
@@ -62295,7 +62393,7 @@
       <c r="D14" s="7" t="n">
         <v>0.0005082</v>
       </c>
-      <c r="E14" s="38" t="n">
+      <c r="E14" s="39" t="n">
         <v>0.00577167472830994</v>
       </c>
     </row>
@@ -62314,7 +62412,7 @@
       <c r="D15" s="7" t="n">
         <v>0.000369</v>
       </c>
-      <c r="E15" s="38" t="n">
+      <c r="E15" s="39" t="n">
         <v>0.004190767364711468</v>
       </c>
     </row>
@@ -62333,7 +62431,7 @@
       <c r="D16" s="7" t="n">
         <v>0.02176</v>
       </c>
-      <c r="E16" s="38" t="n">
+      <c r="E16" s="39" t="n">
         <v>0.2471303464935543</v>
       </c>
     </row>
@@ -62350,7 +62448,7 @@
       <c r="D17" s="11" t="n">
         <v>0.0880507</v>
       </c>
-      <c r="E17" s="39" t="inlineStr">
+      <c r="E17" s="40" t="inlineStr">
         <is>
           <t>100%</t>
         </is>

</xml_diff>

<commit_message>
Add Tokyu-related D column predictions in blue font (45 rows)
Pattern-based matching for 東急（株）facilities (高架下, 駐輪場,
TOKS, 乗務区 etc.), （株）浅野屋 (リトルマーメイド), 東急キッズ,
スープストック. Yellow background retained. ~72 cells still pending.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -140,7 +140,7 @@
       <sz val="8"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="000000FF"/>
     </font>
   </fonts>
   <fills count="9">
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -331,14 +331,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -7990,11 +7986,7 @@
           <t>あらちゃん</t>
         </is>
       </c>
-      <c r="D178" s="35" t="inlineStr">
-        <is>
-          <t>モスアイズリ－（株）アイデイ－ あらちゃん</t>
-        </is>
-      </c>
+      <c r="D178" s="25" t="n"/>
       <c r="E178" s="19" t="n">
         <v>10</v>
       </c>
@@ -8277,7 +8269,7 @@
           <t>ASReal</t>
         </is>
       </c>
-      <c r="D185" s="36" t="n"/>
+      <c r="D185" s="19" t="n"/>
       <c r="E185" s="19" t="n">
         <v>0</v>
       </c>
@@ -8314,7 +8306,7 @@
           <t>ALWAYS OUT OF STOCK</t>
         </is>
       </c>
-      <c r="D186" s="36" t="n"/>
+      <c r="D186" s="19" t="n"/>
       <c r="E186" s="19" t="n">
         <v>0</v>
       </c>
@@ -8474,7 +8466,7 @@
           <t>GYM by LAVISUS</t>
         </is>
       </c>
-      <c r="D190" s="36" t="n"/>
+      <c r="D190" s="19" t="n"/>
       <c r="E190" s="19" t="n">
         <v>0</v>
       </c>
@@ -8552,7 +8544,7 @@
           <t>曼茶羅</t>
         </is>
       </c>
-      <c r="D192" s="36" t="n"/>
+      <c r="D192" s="19" t="n"/>
       <c r="E192" s="19" t="n">
         <v>0</v>
       </c>
@@ -8753,11 +8745,7 @@
           <t>CHANCEジム中目黒店</t>
         </is>
       </c>
-      <c r="D197" s="37" t="inlineStr">
-        <is>
-          <t>ＣＨＡＮＣＥ　ジム　中目黒</t>
-        </is>
-      </c>
+      <c r="D197" s="19" t="n"/>
       <c r="E197" s="19" t="n">
         <v>3</v>
       </c>
@@ -9122,7 +9110,7 @@
           <t>GOOD LUCK 中目黒店</t>
         </is>
       </c>
-      <c r="D206" s="36" t="n"/>
+      <c r="D206" s="19" t="n"/>
       <c r="E206" s="19" t="n">
         <v>5</v>
       </c>
@@ -9938,7 +9926,7 @@
           <t>Mix Bar Rose</t>
         </is>
       </c>
-      <c r="D226" s="36" t="n"/>
+      <c r="D226" s="19" t="n"/>
       <c r="E226" s="19" t="n">
         <v>0</v>
       </c>
@@ -9975,7 +9963,7 @@
           <t>sazan reef</t>
         </is>
       </c>
-      <c r="D227" s="36" t="n"/>
+      <c r="D227" s="19" t="n"/>
       <c r="E227" s="19" t="n">
         <v>1</v>
       </c>
@@ -10012,7 +10000,7 @@
           <t>CHI-FO</t>
         </is>
       </c>
-      <c r="D228" s="36" t="n"/>
+      <c r="D228" s="19" t="n"/>
       <c r="E228" s="19" t="n">
         <v>5</v>
       </c>
@@ -10172,7 +10160,11 @@
           <t>１０BL共用部分</t>
         </is>
       </c>
-      <c r="D232" s="36" t="n"/>
+      <c r="D232" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E232" s="19" t="n">
         <v>0</v>
       </c>
@@ -10332,7 +10324,7 @@
           <t>鮮魚　北浜　学芸大学店</t>
         </is>
       </c>
-      <c r="D236" s="36" t="n"/>
+      <c r="D236" s="19" t="n"/>
       <c r="E236" s="19" t="n">
         <v>5</v>
       </c>
@@ -10492,7 +10484,7 @@
           <t>学大マーチ＆シーズンカフェ</t>
         </is>
       </c>
-      <c r="D240" s="36" t="n"/>
+      <c r="D240" s="19" t="n"/>
       <c r="E240" s="19" t="n">
         <v>0</v>
       </c>
@@ -10570,7 +10562,7 @@
           <t>そばもん　学大店</t>
         </is>
       </c>
-      <c r="D242" s="36" t="n"/>
+      <c r="D242" s="19" t="n"/>
       <c r="E242" s="19" t="n">
         <v>5</v>
       </c>
@@ -10812,11 +10804,7 @@
           <t>MAISON KUROSU学芸</t>
         </is>
       </c>
-      <c r="D248" s="37" t="inlineStr">
-        <is>
-          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
-        </is>
-      </c>
+      <c r="D248" s="19" t="n"/>
       <c r="E248" s="19" t="n">
         <v>30</v>
       </c>
@@ -11550,7 +11538,7 @@
           <t>DEAN&amp;DELUCA</t>
         </is>
       </c>
-      <c r="D266" s="36" t="n"/>
+      <c r="D266" s="19" t="n"/>
       <c r="E266" s="19" t="n">
         <v>80</v>
       </c>
@@ -11751,7 +11739,7 @@
           <t>あの小宮</t>
         </is>
       </c>
-      <c r="D271" s="36" t="n"/>
+      <c r="D271" s="19" t="n"/>
       <c r="E271" s="19" t="n">
         <v>100</v>
       </c>
@@ -11870,7 +11858,7 @@
           <t>あーる工房</t>
         </is>
       </c>
-      <c r="D274" s="36" t="n"/>
+      <c r="D274" s="19" t="n"/>
       <c r="E274" s="19" t="n">
         <v>1</v>
       </c>
@@ -11948,7 +11936,11 @@
           <t>NewWork　都立大</t>
         </is>
       </c>
-      <c r="D276" s="36" t="n"/>
+      <c r="D276" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E276" s="19" t="n">
         <v>0</v>
       </c>
@@ -12149,7 +12141,7 @@
           <t>サーティーワンアイスクリーム</t>
         </is>
       </c>
-      <c r="D281" s="36" t="n"/>
+      <c r="D281" s="19" t="n"/>
       <c r="E281" s="19" t="n">
         <v>1</v>
       </c>
@@ -12186,7 +12178,7 @@
           <t>ルナアース</t>
         </is>
       </c>
-      <c r="D282" s="36" t="n"/>
+      <c r="D282" s="19" t="n"/>
       <c r="E282" s="19" t="n">
         <v>0</v>
       </c>
@@ -12264,7 +12256,7 @@
           <t>オープンマート駒澤大学駅中店</t>
         </is>
       </c>
-      <c r="D284" s="36" t="n"/>
+      <c r="D284" s="19" t="n"/>
       <c r="E284" s="19" t="n">
         <v>0</v>
       </c>
@@ -12301,7 +12293,7 @@
           <t>オハナ　明大前</t>
         </is>
       </c>
-      <c r="D285" s="36" t="n"/>
+      <c r="D285" s="19" t="n"/>
       <c r="E285" s="19" t="n">
         <v>40</v>
       </c>
@@ -12543,7 +12535,7 @@
           <t>roobby-fit 下高井戸店</t>
         </is>
       </c>
-      <c r="D291" s="36" t="n"/>
+      <c r="D291" s="19" t="n"/>
       <c r="E291" s="19" t="n">
         <v>0</v>
       </c>
@@ -12703,7 +12695,7 @@
           <t>MY SWEETS　渋谷店</t>
         </is>
       </c>
-      <c r="D295" s="36" t="n"/>
+      <c r="D295" s="19" t="n"/>
       <c r="E295" s="19" t="n">
         <v>0</v>
       </c>
@@ -12740,7 +12732,11 @@
           <t>ランキンランキン渋谷店</t>
         </is>
       </c>
-      <c r="D296" s="36" t="n"/>
+      <c r="D296" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E296" s="19" t="n">
         <v>5</v>
       </c>
@@ -12777,7 +12773,7 @@
           <t>白洋舎　東京支店</t>
         </is>
       </c>
-      <c r="D297" s="36" t="n"/>
+      <c r="D297" s="19" t="n"/>
       <c r="E297" s="19" t="n">
         <v>150</v>
       </c>
@@ -12814,7 +12810,7 @@
           <t>河合塾　本郷校</t>
         </is>
       </c>
-      <c r="D298" s="36" t="n"/>
+      <c r="D298" s="19" t="n"/>
       <c r="E298" s="19" t="n">
         <v>100</v>
       </c>
@@ -12974,7 +12970,7 @@
           <t>南大塚エースビル</t>
         </is>
       </c>
-      <c r="D302" s="36" t="n"/>
+      <c r="D302" s="19" t="n"/>
       <c r="E302" s="19" t="n">
         <v>45</v>
       </c>
@@ -13011,7 +13007,7 @@
           <t>(株)ハピラル・テストソリューションズ</t>
         </is>
       </c>
-      <c r="D303" s="36" t="n"/>
+      <c r="D303" s="19" t="n"/>
       <c r="E303" s="19" t="n">
         <v>15</v>
       </c>
@@ -13212,7 +13208,7 @@
           <t>ミスターミニット　用賀店</t>
         </is>
       </c>
-      <c r="D308" s="36" t="n"/>
+      <c r="D308" s="19" t="n"/>
       <c r="E308" s="19" t="n">
         <v>5</v>
       </c>
@@ -13454,7 +13450,7 @@
           <t>スタジオマリオグラン　二子玉川店</t>
         </is>
       </c>
-      <c r="D314" s="36" t="n"/>
+      <c r="D314" s="19" t="n"/>
       <c r="E314" s="19" t="n">
         <v>5</v>
       </c>
@@ -13614,7 +13610,7 @@
           <t>こもれび保育園　上野毛園</t>
         </is>
       </c>
-      <c r="D318" s="36" t="n"/>
+      <c r="D318" s="19" t="n"/>
       <c r="E318" s="19" t="n">
         <v>20</v>
       </c>
@@ -13651,7 +13647,7 @@
           <t>あおい皮膚科　駅ナカ上野毛</t>
         </is>
       </c>
-      <c r="D319" s="36" t="n"/>
+      <c r="D319" s="19" t="n"/>
       <c r="E319" s="19" t="n">
         <v>0</v>
       </c>
@@ -13688,7 +13684,11 @@
           <t>大井町線上野毛駅構内店舗</t>
         </is>
       </c>
-      <c r="D320" s="36" t="n"/>
+      <c r="D320" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E320" s="19" t="n">
         <v>0</v>
       </c>
@@ -13889,7 +13889,7 @@
           <t>フラマンドール　田園調布店</t>
         </is>
       </c>
-      <c r="D325" s="36" t="n"/>
+      <c r="D325" s="19" t="n"/>
       <c r="E325" s="19" t="n">
         <v>50</v>
       </c>
@@ -14049,7 +14049,11 @@
           <t>日吉エリア</t>
         </is>
       </c>
-      <c r="D329" s="36" t="n"/>
+      <c r="D329" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E329" s="19" t="n">
         <v>5</v>
       </c>
@@ -14086,7 +14090,11 @@
           <t>リトルマーメイド　多摩川店</t>
         </is>
       </c>
-      <c r="D330" s="36" t="n"/>
+      <c r="D330" s="35" t="inlineStr">
+        <is>
+          <t>（株）浅野屋</t>
+        </is>
+      </c>
       <c r="E330" s="19" t="n">
         <v>20</v>
       </c>
@@ -14123,7 +14131,11 @@
           <t>しぶそば　多摩川店</t>
         </is>
       </c>
-      <c r="D331" s="36" t="n"/>
+      <c r="D331" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E331" s="19" t="n">
         <v>20</v>
       </c>
@@ -14160,7 +14172,7 @@
           <t>銀座マギー　商品センター</t>
         </is>
       </c>
-      <c r="D332" s="36" t="n"/>
+      <c r="D332" s="19" t="n"/>
       <c r="E332" s="19" t="n">
         <v>70</v>
       </c>
@@ -14197,11 +14209,7 @@
           <t>学校法人　聖ドミニコ学園</t>
         </is>
       </c>
-      <c r="D333" s="37" t="inlineStr">
-        <is>
-          <t>聖ドミニコ学園</t>
-        </is>
-      </c>
+      <c r="D333" s="19" t="n"/>
       <c r="E333" s="19" t="n">
         <v>120</v>
       </c>
@@ -14238,11 +14246,7 @@
           <t>東京リーガルマインド　水道橋本校</t>
         </is>
       </c>
-      <c r="D334" s="37" t="inlineStr">
-        <is>
-          <t>（株）東京リーガルマインド</t>
-        </is>
-      </c>
+      <c r="D334" s="19" t="n"/>
       <c r="E334" s="19" t="n">
         <v>30</v>
       </c>
@@ -14402,7 +14406,7 @@
           <t>天才キッズクラブ楽学館仲池上園</t>
         </is>
       </c>
-      <c r="D338" s="36" t="n"/>
+      <c r="D338" s="19" t="n"/>
       <c r="E338" s="19" t="n">
         <v>0</v>
       </c>
@@ -14439,7 +14443,7 @@
           <t>Far Yeast Brewing</t>
         </is>
       </c>
-      <c r="D339" s="36" t="n"/>
+      <c r="D339" s="19" t="n"/>
       <c r="E339" s="19" t="n">
         <v>10</v>
       </c>
@@ -14476,7 +14480,7 @@
           <t>貝々　味海</t>
         </is>
       </c>
-      <c r="D340" s="36" t="n"/>
+      <c r="D340" s="19" t="n"/>
       <c r="E340" s="19" t="n">
         <v>3</v>
       </c>
@@ -14513,7 +14517,7 @@
           <t>東京食堂</t>
         </is>
       </c>
-      <c r="D341" s="36" t="n"/>
+      <c r="D341" s="19" t="n"/>
       <c r="E341" s="19" t="n">
         <v>0</v>
       </c>
@@ -14550,7 +14554,7 @@
           <t>ファットバー</t>
         </is>
       </c>
-      <c r="D342" s="36" t="n"/>
+      <c r="D342" s="19" t="n"/>
       <c r="E342" s="19" t="n">
         <v>0</v>
       </c>
@@ -14587,11 +14591,7 @@
           <t>さみしがりや酒房　ささ</t>
         </is>
       </c>
-      <c r="D343" s="37" t="inlineStr">
-        <is>
-          <t>さみしがりや酒房　ささ</t>
-        </is>
-      </c>
+      <c r="D343" s="19" t="n"/>
       <c r="E343" s="19" t="n">
         <v>0</v>
       </c>
@@ -14628,7 +14628,7 @@
           <t>居酒屋めぐろ川前</t>
         </is>
       </c>
-      <c r="D344" s="36" t="n"/>
+      <c r="D344" s="19" t="n"/>
       <c r="E344" s="19" t="n">
         <v>2</v>
       </c>
@@ -14665,7 +14665,7 @@
           <t>キッチン　クレセント</t>
         </is>
       </c>
-      <c r="D345" s="36" t="n"/>
+      <c r="D345" s="19" t="n"/>
       <c r="E345" s="19" t="n">
         <v>0</v>
       </c>
@@ -14702,11 +14702,7 @@
           <t>イケマル酒場</t>
         </is>
       </c>
-      <c r="D346" s="37" t="inlineStr">
-        <is>
-          <t>イケマル酒場（株）ロ－タスファイブ</t>
-        </is>
-      </c>
+      <c r="D346" s="19" t="n"/>
       <c r="E346" s="19" t="n">
         <v>0</v>
       </c>
@@ -14743,7 +14739,7 @@
           <t>桜小路　共用部</t>
         </is>
       </c>
-      <c r="D347" s="36" t="n"/>
+      <c r="D347" s="19" t="n"/>
       <c r="E347" s="19" t="n">
         <v>0</v>
       </c>
@@ -14862,7 +14858,7 @@
           <t>スターバックスコーヒー大井町駅</t>
         </is>
       </c>
-      <c r="D350" s="36" t="n"/>
+      <c r="D350" s="19" t="n"/>
       <c r="E350" s="19" t="n">
         <v>45</v>
       </c>
@@ -14899,7 +14895,7 @@
           <t>MY SWEETS　大井町店</t>
         </is>
       </c>
-      <c r="D351" s="36" t="n"/>
+      <c r="D351" s="19" t="n"/>
       <c r="E351" s="19" t="n">
         <v>0</v>
       </c>
@@ -14936,7 +14932,7 @@
           <t>えん　大井町店</t>
         </is>
       </c>
-      <c r="D352" s="36" t="n"/>
+      <c r="D352" s="19" t="n"/>
       <c r="E352" s="19" t="n">
         <v>35</v>
       </c>
@@ -14973,7 +14969,7 @@
           <t>E-style大井町校</t>
         </is>
       </c>
-      <c r="D353" s="36" t="n"/>
+      <c r="D353" s="19" t="n"/>
       <c r="E353" s="19" t="n">
         <v>0</v>
       </c>
@@ -15092,7 +15088,11 @@
           <t>都立大学高架下共用部</t>
         </is>
       </c>
-      <c r="D356" s="36" t="n"/>
+      <c r="D356" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E356" s="19" t="n">
         <v>0</v>
       </c>
@@ -15211,7 +15211,7 @@
           <t>ロッジ</t>
         </is>
       </c>
-      <c r="D359" s="36" t="n"/>
+      <c r="D359" s="19" t="n"/>
       <c r="E359" s="19" t="n">
         <v>0</v>
       </c>
@@ -15248,7 +15248,7 @@
           <t>(株)銀座マギー　田園調布ビル</t>
         </is>
       </c>
-      <c r="D360" s="36" t="n"/>
+      <c r="D360" s="19" t="n"/>
       <c r="E360" s="19" t="n">
         <v>15</v>
       </c>
@@ -15326,7 +15326,7 @@
           <t>丸三ストアー</t>
         </is>
       </c>
-      <c r="D362" s="36" t="n"/>
+      <c r="D362" s="19" t="n"/>
       <c r="E362" s="19" t="n">
         <v>30</v>
       </c>
@@ -15404,7 +15404,11 @@
           <t>ローソン＋TOKS　石川台店</t>
         </is>
       </c>
-      <c r="D364" s="36" t="n"/>
+      <c r="D364" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E364" s="19" t="n">
         <v>5</v>
       </c>
@@ -15482,7 +15486,7 @@
           <t>roobby　雪が谷大塚駅</t>
         </is>
       </c>
-      <c r="D366" s="36" t="n"/>
+      <c r="D366" s="19" t="n"/>
       <c r="E366" s="19" t="n">
         <v>3</v>
       </c>
@@ -15519,7 +15523,7 @@
           <t>ドトールコーヒー雪谷大塚店</t>
         </is>
       </c>
-      <c r="D367" s="36" t="n"/>
+      <c r="D367" s="19" t="n"/>
       <c r="E367" s="19" t="n">
         <v>5</v>
       </c>
@@ -15556,7 +15560,7 @@
           <t>カラダファクトリー雪谷大塚店</t>
         </is>
       </c>
-      <c r="D368" s="36" t="n"/>
+      <c r="D368" s="19" t="n"/>
       <c r="E368" s="19" t="n">
         <v>1</v>
       </c>
@@ -15634,7 +15638,11 @@
           <t>武蔵新田駐輪場</t>
         </is>
       </c>
-      <c r="D370" s="36" t="n"/>
+      <c r="D370" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E370" s="19" t="n">
         <v>0</v>
       </c>
@@ -15794,7 +15802,11 @@
           <t>ドコモショップサテライト　エトモ鵜の木</t>
         </is>
       </c>
-      <c r="D374" s="36" t="n"/>
+      <c r="D374" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E374" s="19" t="n">
         <v>0</v>
       </c>
@@ -15995,7 +16007,11 @@
           <t>ローソン＋多摩川駅店</t>
         </is>
       </c>
-      <c r="D379" s="36" t="n"/>
+      <c r="D379" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E379" s="19" t="n">
         <v>2</v>
       </c>
@@ -16073,7 +16089,11 @@
           <t>リトルマーメイド多摩川店</t>
         </is>
       </c>
-      <c r="D381" s="36" t="n"/>
+      <c r="D381" s="35" t="inlineStr">
+        <is>
+          <t>（株）浅野屋</t>
+        </is>
+      </c>
       <c r="E381" s="19" t="n">
         <v>10</v>
       </c>
@@ -16192,7 +16212,7 @@
           <t>緑が丘エキナカ保育園</t>
         </is>
       </c>
-      <c r="D384" s="36" t="n"/>
+      <c r="D384" s="19" t="n"/>
       <c r="E384" s="19" t="n">
         <v>0</v>
       </c>
@@ -16270,7 +16290,7 @@
           <t>FRORIST KADAN</t>
         </is>
       </c>
-      <c r="D386" s="36" t="n"/>
+      <c r="D386" s="19" t="n"/>
       <c r="E386" s="19" t="n">
         <v>0</v>
       </c>
@@ -16348,7 +16368,7 @@
           <t>ゴントラン　シェリエmini自由が丘</t>
         </is>
       </c>
-      <c r="D388" s="36" t="n"/>
+      <c r="D388" s="19" t="n"/>
       <c r="E388" s="19" t="n">
         <v>0</v>
       </c>
@@ -16385,11 +16405,7 @@
           <t>丸山珈琲</t>
         </is>
       </c>
-      <c r="D389" s="37" t="inlineStr">
-        <is>
-          <t>（株）丸山珈琲</t>
-        </is>
-      </c>
+      <c r="D389" s="19" t="n"/>
       <c r="E389" s="19" t="n">
         <v>0</v>
       </c>
@@ -16426,7 +16442,11 @@
           <t>ローソン＋TOKS　自由が丘駅</t>
         </is>
       </c>
-      <c r="D390" s="36" t="n"/>
+      <c r="D390" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E390" s="19" t="n">
         <v>10</v>
       </c>
@@ -16463,7 +16483,11 @@
           <t>スープストック　自由が丘店</t>
         </is>
       </c>
-      <c r="D391" s="36" t="n"/>
+      <c r="D391" s="35" t="inlineStr">
+        <is>
+          <t>（株）スープストックト－キョ－</t>
+        </is>
+      </c>
       <c r="E391" s="19" t="n">
         <v>30</v>
       </c>
@@ -16500,7 +16524,7 @@
           <t>TWG　Tea　自由が丘</t>
         </is>
       </c>
-      <c r="D392" s="36" t="n"/>
+      <c r="D392" s="19" t="n"/>
       <c r="E392" s="19" t="n">
         <v>5</v>
       </c>
@@ -16619,7 +16643,7 @@
           <t>Ben's Cookies 自由が丘店</t>
         </is>
       </c>
-      <c r="D395" s="36" t="n"/>
+      <c r="D395" s="19" t="n"/>
       <c r="E395" s="19" t="n">
         <v>0</v>
       </c>
@@ -16656,7 +16680,7 @@
           <t>リンツショコラ　ブティック</t>
         </is>
       </c>
-      <c r="D396" s="36" t="n"/>
+      <c r="D396" s="19" t="n"/>
       <c r="E396" s="19" t="n">
         <v>3</v>
       </c>
@@ -16734,7 +16758,11 @@
           <t>ブランジェ浅野屋　自由が丘店</t>
         </is>
       </c>
-      <c r="D398" s="36" t="n"/>
+      <c r="D398" s="35" t="inlineStr">
+        <is>
+          <t>（株）浅野屋</t>
+        </is>
+      </c>
       <c r="E398" s="19" t="n">
         <v>45</v>
       </c>
@@ -16812,7 +16840,7 @@
           <t>NATURAL KITCHEN　自由が丘</t>
         </is>
       </c>
-      <c r="D400" s="36" t="n"/>
+      <c r="D400" s="19" t="n"/>
       <c r="E400" s="19" t="n">
         <v>15</v>
       </c>
@@ -16849,7 +16877,7 @@
           <t>DUMBO Doughnuts</t>
         </is>
       </c>
-      <c r="D401" s="36" t="n"/>
+      <c r="D401" s="19" t="n"/>
       <c r="E401" s="19" t="n">
         <v>0</v>
       </c>
@@ -16968,7 +16996,7 @@
           <t>バガブー</t>
         </is>
       </c>
-      <c r="D404" s="36" t="n"/>
+      <c r="D404" s="19" t="n"/>
       <c r="E404" s="19" t="n">
         <v>0</v>
       </c>
@@ -17005,7 +17033,7 @@
           <t>ドリッピン　チュロス</t>
         </is>
       </c>
-      <c r="D405" s="36" t="n"/>
+      <c r="D405" s="19" t="n"/>
       <c r="E405" s="19" t="n">
         <v>1</v>
       </c>
@@ -17042,7 +17070,11 @@
           <t>トレインチ自由が丘　共有部</t>
         </is>
       </c>
-      <c r="D406" s="38" t="n"/>
+      <c r="D406" s="36" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E406" s="19" t="n">
         <v>3</v>
       </c>
@@ -17079,7 +17111,11 @@
           <t>二子玉川乗務区</t>
         </is>
       </c>
-      <c r="D407" s="36" t="n"/>
+      <c r="D407" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E407" s="19" t="n">
         <v>0</v>
       </c>
@@ -17116,7 +17152,11 @@
           <t>二子玉川駅駐輪場</t>
         </is>
       </c>
-      <c r="D408" s="36" t="n"/>
+      <c r="D408" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E408" s="19" t="n">
         <v>5</v>
       </c>
@@ -17153,7 +17193,7 @@
           <t>コーモドドゥーエ</t>
         </is>
       </c>
-      <c r="D409" s="36" t="n"/>
+      <c r="D409" s="19" t="n"/>
       <c r="E409" s="19" t="n">
         <v>0</v>
       </c>
@@ -17190,11 +17230,7 @@
           <t>ファブリック</t>
         </is>
       </c>
-      <c r="D410" s="37" t="inlineStr">
-        <is>
-          <t>マレンロウ.グル－プ．ジャパン（株）ファブリック</t>
-        </is>
-      </c>
+      <c r="D410" s="19" t="n"/>
       <c r="E410" s="19" t="n">
         <v>3</v>
       </c>
@@ -17272,7 +17308,7 @@
           <t>サキュレ　本社営業所</t>
         </is>
       </c>
-      <c r="D412" s="36" t="n"/>
+      <c r="D412" s="19" t="n"/>
       <c r="E412" s="19" t="n">
         <v>15</v>
       </c>
@@ -17309,11 +17345,7 @@
           <t>東京ガスリビングラインライフバル西大田</t>
         </is>
       </c>
-      <c r="D413" s="37" t="inlineStr">
-        <is>
-          <t>東京ガスリビングライン（株）</t>
-        </is>
-      </c>
+      <c r="D413" s="19" t="n"/>
       <c r="E413" s="19" t="n">
         <v>40</v>
       </c>
@@ -17350,11 +17382,7 @@
           <t>白百合幼稚園</t>
         </is>
       </c>
-      <c r="D414" s="37" t="inlineStr">
-        <is>
-          <t>白百合幼稚園（つくしの学園</t>
-        </is>
-      </c>
+      <c r="D414" s="19" t="n"/>
       <c r="E414" s="19" t="n">
         <v>0</v>
       </c>
@@ -17391,11 +17419,7 @@
           <t>MAISON KUROSU</t>
         </is>
       </c>
-      <c r="D415" s="37" t="inlineStr">
-        <is>
-          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
-        </is>
-      </c>
+      <c r="D415" s="19" t="n"/>
       <c r="E415" s="19" t="n">
         <v>0</v>
       </c>
@@ -17432,7 +17456,11 @@
           <t>TOKS　目黒駅</t>
         </is>
       </c>
-      <c r="D416" s="36" t="n"/>
+      <c r="D416" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E416" s="19" t="n">
         <v>0</v>
       </c>
@@ -17469,7 +17497,7 @@
           <t>マツモトキヨシ　目黒店</t>
         </is>
       </c>
-      <c r="D417" s="36" t="n"/>
+      <c r="D417" s="19" t="n"/>
       <c r="E417" s="19" t="n">
         <v>0</v>
       </c>
@@ -17506,7 +17534,11 @@
           <t>キッズスペースキャンプ　大井町</t>
         </is>
       </c>
-      <c r="D418" s="36" t="n"/>
+      <c r="D418" s="35" t="inlineStr">
+        <is>
+          <t>（株）東急キッズボ－ルキャンプ大井町</t>
+        </is>
+      </c>
       <c r="E418" s="19" t="n">
         <v>0</v>
       </c>
@@ -17543,7 +17575,11 @@
           <t>KBCほいくえん　大井町</t>
         </is>
       </c>
-      <c r="D419" s="36" t="n"/>
+      <c r="D419" s="35" t="inlineStr">
+        <is>
+          <t>（株）東急キッズボ－ルキャンプ大井町</t>
+        </is>
+      </c>
       <c r="E419" s="19" t="n">
         <v>0</v>
       </c>
@@ -17621,7 +17657,7 @@
           <t>第一商事</t>
         </is>
       </c>
-      <c r="D421" s="36" t="n"/>
+      <c r="D421" s="19" t="n"/>
       <c r="E421" s="19" t="n">
         <v>10</v>
       </c>
@@ -17699,7 +17735,7 @@
           <t>ミスターミニット　蒲田駅店</t>
         </is>
       </c>
-      <c r="D423" s="36" t="n"/>
+      <c r="D423" s="19" t="n"/>
       <c r="E423" s="19" t="n">
         <v>20</v>
       </c>
@@ -17736,7 +17772,7 @@
           <t>住まいと暮らしのコンシェルジュ</t>
         </is>
       </c>
-      <c r="D424" s="36" t="n"/>
+      <c r="D424" s="19" t="n"/>
       <c r="E424" s="19" t="n">
         <v>5</v>
       </c>
@@ -17773,7 +17809,11 @@
           <t>TOKS　蒲田改札口店</t>
         </is>
       </c>
-      <c r="D425" s="36" t="n"/>
+      <c r="D425" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E425" s="19" t="n">
         <v>10</v>
       </c>
@@ -18015,7 +18055,7 @@
           <t>学校法人上野塾東京高等学校</t>
         </is>
       </c>
-      <c r="D431" s="36" t="n"/>
+      <c r="D431" s="19" t="n"/>
       <c r="E431" s="19" t="n">
         <v>40</v>
       </c>
@@ -18052,11 +18092,7 @@
           <t>日本ロジテム三幸営業所</t>
         </is>
       </c>
-      <c r="D432" s="37" t="inlineStr">
-        <is>
-          <t>日本ロジテム（株）</t>
-        </is>
-      </c>
+      <c r="D432" s="19" t="n"/>
       <c r="E432" s="19" t="n">
         <v>80</v>
       </c>
@@ -18257,11 +18293,7 @@
           <t>キャンバン</t>
         </is>
       </c>
-      <c r="D437" s="37" t="inlineStr">
-        <is>
-          <t>（株）キャンバン</t>
-        </is>
-      </c>
+      <c r="D437" s="19" t="n"/>
       <c r="E437" s="19" t="n">
         <v>3</v>
       </c>
@@ -18298,11 +18330,7 @@
           <t>デルフォニックス</t>
         </is>
       </c>
-      <c r="D438" s="37" t="inlineStr">
-        <is>
-          <t>（株）デルフォニックス</t>
-        </is>
-      </c>
+      <c r="D438" s="19" t="n"/>
       <c r="E438" s="19" t="n">
         <v>5</v>
       </c>
@@ -18376,7 +18404,11 @@
           <t>ローソン＋TOKS　三軒茶屋店</t>
         </is>
       </c>
-      <c r="D440" s="36" t="n"/>
+      <c r="D440" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E440" s="19" t="n">
         <v>20</v>
       </c>
@@ -18688,7 +18720,11 @@
           <t>西小山（南）駐輪場</t>
         </is>
       </c>
-      <c r="D448" s="36" t="n"/>
+      <c r="D448" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E448" s="19" t="n">
         <v>0</v>
       </c>
@@ -18766,7 +18802,11 @@
           <t>武蔵小山西口駐輪場</t>
         </is>
       </c>
-      <c r="D450" s="36" t="n"/>
+      <c r="D450" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E450" s="19" t="n">
         <v>0</v>
       </c>
@@ -18967,11 +19007,7 @@
           <t>メガネスーパーコンタクト五反田エキナカ店</t>
         </is>
       </c>
-      <c r="D455" s="37" t="inlineStr">
-        <is>
-          <t>（株）メガネスーパー</t>
-        </is>
-      </c>
+      <c r="D455" s="19" t="n"/>
       <c r="E455" s="19" t="n">
         <v>0</v>
       </c>
@@ -19090,7 +19126,11 @@
           <t>荏原中延駐輪場</t>
         </is>
       </c>
-      <c r="D458" s="36" t="n"/>
+      <c r="D458" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E458" s="19" t="n">
         <v>10</v>
       </c>
@@ -19168,7 +19208,7 @@
           <t>サキュレ本社営業所</t>
         </is>
       </c>
-      <c r="D460" s="36" t="n"/>
+      <c r="D460" s="19" t="n"/>
       <c r="E460" s="19" t="n">
         <v>5</v>
       </c>
@@ -19246,7 +19286,7 @@
           <t>ミスターワッフル　旗の台エキナカ店</t>
         </is>
       </c>
-      <c r="D462" s="36" t="n"/>
+      <c r="D462" s="19" t="n"/>
       <c r="E462" s="19" t="n">
         <v>5</v>
       </c>
@@ -19283,7 +19323,7 @@
           <t>グローバルキッズ　荏原町保育園</t>
         </is>
       </c>
-      <c r="D463" s="36" t="n"/>
+      <c r="D463" s="19" t="n"/>
       <c r="E463" s="19" t="n">
         <v>20</v>
       </c>
@@ -19402,7 +19442,11 @@
           <t>中延駐輪場</t>
         </is>
       </c>
-      <c r="D466" s="36" t="n"/>
+      <c r="D466" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E466" s="19" t="n">
         <v>0</v>
       </c>
@@ -19603,7 +19647,11 @@
           <t>TOKS 不動前駅</t>
         </is>
       </c>
-      <c r="D471" s="36" t="n"/>
+      <c r="D471" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E471" s="19" t="n">
         <v>5</v>
       </c>
@@ -19722,7 +19770,11 @@
           <t>しぶそば大井町店</t>
         </is>
       </c>
-      <c r="D474" s="36" t="n"/>
+      <c r="D474" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E474" s="19" t="n">
         <v>10</v>
       </c>
@@ -19759,7 +19811,7 @@
           <t>大崎電気工業所</t>
         </is>
       </c>
-      <c r="D475" s="36" t="n"/>
+      <c r="D475" s="19" t="n"/>
       <c r="E475" s="19" t="n">
         <v>30</v>
       </c>
@@ -19796,11 +19848,7 @@
           <t>古賀電機株式会社</t>
         </is>
       </c>
-      <c r="D476" s="37" t="inlineStr">
-        <is>
-          <t>古賀電機（株）</t>
-        </is>
-      </c>
+      <c r="D476" s="19" t="n"/>
       <c r="E476" s="19" t="n">
         <v>85</v>
       </c>
@@ -19837,11 +19885,7 @@
           <t>古賀電機(株)新第二工場</t>
         </is>
       </c>
-      <c r="D477" s="37" t="inlineStr">
-        <is>
-          <t>古賀電機（株）</t>
-        </is>
-      </c>
+      <c r="D477" s="19" t="n"/>
       <c r="E477" s="19" t="n">
         <v>85</v>
       </c>
@@ -19878,11 +19922,7 @@
           <t>古賀電機第三工場</t>
         </is>
       </c>
-      <c r="D478" s="37" t="inlineStr">
-        <is>
-          <t>古賀電機（株）</t>
-        </is>
-      </c>
+      <c r="D478" s="19" t="n"/>
       <c r="E478" s="19" t="n">
         <v>30</v>
       </c>
@@ -19919,11 +19959,7 @@
           <t>堤工業</t>
         </is>
       </c>
-      <c r="D479" s="37" t="inlineStr">
-        <is>
-          <t>堤工業（株）</t>
-        </is>
-      </c>
+      <c r="D479" s="19" t="n"/>
       <c r="E479" s="19" t="n">
         <v>40</v>
       </c>
@@ -19960,11 +19996,7 @@
           <t>共立工芸</t>
         </is>
       </c>
-      <c r="D480" s="37" t="inlineStr">
-        <is>
-          <t>（株）共立工芸</t>
-        </is>
-      </c>
+      <c r="D480" s="19" t="n"/>
       <c r="E480" s="19" t="n">
         <v>35</v>
       </c>
@@ -20001,11 +20033,7 @@
           <t>山崎製作所</t>
         </is>
       </c>
-      <c r="D481" s="37" t="inlineStr">
-        <is>
-          <t>（株）山崎製作所</t>
-        </is>
-      </c>
+      <c r="D481" s="19" t="n"/>
       <c r="E481" s="19" t="n">
         <v>65</v>
       </c>
@@ -20083,7 +20111,7 @@
           <t>マツモトキヨシ　荏原町駅前店</t>
         </is>
       </c>
-      <c r="D483" s="36" t="n"/>
+      <c r="D483" s="19" t="n"/>
       <c r="E483" s="19" t="n">
         <v>30</v>
       </c>
@@ -20120,7 +20148,7 @@
           <t>カラダファクトリー　雪谷大塚店</t>
         </is>
       </c>
-      <c r="D484" s="36" t="n"/>
+      <c r="D484" s="19" t="n"/>
       <c r="E484" s="19" t="n">
         <v>10</v>
       </c>
@@ -20157,7 +20185,11 @@
           <t>中目黒高架下A</t>
         </is>
       </c>
-      <c r="D485" s="36" t="n"/>
+      <c r="D485" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E485" s="19" t="n">
         <v>15</v>
       </c>
@@ -20194,7 +20226,11 @@
           <t>中目黒高架下B</t>
         </is>
       </c>
-      <c r="D486" s="36" t="n"/>
+      <c r="D486" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E486" s="19" t="n">
         <v>50</v>
       </c>
@@ -20231,7 +20267,11 @@
           <t>中目黒高架下D</t>
         </is>
       </c>
-      <c r="D487" s="36" t="n"/>
+      <c r="D487" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E487" s="19" t="n">
         <v>20</v>
       </c>
@@ -20268,7 +20308,11 @@
           <t>中目黒高架下F</t>
         </is>
       </c>
-      <c r="D488" s="36" t="n"/>
+      <c r="D488" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E488" s="19" t="n">
         <v>20</v>
       </c>
@@ -20305,7 +20349,11 @@
           <t>中目黒高架下G</t>
         </is>
       </c>
-      <c r="D489" s="36" t="n"/>
+      <c r="D489" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E489" s="19" t="n">
         <v>20</v>
       </c>
@@ -20342,7 +20390,11 @@
           <t>中目黒高架下H</t>
         </is>
       </c>
-      <c r="D490" s="36" t="n"/>
+      <c r="D490" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E490" s="19" t="n">
         <v>5</v>
       </c>
@@ -20379,7 +20431,11 @@
           <t>中目黒高架下J</t>
         </is>
       </c>
-      <c r="D491" s="36" t="n"/>
+      <c r="D491" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E491" s="19" t="n">
         <v>0</v>
       </c>
@@ -20416,7 +20472,11 @@
           <t>学芸大学高架下（１０BL）</t>
         </is>
       </c>
-      <c r="D492" s="36" t="n"/>
+      <c r="D492" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E492" s="19" t="n">
         <v>10</v>
       </c>
@@ -20453,7 +20513,11 @@
           <t>学芸大学高架下（１３BL）</t>
         </is>
       </c>
-      <c r="D493" s="36" t="n"/>
+      <c r="D493" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E493" s="19" t="n">
         <v>140</v>
       </c>
@@ -20490,7 +20554,11 @@
           <t>学芸大学高架下（１４BL）</t>
         </is>
       </c>
-      <c r="D494" s="36" t="n"/>
+      <c r="D494" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E494" s="19" t="n">
         <v>60</v>
       </c>
@@ -20527,7 +20595,11 @@
           <t>グルメフロント（１５BL）</t>
         </is>
       </c>
-      <c r="D495" s="36" t="n"/>
+      <c r="D495" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E495" s="19" t="n">
         <v>10</v>
       </c>
@@ -20564,7 +20636,11 @@
           <t>学大コレクティブ（１６BL）</t>
         </is>
       </c>
-      <c r="D496" s="36" t="n"/>
+      <c r="D496" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E496" s="19" t="n">
         <v>10</v>
       </c>
@@ -20601,7 +20677,11 @@
           <t>自由が丘駅/北口</t>
         </is>
       </c>
-      <c r="D497" s="36" t="n"/>
+      <c r="D497" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E497" s="19" t="n">
         <v>100</v>
       </c>
@@ -20638,7 +20718,11 @@
           <t>自由が丘駅/南口</t>
         </is>
       </c>
-      <c r="D498" s="36" t="n"/>
+      <c r="D498" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E498" s="19" t="n">
         <v>30</v>
       </c>
@@ -20675,7 +20759,11 @@
           <t>エトモ　荏原町店</t>
         </is>
       </c>
-      <c r="D499" s="36" t="n"/>
+      <c r="D499" s="35" t="inlineStr">
+        <is>
+          <t>東急（株）</t>
+        </is>
+      </c>
       <c r="E499" s="19" t="n">
         <v>40</v>
       </c>
@@ -20712,7 +20800,7 @@
           <t>ケンタッキーフライドチキン　二子玉川店</t>
         </is>
       </c>
-      <c r="D500" s="36" t="n"/>
+      <c r="D500" s="19" t="n"/>
       <c r="E500" s="19" t="n">
         <v>90</v>
       </c>
@@ -20749,11 +20837,7 @@
           <t>MAISON KUROSU　学芸大学</t>
         </is>
       </c>
-      <c r="D501" s="37" t="inlineStr">
-        <is>
-          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
-        </is>
-      </c>
+      <c r="D501" s="19" t="n"/>
       <c r="E501" s="19" t="n">
         <v>0</v>
       </c>
@@ -61796,11 +61880,11 @@
       <c r="C11" s="7" t="n">
         <v>14800</v>
       </c>
-      <c r="D11" s="39" t="n">
+      <c r="D11" s="37" t="n">
         <v>0.02702702702702697</v>
       </c>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="39" t="n"/>
+      <c r="F11" s="37" t="n"/>
       <c r="G11" s="7" t="n">
         <v>0.0053504</v>
       </c>
@@ -61817,11 +61901,11 @@
       <c r="C12" s="7" t="n">
         <v>2300</v>
       </c>
-      <c r="D12" s="39" t="n">
+      <c r="D12" s="37" t="n">
         <v>-0.08695652173913049</v>
       </c>
       <c r="E12" s="7" t="n"/>
-      <c r="F12" s="39" t="n"/>
+      <c r="F12" s="37" t="n"/>
       <c r="G12" s="7" t="n">
         <v>4.851e-05</v>
       </c>
@@ -61838,11 +61922,11 @@
       <c r="C13" s="7" t="n">
         <v>3100</v>
       </c>
-      <c r="D13" s="39" t="n">
+      <c r="D13" s="37" t="n">
         <v>0.09677419354838701</v>
       </c>
       <c r="E13" s="7" t="n"/>
-      <c r="F13" s="39" t="n"/>
+      <c r="F13" s="37" t="n"/>
       <c r="G13" s="7" t="n">
         <v>0.00012546</v>
       </c>
@@ -61859,11 +61943,11 @@
       <c r="C14" s="7" t="n">
         <v>1900</v>
       </c>
-      <c r="D14" s="39" t="n">
+      <c r="D14" s="37" t="n">
         <v>-0.05263157894736847</v>
       </c>
       <c r="E14" s="7" t="n"/>
-      <c r="F14" s="39" t="n"/>
+      <c r="F14" s="37" t="n"/>
       <c r="G14" s="7" t="n">
         <v>4.158e-05</v>
       </c>
@@ -61880,11 +61964,11 @@
       <c r="C15" s="7" t="n">
         <v>750</v>
       </c>
-      <c r="D15" s="39" t="n">
+      <c r="D15" s="37" t="n">
         <v>0.06666666666666665</v>
       </c>
       <c r="E15" s="7" t="n"/>
-      <c r="F15" s="39" t="n"/>
+      <c r="F15" s="37" t="n"/>
       <c r="G15" s="7" t="n">
         <v>2.952e-05</v>
       </c>
@@ -61901,11 +61985,11 @@
       <c r="C16" s="11" t="n">
         <v>22850</v>
       </c>
-      <c r="D16" s="40" t="n">
+      <c r="D16" s="38" t="n">
         <v>0.01969365426695835</v>
       </c>
       <c r="E16" s="11" t="n"/>
-      <c r="F16" s="40" t="n"/>
+      <c r="F16" s="38" t="n"/>
       <c r="G16" s="11" t="n">
         <v>0</v>
       </c>
@@ -62336,7 +62420,7 @@
       <c r="D11" s="7" t="n">
         <v>0.06336</v>
       </c>
-      <c r="E11" s="39" t="n">
+      <c r="E11" s="37" t="n">
         <v>0.719585420672408</v>
       </c>
     </row>
@@ -62355,7 +62439,7 @@
       <c r="D12" s="7" t="n">
         <v>0.0005775</v>
       </c>
-      <c r="E12" s="39" t="n">
+      <c r="E12" s="37" t="n">
         <v>0.006558721282170386</v>
       </c>
     </row>
@@ -62374,7 +62458,7 @@
       <c r="D13" s="7" t="n">
         <v>0.001476</v>
       </c>
-      <c r="E13" s="39" t="n">
+      <c r="E13" s="37" t="n">
         <v>0.01676306945884587</v>
       </c>
     </row>
@@ -62393,7 +62477,7 @@
       <c r="D14" s="7" t="n">
         <v>0.0005082</v>
       </c>
-      <c r="E14" s="39" t="n">
+      <c r="E14" s="37" t="n">
         <v>0.00577167472830994</v>
       </c>
     </row>
@@ -62412,7 +62496,7 @@
       <c r="D15" s="7" t="n">
         <v>0.000369</v>
       </c>
-      <c r="E15" s="39" t="n">
+      <c r="E15" s="37" t="n">
         <v>0.004190767364711468</v>
       </c>
     </row>
@@ -62431,7 +62515,7 @@
       <c r="D16" s="7" t="n">
         <v>0.02176</v>
       </c>
-      <c r="E16" s="39" t="n">
+      <c r="E16" s="37" t="n">
         <v>0.2471303464935543</v>
       </c>
     </row>
@@ -62448,7 +62532,7 @@
       <c r="D17" s="11" t="n">
         <v>0.0880507</v>
       </c>
-      <c r="E17" s="40" t="inlineStr">
+      <c r="E17" s="38" t="inlineStr">
         <is>
           <t>100%</t>
         </is>

</xml_diff>

<commit_message>
Refine Tokyu D column entries using specific 板橋B names (45 rows)
Replaced generic 東急グループ with specific entities:
- 東急（株）: TOKS, 高架下, 乗務区, 駅施設 (33件)
- （株）東急コミュニティ: 駐輪場 (6件)
- （株）東急グルメフロント: グルメフロント, しぶそば (3件)
- （株）東急キッズボ－ルキャンプ大井町 (2件)
- （株）浅野屋: リトルマーメイド, ブランジェ浅野屋 (3件)
- （株）スープストックト－キョ－ (1件)

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -14133,7 +14133,7 @@
       </c>
       <c r="D331" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急グルメフロント</t>
         </is>
       </c>
       <c r="E331" s="19" t="n">
@@ -15640,7 +15640,7 @@
       </c>
       <c r="D370" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急コミュニティ</t>
         </is>
       </c>
       <c r="E370" s="19" t="n">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="D408" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急コミュニティ</t>
         </is>
       </c>
       <c r="E408" s="19" t="n">
@@ -18722,7 +18722,7 @@
       </c>
       <c r="D448" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急コミュニティ</t>
         </is>
       </c>
       <c r="E448" s="19" t="n">
@@ -18804,7 +18804,7 @@
       </c>
       <c r="D450" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急コミュニティ</t>
         </is>
       </c>
       <c r="E450" s="19" t="n">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="D458" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急コミュニティ</t>
         </is>
       </c>
       <c r="E458" s="19" t="n">
@@ -19444,7 +19444,7 @@
       </c>
       <c r="D466" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急コミュニティ</t>
         </is>
       </c>
       <c r="E466" s="19" t="n">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="D474" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急グルメフロント</t>
         </is>
       </c>
       <c r="E474" s="19" t="n">
@@ -20597,7 +20597,7 @@
       </c>
       <c r="D495" s="35" t="inlineStr">
         <is>
-          <t>東急（株）</t>
+          <t>（株）東急グルメフロント</t>
         </is>
       </c>
       <c r="E495" s="19" t="n">

</xml_diff>

<commit_message>
Rebuild v5 D column with all layers preserved (red 23 + blue 45)
Fixed issue where each script run was loading from original file,
overwriting previous step results. Now rebuilds all layers at once:
red font (fuzzy matches 23), blue font (Tokyu patterns 45),
yellow blank (72 remaining).

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -26,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
@@ -138,6 +138,9 @@
       <i val="1"/>
       <color rgb="FF595959"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <color rgb="000000FF"/>
@@ -281,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -331,10 +334,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -7986,7 +7996,11 @@
           <t>あらちゃん</t>
         </is>
       </c>
-      <c r="D178" s="25" t="n"/>
+      <c r="D178" s="35" t="inlineStr">
+        <is>
+          <t>モスアイズリ－（株）アイデイ－ あらちゃん</t>
+        </is>
+      </c>
       <c r="E178" s="19" t="n">
         <v>10</v>
       </c>
@@ -8269,7 +8283,7 @@
           <t>ASReal</t>
         </is>
       </c>
-      <c r="D185" s="19" t="n"/>
+      <c r="D185" s="36" t="n"/>
       <c r="E185" s="19" t="n">
         <v>0</v>
       </c>
@@ -8306,7 +8320,7 @@
           <t>ALWAYS OUT OF STOCK</t>
         </is>
       </c>
-      <c r="D186" s="19" t="n"/>
+      <c r="D186" s="36" t="n"/>
       <c r="E186" s="19" t="n">
         <v>0</v>
       </c>
@@ -8466,7 +8480,7 @@
           <t>GYM by LAVISUS</t>
         </is>
       </c>
-      <c r="D190" s="19" t="n"/>
+      <c r="D190" s="36" t="n"/>
       <c r="E190" s="19" t="n">
         <v>0</v>
       </c>
@@ -8544,7 +8558,7 @@
           <t>曼茶羅</t>
         </is>
       </c>
-      <c r="D192" s="19" t="n"/>
+      <c r="D192" s="36" t="n"/>
       <c r="E192" s="19" t="n">
         <v>0</v>
       </c>
@@ -8745,7 +8759,11 @@
           <t>CHANCEジム中目黒店</t>
         </is>
       </c>
-      <c r="D197" s="19" t="n"/>
+      <c r="D197" s="37" t="inlineStr">
+        <is>
+          <t>ＣＨＡＮＣＥ　ジム　中目黒</t>
+        </is>
+      </c>
       <c r="E197" s="19" t="n">
         <v>3</v>
       </c>
@@ -9110,7 +9128,7 @@
           <t>GOOD LUCK 中目黒店</t>
         </is>
       </c>
-      <c r="D206" s="19" t="n"/>
+      <c r="D206" s="36" t="n"/>
       <c r="E206" s="19" t="n">
         <v>5</v>
       </c>
@@ -9926,7 +9944,7 @@
           <t>Mix Bar Rose</t>
         </is>
       </c>
-      <c r="D226" s="19" t="n"/>
+      <c r="D226" s="36" t="n"/>
       <c r="E226" s="19" t="n">
         <v>0</v>
       </c>
@@ -9963,7 +9981,7 @@
           <t>sazan reef</t>
         </is>
       </c>
-      <c r="D227" s="19" t="n"/>
+      <c r="D227" s="36" t="n"/>
       <c r="E227" s="19" t="n">
         <v>1</v>
       </c>
@@ -10000,7 +10018,7 @@
           <t>CHI-FO</t>
         </is>
       </c>
-      <c r="D228" s="19" t="n"/>
+      <c r="D228" s="36" t="n"/>
       <c r="E228" s="19" t="n">
         <v>5</v>
       </c>
@@ -10160,7 +10178,7 @@
           <t>１０BL共用部分</t>
         </is>
       </c>
-      <c r="D232" s="35" t="inlineStr">
+      <c r="D232" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -10324,7 +10342,7 @@
           <t>鮮魚　北浜　学芸大学店</t>
         </is>
       </c>
-      <c r="D236" s="19" t="n"/>
+      <c r="D236" s="36" t="n"/>
       <c r="E236" s="19" t="n">
         <v>5</v>
       </c>
@@ -10484,7 +10502,7 @@
           <t>学大マーチ＆シーズンカフェ</t>
         </is>
       </c>
-      <c r="D240" s="19" t="n"/>
+      <c r="D240" s="36" t="n"/>
       <c r="E240" s="19" t="n">
         <v>0</v>
       </c>
@@ -10562,7 +10580,7 @@
           <t>そばもん　学大店</t>
         </is>
       </c>
-      <c r="D242" s="19" t="n"/>
+      <c r="D242" s="36" t="n"/>
       <c r="E242" s="19" t="n">
         <v>5</v>
       </c>
@@ -10804,7 +10822,11 @@
           <t>MAISON KUROSU学芸</t>
         </is>
       </c>
-      <c r="D248" s="19" t="n"/>
+      <c r="D248" s="37" t="inlineStr">
+        <is>
+          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
+        </is>
+      </c>
       <c r="E248" s="19" t="n">
         <v>30</v>
       </c>
@@ -11538,7 +11560,7 @@
           <t>DEAN&amp;DELUCA</t>
         </is>
       </c>
-      <c r="D266" s="19" t="n"/>
+      <c r="D266" s="36" t="n"/>
       <c r="E266" s="19" t="n">
         <v>80</v>
       </c>
@@ -11739,7 +11761,7 @@
           <t>あの小宮</t>
         </is>
       </c>
-      <c r="D271" s="19" t="n"/>
+      <c r="D271" s="36" t="n"/>
       <c r="E271" s="19" t="n">
         <v>100</v>
       </c>
@@ -11858,7 +11880,7 @@
           <t>あーる工房</t>
         </is>
       </c>
-      <c r="D274" s="19" t="n"/>
+      <c r="D274" s="36" t="n"/>
       <c r="E274" s="19" t="n">
         <v>1</v>
       </c>
@@ -11936,7 +11958,7 @@
           <t>NewWork　都立大</t>
         </is>
       </c>
-      <c r="D276" s="35" t="inlineStr">
+      <c r="D276" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -12141,7 +12163,7 @@
           <t>サーティーワンアイスクリーム</t>
         </is>
       </c>
-      <c r="D281" s="19" t="n"/>
+      <c r="D281" s="36" t="n"/>
       <c r="E281" s="19" t="n">
         <v>1</v>
       </c>
@@ -12178,7 +12200,7 @@
           <t>ルナアース</t>
         </is>
       </c>
-      <c r="D282" s="19" t="n"/>
+      <c r="D282" s="36" t="n"/>
       <c r="E282" s="19" t="n">
         <v>0</v>
       </c>
@@ -12256,7 +12278,7 @@
           <t>オープンマート駒澤大学駅中店</t>
         </is>
       </c>
-      <c r="D284" s="19" t="n"/>
+      <c r="D284" s="36" t="n"/>
       <c r="E284" s="19" t="n">
         <v>0</v>
       </c>
@@ -12293,7 +12315,7 @@
           <t>オハナ　明大前</t>
         </is>
       </c>
-      <c r="D285" s="19" t="n"/>
+      <c r="D285" s="36" t="n"/>
       <c r="E285" s="19" t="n">
         <v>40</v>
       </c>
@@ -12535,7 +12557,7 @@
           <t>roobby-fit 下高井戸店</t>
         </is>
       </c>
-      <c r="D291" s="19" t="n"/>
+      <c r="D291" s="36" t="n"/>
       <c r="E291" s="19" t="n">
         <v>0</v>
       </c>
@@ -12695,7 +12717,7 @@
           <t>MY SWEETS　渋谷店</t>
         </is>
       </c>
-      <c r="D295" s="19" t="n"/>
+      <c r="D295" s="36" t="n"/>
       <c r="E295" s="19" t="n">
         <v>0</v>
       </c>
@@ -12732,7 +12754,7 @@
           <t>ランキンランキン渋谷店</t>
         </is>
       </c>
-      <c r="D296" s="35" t="inlineStr">
+      <c r="D296" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -12773,7 +12795,7 @@
           <t>白洋舎　東京支店</t>
         </is>
       </c>
-      <c r="D297" s="19" t="n"/>
+      <c r="D297" s="36" t="n"/>
       <c r="E297" s="19" t="n">
         <v>150</v>
       </c>
@@ -12810,7 +12832,7 @@
           <t>河合塾　本郷校</t>
         </is>
       </c>
-      <c r="D298" s="19" t="n"/>
+      <c r="D298" s="36" t="n"/>
       <c r="E298" s="19" t="n">
         <v>100</v>
       </c>
@@ -12970,7 +12992,7 @@
           <t>南大塚エースビル</t>
         </is>
       </c>
-      <c r="D302" s="19" t="n"/>
+      <c r="D302" s="36" t="n"/>
       <c r="E302" s="19" t="n">
         <v>45</v>
       </c>
@@ -13007,7 +13029,7 @@
           <t>(株)ハピラル・テストソリューションズ</t>
         </is>
       </c>
-      <c r="D303" s="19" t="n"/>
+      <c r="D303" s="36" t="n"/>
       <c r="E303" s="19" t="n">
         <v>15</v>
       </c>
@@ -13208,7 +13230,7 @@
           <t>ミスターミニット　用賀店</t>
         </is>
       </c>
-      <c r="D308" s="19" t="n"/>
+      <c r="D308" s="36" t="n"/>
       <c r="E308" s="19" t="n">
         <v>5</v>
       </c>
@@ -13450,7 +13472,7 @@
           <t>スタジオマリオグラン　二子玉川店</t>
         </is>
       </c>
-      <c r="D314" s="19" t="n"/>
+      <c r="D314" s="36" t="n"/>
       <c r="E314" s="19" t="n">
         <v>5</v>
       </c>
@@ -13610,7 +13632,7 @@
           <t>こもれび保育園　上野毛園</t>
         </is>
       </c>
-      <c r="D318" s="19" t="n"/>
+      <c r="D318" s="36" t="n"/>
       <c r="E318" s="19" t="n">
         <v>20</v>
       </c>
@@ -13647,7 +13669,7 @@
           <t>あおい皮膚科　駅ナカ上野毛</t>
         </is>
       </c>
-      <c r="D319" s="19" t="n"/>
+      <c r="D319" s="36" t="n"/>
       <c r="E319" s="19" t="n">
         <v>0</v>
       </c>
@@ -13684,7 +13706,7 @@
           <t>大井町線上野毛駅構内店舗</t>
         </is>
       </c>
-      <c r="D320" s="35" t="inlineStr">
+      <c r="D320" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -13889,7 +13911,7 @@
           <t>フラマンドール　田園調布店</t>
         </is>
       </c>
-      <c r="D325" s="19" t="n"/>
+      <c r="D325" s="36" t="n"/>
       <c r="E325" s="19" t="n">
         <v>50</v>
       </c>
@@ -14049,7 +14071,7 @@
           <t>日吉エリア</t>
         </is>
       </c>
-      <c r="D329" s="35" t="inlineStr">
+      <c r="D329" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -14090,7 +14112,7 @@
           <t>リトルマーメイド　多摩川店</t>
         </is>
       </c>
-      <c r="D330" s="35" t="inlineStr">
+      <c r="D330" s="38" t="inlineStr">
         <is>
           <t>（株）浅野屋</t>
         </is>
@@ -14131,7 +14153,7 @@
           <t>しぶそば　多摩川店</t>
         </is>
       </c>
-      <c r="D331" s="35" t="inlineStr">
+      <c r="D331" s="38" t="inlineStr">
         <is>
           <t>（株）東急グルメフロント</t>
         </is>
@@ -14172,7 +14194,7 @@
           <t>銀座マギー　商品センター</t>
         </is>
       </c>
-      <c r="D332" s="19" t="n"/>
+      <c r="D332" s="36" t="n"/>
       <c r="E332" s="19" t="n">
         <v>70</v>
       </c>
@@ -14209,7 +14231,11 @@
           <t>学校法人　聖ドミニコ学園</t>
         </is>
       </c>
-      <c r="D333" s="19" t="n"/>
+      <c r="D333" s="37" t="inlineStr">
+        <is>
+          <t>聖ドミニコ学園</t>
+        </is>
+      </c>
       <c r="E333" s="19" t="n">
         <v>120</v>
       </c>
@@ -14246,7 +14272,11 @@
           <t>東京リーガルマインド　水道橋本校</t>
         </is>
       </c>
-      <c r="D334" s="19" t="n"/>
+      <c r="D334" s="37" t="inlineStr">
+        <is>
+          <t>（株）東京リーガルマインド</t>
+        </is>
+      </c>
       <c r="E334" s="19" t="n">
         <v>30</v>
       </c>
@@ -14406,7 +14436,7 @@
           <t>天才キッズクラブ楽学館仲池上園</t>
         </is>
       </c>
-      <c r="D338" s="19" t="n"/>
+      <c r="D338" s="36" t="n"/>
       <c r="E338" s="19" t="n">
         <v>0</v>
       </c>
@@ -14443,7 +14473,7 @@
           <t>Far Yeast Brewing</t>
         </is>
       </c>
-      <c r="D339" s="19" t="n"/>
+      <c r="D339" s="36" t="n"/>
       <c r="E339" s="19" t="n">
         <v>10</v>
       </c>
@@ -14480,7 +14510,7 @@
           <t>貝々　味海</t>
         </is>
       </c>
-      <c r="D340" s="19" t="n"/>
+      <c r="D340" s="36" t="n"/>
       <c r="E340" s="19" t="n">
         <v>3</v>
       </c>
@@ -14517,7 +14547,7 @@
           <t>東京食堂</t>
         </is>
       </c>
-      <c r="D341" s="19" t="n"/>
+      <c r="D341" s="36" t="n"/>
       <c r="E341" s="19" t="n">
         <v>0</v>
       </c>
@@ -14554,7 +14584,7 @@
           <t>ファットバー</t>
         </is>
       </c>
-      <c r="D342" s="19" t="n"/>
+      <c r="D342" s="36" t="n"/>
       <c r="E342" s="19" t="n">
         <v>0</v>
       </c>
@@ -14591,7 +14621,11 @@
           <t>さみしがりや酒房　ささ</t>
         </is>
       </c>
-      <c r="D343" s="19" t="n"/>
+      <c r="D343" s="37" t="inlineStr">
+        <is>
+          <t>さみしがりや酒房　ささ</t>
+        </is>
+      </c>
       <c r="E343" s="19" t="n">
         <v>0</v>
       </c>
@@ -14628,7 +14662,7 @@
           <t>居酒屋めぐろ川前</t>
         </is>
       </c>
-      <c r="D344" s="19" t="n"/>
+      <c r="D344" s="36" t="n"/>
       <c r="E344" s="19" t="n">
         <v>2</v>
       </c>
@@ -14665,7 +14699,7 @@
           <t>キッチン　クレセント</t>
         </is>
       </c>
-      <c r="D345" s="19" t="n"/>
+      <c r="D345" s="36" t="n"/>
       <c r="E345" s="19" t="n">
         <v>0</v>
       </c>
@@ -14702,7 +14736,11 @@
           <t>イケマル酒場</t>
         </is>
       </c>
-      <c r="D346" s="19" t="n"/>
+      <c r="D346" s="37" t="inlineStr">
+        <is>
+          <t>イケマル酒場（株）ロ－タスファイブ</t>
+        </is>
+      </c>
       <c r="E346" s="19" t="n">
         <v>0</v>
       </c>
@@ -14739,7 +14777,7 @@
           <t>桜小路　共用部</t>
         </is>
       </c>
-      <c r="D347" s="19" t="n"/>
+      <c r="D347" s="36" t="n"/>
       <c r="E347" s="19" t="n">
         <v>0</v>
       </c>
@@ -14858,7 +14896,7 @@
           <t>スターバックスコーヒー大井町駅</t>
         </is>
       </c>
-      <c r="D350" s="19" t="n"/>
+      <c r="D350" s="36" t="n"/>
       <c r="E350" s="19" t="n">
         <v>45</v>
       </c>
@@ -14895,7 +14933,7 @@
           <t>MY SWEETS　大井町店</t>
         </is>
       </c>
-      <c r="D351" s="19" t="n"/>
+      <c r="D351" s="36" t="n"/>
       <c r="E351" s="19" t="n">
         <v>0</v>
       </c>
@@ -14932,7 +14970,7 @@
           <t>えん　大井町店</t>
         </is>
       </c>
-      <c r="D352" s="19" t="n"/>
+      <c r="D352" s="36" t="n"/>
       <c r="E352" s="19" t="n">
         <v>35</v>
       </c>
@@ -14969,7 +15007,7 @@
           <t>E-style大井町校</t>
         </is>
       </c>
-      <c r="D353" s="19" t="n"/>
+      <c r="D353" s="36" t="n"/>
       <c r="E353" s="19" t="n">
         <v>0</v>
       </c>
@@ -15088,7 +15126,7 @@
           <t>都立大学高架下共用部</t>
         </is>
       </c>
-      <c r="D356" s="35" t="inlineStr">
+      <c r="D356" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -15211,7 +15249,7 @@
           <t>ロッジ</t>
         </is>
       </c>
-      <c r="D359" s="19" t="n"/>
+      <c r="D359" s="36" t="n"/>
       <c r="E359" s="19" t="n">
         <v>0</v>
       </c>
@@ -15248,7 +15286,7 @@
           <t>(株)銀座マギー　田園調布ビル</t>
         </is>
       </c>
-      <c r="D360" s="19" t="n"/>
+      <c r="D360" s="36" t="n"/>
       <c r="E360" s="19" t="n">
         <v>15</v>
       </c>
@@ -15326,7 +15364,7 @@
           <t>丸三ストアー</t>
         </is>
       </c>
-      <c r="D362" s="19" t="n"/>
+      <c r="D362" s="36" t="n"/>
       <c r="E362" s="19" t="n">
         <v>30</v>
       </c>
@@ -15404,7 +15442,7 @@
           <t>ローソン＋TOKS　石川台店</t>
         </is>
       </c>
-      <c r="D364" s="35" t="inlineStr">
+      <c r="D364" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -15486,7 +15524,7 @@
           <t>roobby　雪が谷大塚駅</t>
         </is>
       </c>
-      <c r="D366" s="19" t="n"/>
+      <c r="D366" s="36" t="n"/>
       <c r="E366" s="19" t="n">
         <v>3</v>
       </c>
@@ -15523,7 +15561,7 @@
           <t>ドトールコーヒー雪谷大塚店</t>
         </is>
       </c>
-      <c r="D367" s="19" t="n"/>
+      <c r="D367" s="36" t="n"/>
       <c r="E367" s="19" t="n">
         <v>5</v>
       </c>
@@ -15560,7 +15598,7 @@
           <t>カラダファクトリー雪谷大塚店</t>
         </is>
       </c>
-      <c r="D368" s="19" t="n"/>
+      <c r="D368" s="36" t="n"/>
       <c r="E368" s="19" t="n">
         <v>1</v>
       </c>
@@ -15638,7 +15676,7 @@
           <t>武蔵新田駐輪場</t>
         </is>
       </c>
-      <c r="D370" s="35" t="inlineStr">
+      <c r="D370" s="38" t="inlineStr">
         <is>
           <t>（株）東急コミュニティ</t>
         </is>
@@ -15802,7 +15840,7 @@
           <t>ドコモショップサテライト　エトモ鵜の木</t>
         </is>
       </c>
-      <c r="D374" s="35" t="inlineStr">
+      <c r="D374" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -16007,7 +16045,7 @@
           <t>ローソン＋多摩川駅店</t>
         </is>
       </c>
-      <c r="D379" s="35" t="inlineStr">
+      <c r="D379" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -16089,7 +16127,7 @@
           <t>リトルマーメイド多摩川店</t>
         </is>
       </c>
-      <c r="D381" s="35" t="inlineStr">
+      <c r="D381" s="38" t="inlineStr">
         <is>
           <t>（株）浅野屋</t>
         </is>
@@ -16212,7 +16250,7 @@
           <t>緑が丘エキナカ保育園</t>
         </is>
       </c>
-      <c r="D384" s="19" t="n"/>
+      <c r="D384" s="36" t="n"/>
       <c r="E384" s="19" t="n">
         <v>0</v>
       </c>
@@ -16290,7 +16328,7 @@
           <t>FRORIST KADAN</t>
         </is>
       </c>
-      <c r="D386" s="19" t="n"/>
+      <c r="D386" s="36" t="n"/>
       <c r="E386" s="19" t="n">
         <v>0</v>
       </c>
@@ -16368,7 +16406,7 @@
           <t>ゴントラン　シェリエmini自由が丘</t>
         </is>
       </c>
-      <c r="D388" s="19" t="n"/>
+      <c r="D388" s="36" t="n"/>
       <c r="E388" s="19" t="n">
         <v>0</v>
       </c>
@@ -16405,7 +16443,11 @@
           <t>丸山珈琲</t>
         </is>
       </c>
-      <c r="D389" s="19" t="n"/>
+      <c r="D389" s="37" t="inlineStr">
+        <is>
+          <t>（株）丸山珈琲</t>
+        </is>
+      </c>
       <c r="E389" s="19" t="n">
         <v>0</v>
       </c>
@@ -16442,7 +16484,7 @@
           <t>ローソン＋TOKS　自由が丘駅</t>
         </is>
       </c>
-      <c r="D390" s="35" t="inlineStr">
+      <c r="D390" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -16483,7 +16525,7 @@
           <t>スープストック　自由が丘店</t>
         </is>
       </c>
-      <c r="D391" s="35" t="inlineStr">
+      <c r="D391" s="38" t="inlineStr">
         <is>
           <t>（株）スープストックト－キョ－</t>
         </is>
@@ -16524,7 +16566,7 @@
           <t>TWG　Tea　自由が丘</t>
         </is>
       </c>
-      <c r="D392" s="19" t="n"/>
+      <c r="D392" s="36" t="n"/>
       <c r="E392" s="19" t="n">
         <v>5</v>
       </c>
@@ -16643,7 +16685,7 @@
           <t>Ben's Cookies 自由が丘店</t>
         </is>
       </c>
-      <c r="D395" s="19" t="n"/>
+      <c r="D395" s="36" t="n"/>
       <c r="E395" s="19" t="n">
         <v>0</v>
       </c>
@@ -16680,7 +16722,7 @@
           <t>リンツショコラ　ブティック</t>
         </is>
       </c>
-      <c r="D396" s="19" t="n"/>
+      <c r="D396" s="36" t="n"/>
       <c r="E396" s="19" t="n">
         <v>3</v>
       </c>
@@ -16758,7 +16800,7 @@
           <t>ブランジェ浅野屋　自由が丘店</t>
         </is>
       </c>
-      <c r="D398" s="35" t="inlineStr">
+      <c r="D398" s="38" t="inlineStr">
         <is>
           <t>（株）浅野屋</t>
         </is>
@@ -16840,7 +16882,7 @@
           <t>NATURAL KITCHEN　自由が丘</t>
         </is>
       </c>
-      <c r="D400" s="19" t="n"/>
+      <c r="D400" s="36" t="n"/>
       <c r="E400" s="19" t="n">
         <v>15</v>
       </c>
@@ -16877,7 +16919,7 @@
           <t>DUMBO Doughnuts</t>
         </is>
       </c>
-      <c r="D401" s="19" t="n"/>
+      <c r="D401" s="36" t="n"/>
       <c r="E401" s="19" t="n">
         <v>0</v>
       </c>
@@ -16996,7 +17038,7 @@
           <t>バガブー</t>
         </is>
       </c>
-      <c r="D404" s="19" t="n"/>
+      <c r="D404" s="36" t="n"/>
       <c r="E404" s="19" t="n">
         <v>0</v>
       </c>
@@ -17033,7 +17075,7 @@
           <t>ドリッピン　チュロス</t>
         </is>
       </c>
-      <c r="D405" s="19" t="n"/>
+      <c r="D405" s="36" t="n"/>
       <c r="E405" s="19" t="n">
         <v>1</v>
       </c>
@@ -17070,7 +17112,7 @@
           <t>トレインチ自由が丘　共有部</t>
         </is>
       </c>
-      <c r="D406" s="36" t="inlineStr">
+      <c r="D406" s="39" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -17111,7 +17153,7 @@
           <t>二子玉川乗務区</t>
         </is>
       </c>
-      <c r="D407" s="35" t="inlineStr">
+      <c r="D407" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -17152,7 +17194,7 @@
           <t>二子玉川駅駐輪場</t>
         </is>
       </c>
-      <c r="D408" s="35" t="inlineStr">
+      <c r="D408" s="38" t="inlineStr">
         <is>
           <t>（株）東急コミュニティ</t>
         </is>
@@ -17193,7 +17235,7 @@
           <t>コーモドドゥーエ</t>
         </is>
       </c>
-      <c r="D409" s="19" t="n"/>
+      <c r="D409" s="36" t="n"/>
       <c r="E409" s="19" t="n">
         <v>0</v>
       </c>
@@ -17230,7 +17272,11 @@
           <t>ファブリック</t>
         </is>
       </c>
-      <c r="D410" s="19" t="n"/>
+      <c r="D410" s="37" t="inlineStr">
+        <is>
+          <t>マレンロウ.グル－プ．ジャパン（株）ファブリック</t>
+        </is>
+      </c>
       <c r="E410" s="19" t="n">
         <v>3</v>
       </c>
@@ -17308,7 +17354,7 @@
           <t>サキュレ　本社営業所</t>
         </is>
       </c>
-      <c r="D412" s="19" t="n"/>
+      <c r="D412" s="36" t="n"/>
       <c r="E412" s="19" t="n">
         <v>15</v>
       </c>
@@ -17345,7 +17391,11 @@
           <t>東京ガスリビングラインライフバル西大田</t>
         </is>
       </c>
-      <c r="D413" s="19" t="n"/>
+      <c r="D413" s="37" t="inlineStr">
+        <is>
+          <t>東京ガスリビングライン（株）</t>
+        </is>
+      </c>
       <c r="E413" s="19" t="n">
         <v>40</v>
       </c>
@@ -17382,7 +17432,11 @@
           <t>白百合幼稚園</t>
         </is>
       </c>
-      <c r="D414" s="19" t="n"/>
+      <c r="D414" s="37" t="inlineStr">
+        <is>
+          <t>白百合幼稚園（つくしの学園</t>
+        </is>
+      </c>
       <c r="E414" s="19" t="n">
         <v>0</v>
       </c>
@@ -17419,7 +17473,11 @@
           <t>MAISON KUROSU</t>
         </is>
       </c>
-      <c r="D415" s="19" t="n"/>
+      <c r="D415" s="37" t="inlineStr">
+        <is>
+          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
+        </is>
+      </c>
       <c r="E415" s="19" t="n">
         <v>0</v>
       </c>
@@ -17456,7 +17514,7 @@
           <t>TOKS　目黒駅</t>
         </is>
       </c>
-      <c r="D416" s="35" t="inlineStr">
+      <c r="D416" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -17497,7 +17555,7 @@
           <t>マツモトキヨシ　目黒店</t>
         </is>
       </c>
-      <c r="D417" s="19" t="n"/>
+      <c r="D417" s="36" t="n"/>
       <c r="E417" s="19" t="n">
         <v>0</v>
       </c>
@@ -17534,7 +17592,7 @@
           <t>キッズスペースキャンプ　大井町</t>
         </is>
       </c>
-      <c r="D418" s="35" t="inlineStr">
+      <c r="D418" s="38" t="inlineStr">
         <is>
           <t>（株）東急キッズボ－ルキャンプ大井町</t>
         </is>
@@ -17575,7 +17633,7 @@
           <t>KBCほいくえん　大井町</t>
         </is>
       </c>
-      <c r="D419" s="35" t="inlineStr">
+      <c r="D419" s="38" t="inlineStr">
         <is>
           <t>（株）東急キッズボ－ルキャンプ大井町</t>
         </is>
@@ -17657,7 +17715,7 @@
           <t>第一商事</t>
         </is>
       </c>
-      <c r="D421" s="19" t="n"/>
+      <c r="D421" s="36" t="n"/>
       <c r="E421" s="19" t="n">
         <v>10</v>
       </c>
@@ -17735,7 +17793,7 @@
           <t>ミスターミニット　蒲田駅店</t>
         </is>
       </c>
-      <c r="D423" s="19" t="n"/>
+      <c r="D423" s="36" t="n"/>
       <c r="E423" s="19" t="n">
         <v>20</v>
       </c>
@@ -17772,7 +17830,7 @@
           <t>住まいと暮らしのコンシェルジュ</t>
         </is>
       </c>
-      <c r="D424" s="19" t="n"/>
+      <c r="D424" s="36" t="n"/>
       <c r="E424" s="19" t="n">
         <v>5</v>
       </c>
@@ -17809,7 +17867,7 @@
           <t>TOKS　蒲田改札口店</t>
         </is>
       </c>
-      <c r="D425" s="35" t="inlineStr">
+      <c r="D425" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -18055,7 +18113,7 @@
           <t>学校法人上野塾東京高等学校</t>
         </is>
       </c>
-      <c r="D431" s="19" t="n"/>
+      <c r="D431" s="36" t="n"/>
       <c r="E431" s="19" t="n">
         <v>40</v>
       </c>
@@ -18092,7 +18150,11 @@
           <t>日本ロジテム三幸営業所</t>
         </is>
       </c>
-      <c r="D432" s="19" t="n"/>
+      <c r="D432" s="37" t="inlineStr">
+        <is>
+          <t>日本ロジテム（株）</t>
+        </is>
+      </c>
       <c r="E432" s="19" t="n">
         <v>80</v>
       </c>
@@ -18293,7 +18355,11 @@
           <t>キャンバン</t>
         </is>
       </c>
-      <c r="D437" s="19" t="n"/>
+      <c r="D437" s="37" t="inlineStr">
+        <is>
+          <t>（株）キャンバン</t>
+        </is>
+      </c>
       <c r="E437" s="19" t="n">
         <v>3</v>
       </c>
@@ -18330,7 +18396,11 @@
           <t>デルフォニックス</t>
         </is>
       </c>
-      <c r="D438" s="19" t="n"/>
+      <c r="D438" s="37" t="inlineStr">
+        <is>
+          <t>（株）デルフォニックス</t>
+        </is>
+      </c>
       <c r="E438" s="19" t="n">
         <v>5</v>
       </c>
@@ -18404,7 +18474,7 @@
           <t>ローソン＋TOKS　三軒茶屋店</t>
         </is>
       </c>
-      <c r="D440" s="35" t="inlineStr">
+      <c r="D440" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -18720,7 +18790,7 @@
           <t>西小山（南）駐輪場</t>
         </is>
       </c>
-      <c r="D448" s="35" t="inlineStr">
+      <c r="D448" s="38" t="inlineStr">
         <is>
           <t>（株）東急コミュニティ</t>
         </is>
@@ -18802,7 +18872,7 @@
           <t>武蔵小山西口駐輪場</t>
         </is>
       </c>
-      <c r="D450" s="35" t="inlineStr">
+      <c r="D450" s="38" t="inlineStr">
         <is>
           <t>（株）東急コミュニティ</t>
         </is>
@@ -19007,7 +19077,11 @@
           <t>メガネスーパーコンタクト五反田エキナカ店</t>
         </is>
       </c>
-      <c r="D455" s="19" t="n"/>
+      <c r="D455" s="37" t="inlineStr">
+        <is>
+          <t>（株）メガネスーパー</t>
+        </is>
+      </c>
       <c r="E455" s="19" t="n">
         <v>0</v>
       </c>
@@ -19126,7 +19200,7 @@
           <t>荏原中延駐輪場</t>
         </is>
       </c>
-      <c r="D458" s="35" t="inlineStr">
+      <c r="D458" s="38" t="inlineStr">
         <is>
           <t>（株）東急コミュニティ</t>
         </is>
@@ -19208,7 +19282,7 @@
           <t>サキュレ本社営業所</t>
         </is>
       </c>
-      <c r="D460" s="19" t="n"/>
+      <c r="D460" s="36" t="n"/>
       <c r="E460" s="19" t="n">
         <v>5</v>
       </c>
@@ -19286,7 +19360,7 @@
           <t>ミスターワッフル　旗の台エキナカ店</t>
         </is>
       </c>
-      <c r="D462" s="19" t="n"/>
+      <c r="D462" s="36" t="n"/>
       <c r="E462" s="19" t="n">
         <v>5</v>
       </c>
@@ -19323,7 +19397,7 @@
           <t>グローバルキッズ　荏原町保育園</t>
         </is>
       </c>
-      <c r="D463" s="19" t="n"/>
+      <c r="D463" s="36" t="n"/>
       <c r="E463" s="19" t="n">
         <v>20</v>
       </c>
@@ -19442,7 +19516,7 @@
           <t>中延駐輪場</t>
         </is>
       </c>
-      <c r="D466" s="35" t="inlineStr">
+      <c r="D466" s="38" t="inlineStr">
         <is>
           <t>（株）東急コミュニティ</t>
         </is>
@@ -19647,7 +19721,7 @@
           <t>TOKS 不動前駅</t>
         </is>
       </c>
-      <c r="D471" s="35" t="inlineStr">
+      <c r="D471" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -19770,7 +19844,7 @@
           <t>しぶそば大井町店</t>
         </is>
       </c>
-      <c r="D474" s="35" t="inlineStr">
+      <c r="D474" s="38" t="inlineStr">
         <is>
           <t>（株）東急グルメフロント</t>
         </is>
@@ -19811,7 +19885,7 @@
           <t>大崎電気工業所</t>
         </is>
       </c>
-      <c r="D475" s="19" t="n"/>
+      <c r="D475" s="36" t="n"/>
       <c r="E475" s="19" t="n">
         <v>30</v>
       </c>
@@ -19848,7 +19922,11 @@
           <t>古賀電機株式会社</t>
         </is>
       </c>
-      <c r="D476" s="19" t="n"/>
+      <c r="D476" s="37" t="inlineStr">
+        <is>
+          <t>古賀電機（株）</t>
+        </is>
+      </c>
       <c r="E476" s="19" t="n">
         <v>85</v>
       </c>
@@ -19885,7 +19963,11 @@
           <t>古賀電機(株)新第二工場</t>
         </is>
       </c>
-      <c r="D477" s="19" t="n"/>
+      <c r="D477" s="37" t="inlineStr">
+        <is>
+          <t>古賀電機（株）</t>
+        </is>
+      </c>
       <c r="E477" s="19" t="n">
         <v>85</v>
       </c>
@@ -19922,7 +20004,11 @@
           <t>古賀電機第三工場</t>
         </is>
       </c>
-      <c r="D478" s="19" t="n"/>
+      <c r="D478" s="37" t="inlineStr">
+        <is>
+          <t>古賀電機（株）</t>
+        </is>
+      </c>
       <c r="E478" s="19" t="n">
         <v>30</v>
       </c>
@@ -19959,7 +20045,11 @@
           <t>堤工業</t>
         </is>
       </c>
-      <c r="D479" s="19" t="n"/>
+      <c r="D479" s="37" t="inlineStr">
+        <is>
+          <t>堤工業（株）</t>
+        </is>
+      </c>
       <c r="E479" s="19" t="n">
         <v>40</v>
       </c>
@@ -19996,7 +20086,11 @@
           <t>共立工芸</t>
         </is>
       </c>
-      <c r="D480" s="19" t="n"/>
+      <c r="D480" s="37" t="inlineStr">
+        <is>
+          <t>（株）共立工芸</t>
+        </is>
+      </c>
       <c r="E480" s="19" t="n">
         <v>35</v>
       </c>
@@ -20033,7 +20127,11 @@
           <t>山崎製作所</t>
         </is>
       </c>
-      <c r="D481" s="19" t="n"/>
+      <c r="D481" s="37" t="inlineStr">
+        <is>
+          <t>（株）山崎製作所</t>
+        </is>
+      </c>
       <c r="E481" s="19" t="n">
         <v>65</v>
       </c>
@@ -20111,7 +20209,7 @@
           <t>マツモトキヨシ　荏原町駅前店</t>
         </is>
       </c>
-      <c r="D483" s="19" t="n"/>
+      <c r="D483" s="36" t="n"/>
       <c r="E483" s="19" t="n">
         <v>30</v>
       </c>
@@ -20148,7 +20246,7 @@
           <t>カラダファクトリー　雪谷大塚店</t>
         </is>
       </c>
-      <c r="D484" s="19" t="n"/>
+      <c r="D484" s="36" t="n"/>
       <c r="E484" s="19" t="n">
         <v>10</v>
       </c>
@@ -20185,7 +20283,7 @@
           <t>中目黒高架下A</t>
         </is>
       </c>
-      <c r="D485" s="35" t="inlineStr">
+      <c r="D485" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20226,7 +20324,7 @@
           <t>中目黒高架下B</t>
         </is>
       </c>
-      <c r="D486" s="35" t="inlineStr">
+      <c r="D486" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20267,7 +20365,7 @@
           <t>中目黒高架下D</t>
         </is>
       </c>
-      <c r="D487" s="35" t="inlineStr">
+      <c r="D487" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20308,7 +20406,7 @@
           <t>中目黒高架下F</t>
         </is>
       </c>
-      <c r="D488" s="35" t="inlineStr">
+      <c r="D488" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20349,7 +20447,7 @@
           <t>中目黒高架下G</t>
         </is>
       </c>
-      <c r="D489" s="35" t="inlineStr">
+      <c r="D489" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20390,7 +20488,7 @@
           <t>中目黒高架下H</t>
         </is>
       </c>
-      <c r="D490" s="35" t="inlineStr">
+      <c r="D490" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20431,7 +20529,7 @@
           <t>中目黒高架下J</t>
         </is>
       </c>
-      <c r="D491" s="35" t="inlineStr">
+      <c r="D491" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20472,7 +20570,7 @@
           <t>学芸大学高架下（１０BL）</t>
         </is>
       </c>
-      <c r="D492" s="35" t="inlineStr">
+      <c r="D492" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20513,7 +20611,7 @@
           <t>学芸大学高架下（１３BL）</t>
         </is>
       </c>
-      <c r="D493" s="35" t="inlineStr">
+      <c r="D493" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20554,7 +20652,7 @@
           <t>学芸大学高架下（１４BL）</t>
         </is>
       </c>
-      <c r="D494" s="35" t="inlineStr">
+      <c r="D494" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20595,7 +20693,7 @@
           <t>グルメフロント（１５BL）</t>
         </is>
       </c>
-      <c r="D495" s="35" t="inlineStr">
+      <c r="D495" s="38" t="inlineStr">
         <is>
           <t>（株）東急グルメフロント</t>
         </is>
@@ -20636,7 +20734,7 @@
           <t>学大コレクティブ（１６BL）</t>
         </is>
       </c>
-      <c r="D496" s="35" t="inlineStr">
+      <c r="D496" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20677,7 +20775,7 @@
           <t>自由が丘駅/北口</t>
         </is>
       </c>
-      <c r="D497" s="35" t="inlineStr">
+      <c r="D497" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20718,7 +20816,7 @@
           <t>自由が丘駅/南口</t>
         </is>
       </c>
-      <c r="D498" s="35" t="inlineStr">
+      <c r="D498" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20759,7 +20857,7 @@
           <t>エトモ　荏原町店</t>
         </is>
       </c>
-      <c r="D499" s="35" t="inlineStr">
+      <c r="D499" s="38" t="inlineStr">
         <is>
           <t>東急（株）</t>
         </is>
@@ -20800,7 +20898,7 @@
           <t>ケンタッキーフライドチキン　二子玉川店</t>
         </is>
       </c>
-      <c r="D500" s="19" t="n"/>
+      <c r="D500" s="36" t="n"/>
       <c r="E500" s="19" t="n">
         <v>90</v>
       </c>
@@ -20837,7 +20935,11 @@
           <t>MAISON KUROSU　学芸大学</t>
         </is>
       </c>
-      <c r="D501" s="19" t="n"/>
+      <c r="D501" s="37" t="inlineStr">
+        <is>
+          <t>ＭＡＩＳＯＮ　ＫＵＲＯＳＵ</t>
+        </is>
+      </c>
       <c r="E501" s="19" t="n">
         <v>0</v>
       </c>
@@ -61880,11 +61982,11 @@
       <c r="C11" s="7" t="n">
         <v>14800</v>
       </c>
-      <c r="D11" s="37" t="n">
+      <c r="D11" s="40" t="n">
         <v>0.02702702702702697</v>
       </c>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="37" t="n"/>
+      <c r="F11" s="40" t="n"/>
       <c r="G11" s="7" t="n">
         <v>0.0053504</v>
       </c>
@@ -61901,11 +62003,11 @@
       <c r="C12" s="7" t="n">
         <v>2300</v>
       </c>
-      <c r="D12" s="37" t="n">
+      <c r="D12" s="40" t="n">
         <v>-0.08695652173913049</v>
       </c>
       <c r="E12" s="7" t="n"/>
-      <c r="F12" s="37" t="n"/>
+      <c r="F12" s="40" t="n"/>
       <c r="G12" s="7" t="n">
         <v>4.851e-05</v>
       </c>
@@ -61922,11 +62024,11 @@
       <c r="C13" s="7" t="n">
         <v>3100</v>
       </c>
-      <c r="D13" s="37" t="n">
+      <c r="D13" s="40" t="n">
         <v>0.09677419354838701</v>
       </c>
       <c r="E13" s="7" t="n"/>
-      <c r="F13" s="37" t="n"/>
+      <c r="F13" s="40" t="n"/>
       <c r="G13" s="7" t="n">
         <v>0.00012546</v>
       </c>
@@ -61943,11 +62045,11 @@
       <c r="C14" s="7" t="n">
         <v>1900</v>
       </c>
-      <c r="D14" s="37" t="n">
+      <c r="D14" s="40" t="n">
         <v>-0.05263157894736847</v>
       </c>
       <c r="E14" s="7" t="n"/>
-      <c r="F14" s="37" t="n"/>
+      <c r="F14" s="40" t="n"/>
       <c r="G14" s="7" t="n">
         <v>4.158e-05</v>
       </c>
@@ -61964,11 +62066,11 @@
       <c r="C15" s="7" t="n">
         <v>750</v>
       </c>
-      <c r="D15" s="37" t="n">
+      <c r="D15" s="40" t="n">
         <v>0.06666666666666665</v>
       </c>
       <c r="E15" s="7" t="n"/>
-      <c r="F15" s="37" t="n"/>
+      <c r="F15" s="40" t="n"/>
       <c r="G15" s="7" t="n">
         <v>2.952e-05</v>
       </c>
@@ -61985,11 +62087,11 @@
       <c r="C16" s="11" t="n">
         <v>22850</v>
       </c>
-      <c r="D16" s="38" t="n">
+      <c r="D16" s="41" t="n">
         <v>0.01969365426695835</v>
       </c>
       <c r="E16" s="11" t="n"/>
-      <c r="F16" s="38" t="n"/>
+      <c r="F16" s="41" t="n"/>
       <c r="G16" s="11" t="n">
         <v>0</v>
       </c>
@@ -62420,7 +62522,7 @@
       <c r="D11" s="7" t="n">
         <v>0.06336</v>
       </c>
-      <c r="E11" s="37" t="n">
+      <c r="E11" s="40" t="n">
         <v>0.719585420672408</v>
       </c>
     </row>
@@ -62439,7 +62541,7 @@
       <c r="D12" s="7" t="n">
         <v>0.0005775</v>
       </c>
-      <c r="E12" s="37" t="n">
+      <c r="E12" s="40" t="n">
         <v>0.006558721282170386</v>
       </c>
     </row>
@@ -62458,7 +62560,7 @@
       <c r="D13" s="7" t="n">
         <v>0.001476</v>
       </c>
-      <c r="E13" s="37" t="n">
+      <c r="E13" s="40" t="n">
         <v>0.01676306945884587</v>
       </c>
     </row>
@@ -62477,7 +62579,7 @@
       <c r="D14" s="7" t="n">
         <v>0.0005082</v>
       </c>
-      <c r="E14" s="37" t="n">
+      <c r="E14" s="40" t="n">
         <v>0.00577167472830994</v>
       </c>
     </row>
@@ -62496,7 +62598,7 @@
       <c r="D15" s="7" t="n">
         <v>0.000369</v>
       </c>
-      <c r="E15" s="37" t="n">
+      <c r="E15" s="40" t="n">
         <v>0.004190767364711468</v>
       </c>
     </row>
@@ -62515,7 +62617,7 @@
       <c r="D16" s="7" t="n">
         <v>0.02176</v>
       </c>
-      <c r="E16" s="37" t="n">
+      <c r="E16" s="40" t="n">
         <v>0.2471303464935543</v>
       </c>
     </row>
@@ -62532,7 +62634,7 @@
       <c r="D17" s="11" t="n">
         <v>0.0880507</v>
       </c>
-      <c r="E17" s="38" t="inlineStr">
+      <c r="E17" s="41" t="inlineStr">
         <is>
           <t>100%</t>
         </is>

</xml_diff>

<commit_message>
Add 18 more red font entries matched from 板橋B column
Direct keyword matches: 白洋舎, 河合塾, 銀座マギー, ハピラル,
丸三ストアー, 天才キッズクラブ, 上野塾, リンツ, オープンマート,
サキュレ本社, ミスターミニット(x2), Far Yeast, グローバルキッズ,
ドリッピン, バガブー, (x18 total). 54 cells remain blank yellow.

https://claude.ai/code/session_01BgHAFjDQSmbvXBnKUF79fq
</commit_message>
<xml_diff>
--- a/サキュレ_拠点マスターv5_D列更新.xlsx
+++ b/サキュレ_拠点マスターv5_D列更新.xlsx
@@ -12278,7 +12278,11 @@
           <t>オープンマート駒澤大学駅中店</t>
         </is>
       </c>
-      <c r="D284" s="36" t="n"/>
+      <c r="D284" s="37" t="inlineStr">
+        <is>
+          <t>オ－プンマ－ト駒澤大学駅中店　空き地企画</t>
+        </is>
+      </c>
       <c r="E284" s="19" t="n">
         <v>0</v>
       </c>
@@ -12795,7 +12799,11 @@
           <t>白洋舎　東京支店</t>
         </is>
       </c>
-      <c r="D297" s="36" t="n"/>
+      <c r="D297" s="37" t="inlineStr">
+        <is>
+          <t>（株）白洋舎</t>
+        </is>
+      </c>
       <c r="E297" s="19" t="n">
         <v>150</v>
       </c>
@@ -12832,7 +12840,11 @@
           <t>河合塾　本郷校</t>
         </is>
       </c>
-      <c r="D298" s="36" t="n"/>
+      <c r="D298" s="37" t="inlineStr">
+        <is>
+          <t>河合塾</t>
+        </is>
+      </c>
       <c r="E298" s="19" t="n">
         <v>100</v>
       </c>
@@ -13029,7 +13041,11 @@
           <t>(株)ハピラル・テストソリューションズ</t>
         </is>
       </c>
-      <c r="D303" s="36" t="n"/>
+      <c r="D303" s="37" t="inlineStr">
+        <is>
+          <t>（株）ハピラルテストソリュ－ションズ</t>
+        </is>
+      </c>
       <c r="E303" s="19" t="n">
         <v>15</v>
       </c>
@@ -13230,7 +13246,11 @@
           <t>ミスターミニット　用賀店</t>
         </is>
       </c>
-      <c r="D308" s="36" t="n"/>
+      <c r="D308" s="37" t="inlineStr">
+        <is>
+          <t>ミニットアジアパシフィック（株）</t>
+        </is>
+      </c>
       <c r="E308" s="19" t="n">
         <v>5</v>
       </c>
@@ -14194,7 +14214,11 @@
           <t>銀座マギー　商品センター</t>
         </is>
       </c>
-      <c r="D332" s="36" t="n"/>
+      <c r="D332" s="37" t="inlineStr">
+        <is>
+          <t>（株）銀座マギ－</t>
+        </is>
+      </c>
       <c r="E332" s="19" t="n">
         <v>70</v>
       </c>
@@ -14436,7 +14460,11 @@
           <t>天才キッズクラブ楽学館仲池上園</t>
         </is>
       </c>
-      <c r="D338" s="36" t="n"/>
+      <c r="D338" s="37" t="inlineStr">
+        <is>
+          <t>天才キッズクラブ楽学館（株）ＴＫＣ</t>
+        </is>
+      </c>
       <c r="E338" s="19" t="n">
         <v>0</v>
       </c>
@@ -14473,7 +14501,11 @@
           <t>Far Yeast Brewing</t>
         </is>
       </c>
-      <c r="D339" s="36" t="n"/>
+      <c r="D339" s="37" t="inlineStr">
+        <is>
+          <t>Ｆａｒ　Ｅｅａｓｔ　Ｂｒｅｗｉｎｇ（株）</t>
+        </is>
+      </c>
       <c r="E339" s="19" t="n">
         <v>10</v>
       </c>
@@ -15286,7 +15318,11 @@
           <t>(株)銀座マギー　田園調布ビル</t>
         </is>
       </c>
-      <c r="D360" s="36" t="n"/>
+      <c r="D360" s="37" t="inlineStr">
+        <is>
+          <t>（株）銀座マギ－</t>
+        </is>
+      </c>
       <c r="E360" s="19" t="n">
         <v>15</v>
       </c>
@@ -15364,7 +15400,11 @@
           <t>丸三ストアー</t>
         </is>
       </c>
-      <c r="D362" s="36" t="n"/>
+      <c r="D362" s="37" t="inlineStr">
+        <is>
+          <t>（株）丸三ストア－</t>
+        </is>
+      </c>
       <c r="E362" s="19" t="n">
         <v>30</v>
       </c>
@@ -16722,7 +16762,11 @@
           <t>リンツショコラ　ブティック</t>
         </is>
       </c>
-      <c r="D396" s="36" t="n"/>
+      <c r="D396" s="37" t="inlineStr">
+        <is>
+          <t>リンツ＆シュプルングリ－ジャパン（株）</t>
+        </is>
+      </c>
       <c r="E396" s="19" t="n">
         <v>3</v>
       </c>
@@ -17038,7 +17082,11 @@
           <t>バガブー</t>
         </is>
       </c>
-      <c r="D404" s="36" t="n"/>
+      <c r="D404" s="37" t="inlineStr">
+        <is>
+          <t>バガブ－ジャパン（株）</t>
+        </is>
+      </c>
       <c r="E404" s="19" t="n">
         <v>0</v>
       </c>
@@ -17075,7 +17123,11 @@
           <t>ドリッピン　チュロス</t>
         </is>
       </c>
-      <c r="D405" s="36" t="n"/>
+      <c r="D405" s="37" t="inlineStr">
+        <is>
+          <t>ｄｒｉｐｐｉｎ’ｃｈｕｒｒｏｓ</t>
+        </is>
+      </c>
       <c r="E405" s="19" t="n">
         <v>1</v>
       </c>
@@ -17354,7 +17406,11 @@
           <t>サキュレ　本社営業所</t>
         </is>
       </c>
-      <c r="D412" s="36" t="n"/>
+      <c r="D412" s="37" t="inlineStr">
+        <is>
+          <t>ＫＣサキュレ（株）</t>
+        </is>
+      </c>
       <c r="E412" s="19" t="n">
         <v>15</v>
       </c>
@@ -17793,7 +17849,11 @@
           <t>ミスターミニット　蒲田駅店</t>
         </is>
       </c>
-      <c r="D423" s="36" t="n"/>
+      <c r="D423" s="37" t="inlineStr">
+        <is>
+          <t>ミニットアジアパシフィック（株）</t>
+        </is>
+      </c>
       <c r="E423" s="19" t="n">
         <v>20</v>
       </c>
@@ -18113,7 +18173,11 @@
           <t>学校法人上野塾東京高等学校</t>
         </is>
       </c>
-      <c r="D431" s="36" t="n"/>
+      <c r="D431" s="37" t="inlineStr">
+        <is>
+          <t>東京高等学校　上野塾</t>
+        </is>
+      </c>
       <c r="E431" s="19" t="n">
         <v>40</v>
       </c>
@@ -19282,7 +19346,11 @@
           <t>サキュレ本社営業所</t>
         </is>
       </c>
-      <c r="D460" s="36" t="n"/>
+      <c r="D460" s="37" t="inlineStr">
+        <is>
+          <t>ＫＣサキュレ（株）</t>
+        </is>
+      </c>
       <c r="E460" s="19" t="n">
         <v>5</v>
       </c>
@@ -19397,7 +19465,11 @@
           <t>グローバルキッズ　荏原町保育園</t>
         </is>
       </c>
-      <c r="D463" s="36" t="n"/>
+      <c r="D463" s="37" t="inlineStr">
+        <is>
+          <t>（株）グロ－バルキッズ</t>
+        </is>
+      </c>
       <c r="E463" s="19" t="n">
         <v>20</v>
       </c>

</xml_diff>